<commit_message>
docs: update test cases, with type and tools cols
</commit_message>
<xml_diff>
--- a/docs/tests/breco - cas de test.xlsx
+++ b/docs/tests/breco - cas de test.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\4-SYNC\PRO\ICADEMIE\DOSSIER-TECH\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5526A3A0-9F30-4110-99DC-90834D2E7E08}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{069336C2-1BA8-4D5C-8CDB-F3D05E9C9DCD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Story1 - Auth" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="594" uniqueCount="276">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="840" uniqueCount="287">
   <si>
     <t>Plan de test Breco, cas de test</t>
   </si>
@@ -1402,9 +1402,6 @@
   </si>
   <si>
     <t>Story 5 : Proposer des covoiturages</t>
-  </si>
-  <si>
-    <t>Story 2 : Pré-remplir les champs</t>
   </si>
   <si>
     <t>TC-66</t>
@@ -1521,6 +1518,42 @@
   </si>
   <si>
     <t>Erreur : "La recherche doit contenir au moins 2 caractères". En frontend, liste vide retournée, sans erreur</t>
+  </si>
+  <si>
+    <t>Type</t>
+  </si>
+  <si>
+    <t>Unitaire</t>
+  </si>
+  <si>
+    <t>Intégration</t>
+  </si>
+  <si>
+    <t>Outil</t>
+  </si>
+  <si>
+    <t>Couche</t>
+  </si>
+  <si>
+    <t>Vitest</t>
+  </si>
+  <si>
+    <t>Frontend</t>
+  </si>
+  <si>
+    <t>Vitest + PHPUnit</t>
+  </si>
+  <si>
+    <t>Frontend + Backend</t>
+  </si>
+  <si>
+    <t>Story 4 : Pré-remplir les champs</t>
+  </si>
+  <si>
+    <t>PHPUnit</t>
+  </si>
+  <si>
+    <t>Backend</t>
   </si>
 </sst>
 </file>
@@ -1856,19 +1889,19 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:Q79"/>
+  <dimension ref="A1:T79"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.5703125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="11.5703125" style="1"/>
-    <col min="2" max="2" width="15" style="1" customWidth="1"/>
-    <col min="3" max="3" width="38.5703125" style="2" customWidth="1"/>
-    <col min="4" max="4" width="26.85546875" style="3" customWidth="1"/>
-    <col min="5" max="5" width="40.28515625" style="2" customWidth="1"/>
-    <col min="6" max="6" width="28.140625" style="1" customWidth="1"/>
-    <col min="7" max="16384" width="11.5703125" style="1"/>
+    <col min="1" max="4" width="11.5703125" style="1"/>
+    <col min="5" max="5" width="15" style="1" customWidth="1"/>
+    <col min="6" max="6" width="38.5703125" style="2" customWidth="1"/>
+    <col min="7" max="7" width="26.85546875" style="3" customWidth="1"/>
+    <col min="8" max="8" width="40.28515625" style="2" customWidth="1"/>
+    <col min="9" max="9" width="28.140625" style="1" customWidth="1"/>
+    <col min="10" max="16384" width="11.5703125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="19.350000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:11" ht="19.350000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="21" t="s">
         <v>0</v>
       </c>
@@ -1878,9 +1911,12 @@
       <c r="E1" s="21"/>
       <c r="F1" s="21"/>
       <c r="G1" s="21"/>
-      <c r="H1" s="4"/>
-    </row>
-    <row r="2" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="H1" s="21"/>
+      <c r="I1" s="21"/>
+      <c r="J1" s="21"/>
+      <c r="K1" s="4"/>
+    </row>
+    <row r="2" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="22" t="s">
         <v>1</v>
       </c>
@@ -1890,1317 +1926,1812 @@
       <c r="E2" s="22"/>
       <c r="F2" s="22"/>
       <c r="G2" s="22"/>
-      <c r="H2" s="4"/>
-    </row>
-    <row r="3" spans="1:8" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="H2" s="22"/>
+      <c r="I2" s="22"/>
+      <c r="J2" s="22"/>
+      <c r="K2" s="4"/>
+    </row>
+    <row r="3" spans="1:11" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A3" s="5" t="s">
         <v>2</v>
       </c>
       <c r="B3" s="5" t="s">
+        <v>275</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>278</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>279</v>
+      </c>
+      <c r="E3" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="C3" s="5" t="s">
+      <c r="F3" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="D3" s="6" t="s">
+      <c r="G3" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="E3" s="5" t="s">
+      <c r="H3" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="F3" s="5" t="s">
+      <c r="I3" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="G3" s="5" t="s">
+      <c r="J3" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="H3" s="4"/>
-    </row>
-    <row r="4" spans="1:8" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="K3" s="4"/>
+    </row>
+    <row r="4" spans="1:11" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A4" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="B4" s="8" t="s">
+      <c r="B4" s="7" t="s">
+        <v>276</v>
+      </c>
+      <c r="C4" s="7" t="s">
+        <v>280</v>
+      </c>
+      <c r="D4" s="7" t="s">
+        <v>281</v>
+      </c>
+      <c r="E4" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="C4" s="8" t="s">
+      <c r="F4" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="D4" s="9" t="s">
+      <c r="G4" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="E4" s="8" t="s">
+      <c r="H4" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="F4" s="8" t="s">
+      <c r="I4" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="G4" s="10" t="s">
+      <c r="J4" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="H4" s="4"/>
-    </row>
-    <row r="5" spans="1:8" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="K4" s="4"/>
+    </row>
+    <row r="5" spans="1:11" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A5" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="B5" s="8" t="s">
+      <c r="B5" s="7" t="s">
+        <v>276</v>
+      </c>
+      <c r="C5" s="7" t="s">
+        <v>280</v>
+      </c>
+      <c r="D5" s="7" t="s">
+        <v>281</v>
+      </c>
+      <c r="E5" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="C5" s="8" t="s">
+      <c r="F5" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="D5" s="9" t="s">
+      <c r="G5" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="E5" s="8" t="s">
+      <c r="H5" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="F5" s="8" t="s">
+      <c r="I5" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="G5" s="10" t="s">
+      <c r="J5" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="H5" s="4"/>
-    </row>
-    <row r="6" spans="1:8" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="K5" s="4"/>
+    </row>
+    <row r="6" spans="1:11" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A6" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="B6" s="8" t="s">
+      <c r="B6" s="7" t="s">
+        <v>276</v>
+      </c>
+      <c r="C6" s="7" t="s">
+        <v>280</v>
+      </c>
+      <c r="D6" s="7" t="s">
+        <v>281</v>
+      </c>
+      <c r="E6" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="C6" s="8" t="s">
+      <c r="F6" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="D6" s="9" t="s">
+      <c r="G6" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="E6" s="8" t="s">
+      <c r="H6" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="F6" s="8" t="s">
+      <c r="I6" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="G6" s="10" t="s">
+      <c r="J6" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="H6" s="4"/>
-    </row>
-    <row r="7" spans="1:8" ht="25.5" x14ac:dyDescent="0.2">
+      <c r="K6" s="4"/>
+    </row>
+    <row r="7" spans="1:11" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A7" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="B7" s="8" t="s">
+      <c r="B7" s="7" t="s">
+        <v>276</v>
+      </c>
+      <c r="C7" s="7" t="s">
+        <v>280</v>
+      </c>
+      <c r="D7" s="7" t="s">
+        <v>281</v>
+      </c>
+      <c r="E7" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="C7" s="8" t="s">
+      <c r="F7" s="8" t="s">
         <v>24</v>
       </c>
-      <c r="D7" s="9" t="s">
+      <c r="G7" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="E7" s="8" t="s">
+      <c r="H7" s="8" t="s">
         <v>26</v>
       </c>
-      <c r="F7" s="8" t="s">
+      <c r="I7" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="G7" s="11" t="s">
+      <c r="J7" s="11" t="s">
         <v>28</v>
       </c>
-      <c r="H7" s="4"/>
-    </row>
-    <row r="8" spans="1:8" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="K7" s="4"/>
+    </row>
+    <row r="8" spans="1:11" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A8" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="B8" s="8" t="s">
+      <c r="B8" s="7" t="s">
+        <v>276</v>
+      </c>
+      <c r="C8" s="7" t="s">
+        <v>280</v>
+      </c>
+      <c r="D8" s="7" t="s">
+        <v>281</v>
+      </c>
+      <c r="E8" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="C8" s="8" t="s">
+      <c r="F8" s="8" t="s">
         <v>30</v>
       </c>
-      <c r="D8" s="9" t="s">
+      <c r="G8" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="E8" s="8" t="s">
+      <c r="H8" s="8" t="s">
         <v>32</v>
       </c>
-      <c r="F8" s="8" t="s">
+      <c r="I8" s="8" t="s">
         <v>33</v>
       </c>
-      <c r="G8" s="10" t="s">
+      <c r="J8" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="H8" s="4"/>
-    </row>
-    <row r="9" spans="1:8" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="K8" s="4"/>
+    </row>
+    <row r="9" spans="1:11" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A9" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="B9" s="8" t="s">
+      <c r="B9" s="7" t="s">
+        <v>276</v>
+      </c>
+      <c r="C9" s="7" t="s">
+        <v>280</v>
+      </c>
+      <c r="D9" s="7" t="s">
+        <v>281</v>
+      </c>
+      <c r="E9" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="C9" s="8" t="s">
+      <c r="F9" s="8" t="s">
         <v>35</v>
       </c>
-      <c r="D9" s="9" t="s">
+      <c r="G9" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="E9" s="8" t="s">
+      <c r="H9" s="8" t="s">
         <v>37</v>
       </c>
-      <c r="F9" s="8" t="s">
+      <c r="I9" s="8" t="s">
         <v>33</v>
       </c>
-      <c r="G9" s="10" t="s">
+      <c r="J9" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="H9" s="4"/>
-    </row>
-    <row r="10" spans="1:8" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="K9" s="4"/>
+    </row>
+    <row r="10" spans="1:11" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A10" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="B10" s="8" t="s">
+      <c r="B10" s="7" t="s">
+        <v>276</v>
+      </c>
+      <c r="C10" s="7" t="s">
+        <v>280</v>
+      </c>
+      <c r="D10" s="7" t="s">
+        <v>281</v>
+      </c>
+      <c r="E10" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="C10" s="12" t="s">
+      <c r="F10" s="12" t="s">
         <v>39</v>
       </c>
-      <c r="D10" s="13" t="s">
+      <c r="G10" s="13" t="s">
         <v>40</v>
       </c>
-      <c r="E10" s="8" t="s">
+      <c r="H10" s="8" t="s">
         <v>41</v>
       </c>
-      <c r="F10" s="8" t="s">
+      <c r="I10" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="G10" s="10" t="s">
+      <c r="J10" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="H10" s="4"/>
-    </row>
-    <row r="11" spans="1:8" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="K10" s="4"/>
+    </row>
+    <row r="11" spans="1:11" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A11" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="B11" s="8" t="s">
+      <c r="B11" s="7" t="s">
+        <v>276</v>
+      </c>
+      <c r="C11" s="7" t="s">
+        <v>280</v>
+      </c>
+      <c r="D11" s="7" t="s">
+        <v>281</v>
+      </c>
+      <c r="E11" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="C11" s="14" t="s">
+      <c r="F11" s="14" t="s">
         <v>43</v>
       </c>
-      <c r="D11" s="13" t="s">
+      <c r="G11" s="13" t="s">
         <v>44</v>
       </c>
-      <c r="E11" s="8" t="s">
+      <c r="H11" s="8" t="s">
         <v>45</v>
       </c>
-      <c r="F11" s="8" t="s">
+      <c r="I11" s="8" t="s">
         <v>33</v>
       </c>
-      <c r="G11" s="10" t="s">
+      <c r="J11" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="H11" s="4"/>
-    </row>
-    <row r="12" spans="1:8" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="K11" s="4"/>
+    </row>
+    <row r="12" spans="1:11" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A12" s="7" t="s">
         <v>46</v>
       </c>
-      <c r="B12" s="8" t="s">
+      <c r="B12" s="7" t="s">
+        <v>276</v>
+      </c>
+      <c r="C12" s="7" t="s">
+        <v>280</v>
+      </c>
+      <c r="D12" s="7" t="s">
+        <v>281</v>
+      </c>
+      <c r="E12" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="C12" s="12" t="s">
+      <c r="F12" s="12" t="s">
         <v>47</v>
       </c>
-      <c r="D12" s="13" t="s">
+      <c r="G12" s="13" t="s">
         <v>48</v>
       </c>
-      <c r="E12" s="12" t="s">
+      <c r="H12" s="12" t="s">
         <v>49</v>
       </c>
-      <c r="F12" s="8" t="s">
+      <c r="I12" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="G12" s="11" t="s">
+      <c r="J12" s="11" t="s">
         <v>28</v>
       </c>
-      <c r="H12" s="4"/>
-    </row>
-    <row r="13" spans="1:8" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="K12" s="4"/>
+    </row>
+    <row r="13" spans="1:11" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A13" s="7" t="s">
         <v>50</v>
       </c>
-      <c r="B13" s="8" t="s">
+      <c r="B13" s="7" t="s">
+        <v>276</v>
+      </c>
+      <c r="C13" s="7" t="s">
+        <v>280</v>
+      </c>
+      <c r="D13" s="7" t="s">
+        <v>281</v>
+      </c>
+      <c r="E13" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="C13" s="12" t="s">
+      <c r="F13" s="12" t="s">
         <v>51</v>
       </c>
-      <c r="D13" s="13" t="s">
+      <c r="G13" s="13" t="s">
         <v>52</v>
       </c>
-      <c r="E13" s="8" t="s">
+      <c r="H13" s="8" t="s">
         <v>53</v>
       </c>
-      <c r="F13" s="8" t="s">
+      <c r="I13" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="G13" s="10" t="s">
+      <c r="J13" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="H13" s="4"/>
-    </row>
-    <row r="14" spans="1:8" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="K13" s="4"/>
+    </row>
+    <row r="14" spans="1:11" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A14" s="7" t="s">
         <v>54</v>
       </c>
-      <c r="B14" s="8" t="s">
+      <c r="B14" s="7" t="s">
+        <v>276</v>
+      </c>
+      <c r="C14" s="7" t="s">
+        <v>280</v>
+      </c>
+      <c r="D14" s="7" t="s">
+        <v>281</v>
+      </c>
+      <c r="E14" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="C14" s="14" t="s">
+      <c r="F14" s="14" t="s">
         <v>55</v>
       </c>
-      <c r="D14" s="13" t="s">
+      <c r="G14" s="13" t="s">
         <v>56</v>
       </c>
-      <c r="E14" s="8" t="s">
+      <c r="H14" s="8" t="s">
         <v>57</v>
       </c>
-      <c r="F14" s="8" t="s">
+      <c r="I14" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="G14" s="10" t="s">
+      <c r="J14" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="H14" s="4"/>
-    </row>
-    <row r="15" spans="1:8" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="K14" s="4"/>
+    </row>
+    <row r="15" spans="1:11" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A15" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="B15" s="8" t="s">
+      <c r="B15" s="7" t="s">
+        <v>276</v>
+      </c>
+      <c r="C15" s="7" t="s">
+        <v>280</v>
+      </c>
+      <c r="D15" s="7" t="s">
+        <v>281</v>
+      </c>
+      <c r="E15" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="C15" s="14" t="s">
+      <c r="F15" s="14" t="s">
         <v>59</v>
       </c>
-      <c r="D15" s="13" t="s">
+      <c r="G15" s="13" t="s">
         <v>60</v>
       </c>
-      <c r="E15" s="8" t="s">
+      <c r="H15" s="8" t="s">
         <v>61</v>
       </c>
-      <c r="F15" s="8" t="s">
+      <c r="I15" s="8" t="s">
         <v>33</v>
       </c>
-      <c r="G15" s="10" t="s">
+      <c r="J15" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="H15" s="4"/>
-    </row>
-    <row r="16" spans="1:8" ht="25.5" x14ac:dyDescent="0.2">
+      <c r="K15" s="4"/>
+    </row>
+    <row r="16" spans="1:11" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A16" s="7" t="s">
         <v>62</v>
       </c>
-      <c r="B16" s="8" t="s">
+      <c r="B16" s="7" t="s">
+        <v>276</v>
+      </c>
+      <c r="C16" s="7" t="s">
+        <v>280</v>
+      </c>
+      <c r="D16" s="7" t="s">
+        <v>281</v>
+      </c>
+      <c r="E16" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="C16" s="12" t="s">
+      <c r="F16" s="12" t="s">
         <v>63</v>
       </c>
-      <c r="D16" s="15" t="s">
+      <c r="G16" s="15" t="s">
         <v>64</v>
       </c>
-      <c r="E16" s="12" t="s">
+      <c r="H16" s="12" t="s">
         <v>65</v>
       </c>
-      <c r="F16" s="8" t="s">
+      <c r="I16" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="G16" s="11" t="s">
+      <c r="J16" s="11" t="s">
         <v>28</v>
       </c>
-      <c r="H16" s="4"/>
-    </row>
-    <row r="17" spans="1:8" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="K16" s="4"/>
+    </row>
+    <row r="17" spans="1:11" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A17" s="7" t="s">
         <v>66</v>
       </c>
-      <c r="B17" s="8" t="s">
+      <c r="B17" s="7" t="s">
+        <v>276</v>
+      </c>
+      <c r="C17" s="7" t="s">
+        <v>280</v>
+      </c>
+      <c r="D17" s="7" t="s">
+        <v>281</v>
+      </c>
+      <c r="E17" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="C17" s="12" t="s">
+      <c r="F17" s="12" t="s">
         <v>67</v>
       </c>
-      <c r="D17" s="15" t="s">
+      <c r="G17" s="15" t="s">
         <v>68</v>
       </c>
-      <c r="E17" s="8" t="s">
+      <c r="H17" s="8" t="s">
         <v>69</v>
       </c>
-      <c r="F17" s="8" t="s">
+      <c r="I17" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="G17" s="10" t="s">
+      <c r="J17" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="H17" s="4"/>
-    </row>
-    <row r="18" spans="1:8" ht="51" x14ac:dyDescent="0.2">
+      <c r="K17" s="4"/>
+    </row>
+    <row r="18" spans="1:11" ht="51" x14ac:dyDescent="0.2">
       <c r="A18" s="7" t="s">
         <v>70</v>
       </c>
-      <c r="B18" s="8" t="s">
+      <c r="B18" s="7" t="s">
+        <v>276</v>
+      </c>
+      <c r="C18" s="7" t="s">
+        <v>280</v>
+      </c>
+      <c r="D18" s="7" t="s">
+        <v>281</v>
+      </c>
+      <c r="E18" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="C18" s="12" t="s">
+      <c r="F18" s="12" t="s">
         <v>71</v>
       </c>
-      <c r="D18" s="13" t="s">
+      <c r="G18" s="13" t="s">
         <v>72</v>
       </c>
-      <c r="E18" s="8" t="s">
+      <c r="H18" s="8" t="s">
         <v>73</v>
       </c>
-      <c r="F18" s="8" t="s">
+      <c r="I18" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="G18" s="10" t="s">
+      <c r="J18" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="H18" s="4"/>
-    </row>
-    <row r="19" spans="1:8" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="K18" s="4"/>
+    </row>
+    <row r="19" spans="1:11" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A19" s="7" t="s">
         <v>74</v>
       </c>
-      <c r="B19" s="8" t="s">
+      <c r="B19" s="7" t="s">
+        <v>276</v>
+      </c>
+      <c r="C19" s="7" t="s">
+        <v>280</v>
+      </c>
+      <c r="D19" s="7" t="s">
+        <v>281</v>
+      </c>
+      <c r="E19" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="C19" s="12" t="s">
+      <c r="F19" s="12" t="s">
         <v>75</v>
       </c>
-      <c r="D19" s="15" t="s">
+      <c r="G19" s="15" t="s">
         <v>76</v>
       </c>
-      <c r="E19" s="12" t="s">
+      <c r="H19" s="12" t="s">
         <v>77</v>
       </c>
-      <c r="F19" s="8" t="s">
+      <c r="I19" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="G19" s="11" t="s">
+      <c r="J19" s="11" t="s">
         <v>28</v>
       </c>
-      <c r="H19" s="4"/>
-    </row>
-    <row r="20" spans="1:8" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="K19" s="4"/>
+    </row>
+    <row r="20" spans="1:11" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A20" s="7" t="s">
         <v>78</v>
       </c>
-      <c r="B20" s="8" t="s">
+      <c r="B20" s="7" t="s">
+        <v>276</v>
+      </c>
+      <c r="C20" s="7" t="s">
+        <v>280</v>
+      </c>
+      <c r="D20" s="7" t="s">
+        <v>281</v>
+      </c>
+      <c r="E20" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="C20" s="12" t="s">
+      <c r="F20" s="12" t="s">
         <v>79</v>
       </c>
-      <c r="D20" s="15" t="s">
+      <c r="G20" s="15" t="s">
         <v>80</v>
       </c>
-      <c r="E20" s="8" t="s">
+      <c r="H20" s="8" t="s">
         <v>81</v>
       </c>
-      <c r="F20" s="8" t="s">
+      <c r="I20" s="8" t="s">
         <v>33</v>
       </c>
-      <c r="G20" s="10" t="s">
+      <c r="J20" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="H20" s="4"/>
-    </row>
-    <row r="21" spans="1:8" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="K20" s="4"/>
+    </row>
+    <row r="21" spans="1:11" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A21" s="7" t="s">
         <v>82</v>
       </c>
-      <c r="B21" s="8" t="s">
+      <c r="B21" s="7" t="s">
+        <v>276</v>
+      </c>
+      <c r="C21" s="7" t="s">
+        <v>280</v>
+      </c>
+      <c r="D21" s="7" t="s">
+        <v>281</v>
+      </c>
+      <c r="E21" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="C21" s="12" t="s">
+      <c r="F21" s="12" t="s">
         <v>83</v>
       </c>
-      <c r="D21" s="13" t="s">
+      <c r="G21" s="13" t="s">
         <v>84</v>
       </c>
-      <c r="E21" s="12" t="s">
+      <c r="H21" s="12" t="s">
         <v>77</v>
       </c>
-      <c r="F21" s="8" t="s">
+      <c r="I21" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="G21" s="11" t="s">
+      <c r="J21" s="11" t="s">
         <v>28</v>
       </c>
-      <c r="H21" s="4"/>
-    </row>
-    <row r="22" spans="1:8" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="K21" s="4"/>
+    </row>
+    <row r="22" spans="1:11" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A22" s="7" t="s">
         <v>85</v>
       </c>
-      <c r="B22" s="8" t="s">
+      <c r="B22" s="7" t="s">
+        <v>276</v>
+      </c>
+      <c r="C22" s="7" t="s">
+        <v>280</v>
+      </c>
+      <c r="D22" s="7" t="s">
+        <v>281</v>
+      </c>
+      <c r="E22" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="C22" s="12" t="s">
+      <c r="F22" s="12" t="s">
         <v>86</v>
       </c>
-      <c r="D22" s="13" t="s">
+      <c r="G22" s="13" t="s">
         <v>87</v>
       </c>
-      <c r="E22" s="12" t="s">
+      <c r="H22" s="12" t="s">
         <v>77</v>
       </c>
-      <c r="F22" s="8" t="s">
+      <c r="I22" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="G22" s="11" t="s">
+      <c r="J22" s="11" t="s">
         <v>28</v>
       </c>
-      <c r="H22" s="4"/>
-    </row>
-    <row r="23" spans="1:8" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="K22" s="4"/>
+    </row>
+    <row r="23" spans="1:11" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A23" s="7" t="s">
         <v>88</v>
       </c>
-      <c r="B23" s="8" t="s">
+      <c r="B23" s="7" t="s">
+        <v>276</v>
+      </c>
+      <c r="C23" s="7" t="s">
+        <v>280</v>
+      </c>
+      <c r="D23" s="7" t="s">
+        <v>281</v>
+      </c>
+      <c r="E23" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="C23" s="12" t="s">
+      <c r="F23" s="12" t="s">
         <v>89</v>
       </c>
-      <c r="D23" s="13" t="s">
+      <c r="G23" s="13" t="s">
         <v>90</v>
       </c>
-      <c r="E23" s="12" t="s">
+      <c r="H23" s="12" t="s">
         <v>77</v>
       </c>
-      <c r="F23" s="8" t="s">
+      <c r="I23" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="G23" s="11" t="s">
+      <c r="J23" s="11" t="s">
         <v>28</v>
       </c>
-      <c r="H23" s="4"/>
-    </row>
-    <row r="24" spans="1:8" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="K23" s="4"/>
+    </row>
+    <row r="24" spans="1:11" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A24" s="7" t="s">
         <v>91</v>
       </c>
-      <c r="B24" s="8" t="s">
+      <c r="B24" s="7" t="s">
+        <v>276</v>
+      </c>
+      <c r="C24" s="7" t="s">
+        <v>280</v>
+      </c>
+      <c r="D24" s="7" t="s">
+        <v>281</v>
+      </c>
+      <c r="E24" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="C24" s="12" t="s">
+      <c r="F24" s="12" t="s">
         <v>92</v>
       </c>
-      <c r="D24" s="13" t="s">
+      <c r="G24" s="13" t="s">
         <v>93</v>
       </c>
-      <c r="E24" s="12" t="s">
+      <c r="H24" s="12" t="s">
         <v>77</v>
       </c>
-      <c r="F24" s="8" t="s">
+      <c r="I24" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="G24" s="11" t="s">
+      <c r="J24" s="11" t="s">
         <v>28</v>
       </c>
-      <c r="H24" s="4"/>
-    </row>
-    <row r="25" spans="1:8" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="K24" s="4"/>
+    </row>
+    <row r="25" spans="1:11" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A25" s="7" t="s">
         <v>94</v>
       </c>
-      <c r="B25" s="8" t="s">
+      <c r="B25" s="7" t="s">
+        <v>276</v>
+      </c>
+      <c r="C25" s="7" t="s">
+        <v>280</v>
+      </c>
+      <c r="D25" s="7" t="s">
+        <v>281</v>
+      </c>
+      <c r="E25" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="C25" s="12" t="s">
+      <c r="F25" s="12" t="s">
         <v>95</v>
       </c>
-      <c r="D25" s="15" t="s">
+      <c r="G25" s="15" t="s">
         <v>96</v>
       </c>
-      <c r="E25" s="8" t="s">
+      <c r="H25" s="8" t="s">
         <v>97</v>
       </c>
-      <c r="F25" s="8" t="s">
+      <c r="I25" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="G25" s="10" t="s">
+      <c r="J25" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="H25" s="4"/>
-    </row>
-    <row r="26" spans="1:8" ht="51" x14ac:dyDescent="0.2">
+      <c r="K25" s="4"/>
+    </row>
+    <row r="26" spans="1:11" ht="51" x14ac:dyDescent="0.2">
       <c r="A26" s="7" t="s">
         <v>98</v>
       </c>
-      <c r="B26" s="8" t="s">
+      <c r="B26" s="7" t="s">
+        <v>276</v>
+      </c>
+      <c r="C26" s="7" t="s">
+        <v>280</v>
+      </c>
+      <c r="D26" s="7" t="s">
+        <v>281</v>
+      </c>
+      <c r="E26" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="C26" s="12" t="s">
+      <c r="F26" s="12" t="s">
         <v>99</v>
       </c>
-      <c r="D26" s="13" t="s">
+      <c r="G26" s="13" t="s">
         <v>100</v>
       </c>
-      <c r="E26" s="8" t="s">
+      <c r="H26" s="8" t="s">
         <v>101</v>
       </c>
-      <c r="F26" s="8" t="s">
+      <c r="I26" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="G26" s="10" t="s">
+      <c r="J26" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="H26" s="4"/>
-    </row>
-    <row r="27" spans="1:8" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="K26" s="4"/>
+    </row>
+    <row r="27" spans="1:11" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A27" s="7" t="s">
         <v>102</v>
       </c>
-      <c r="B27" s="8" t="s">
+      <c r="B27" s="7" t="s">
+        <v>276</v>
+      </c>
+      <c r="C27" s="7" t="s">
+        <v>280</v>
+      </c>
+      <c r="D27" s="7" t="s">
+        <v>281</v>
+      </c>
+      <c r="E27" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="C27" s="12" t="s">
+      <c r="F27" s="12" t="s">
         <v>103</v>
       </c>
-      <c r="D27" s="15" t="s">
+      <c r="G27" s="15" t="s">
         <v>104</v>
       </c>
-      <c r="E27" s="14" t="s">
+      <c r="H27" s="14" t="s">
         <v>105</v>
       </c>
-      <c r="F27" s="8" t="s">
+      <c r="I27" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="G27" s="11" t="s">
+      <c r="J27" s="11" t="s">
         <v>28</v>
       </c>
-      <c r="H27" s="4"/>
-    </row>
-    <row r="28" spans="1:8" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="K27" s="4"/>
+    </row>
+    <row r="28" spans="1:11" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A28" s="7" t="s">
         <v>106</v>
       </c>
-      <c r="B28" s="8" t="s">
+      <c r="B28" s="7" t="s">
+        <v>276</v>
+      </c>
+      <c r="C28" s="7" t="s">
+        <v>280</v>
+      </c>
+      <c r="D28" s="7" t="s">
+        <v>281</v>
+      </c>
+      <c r="E28" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="C28" s="12" t="s">
+      <c r="F28" s="12" t="s">
         <v>107</v>
       </c>
-      <c r="D28" s="15" t="s">
+      <c r="G28" s="15" t="s">
         <v>108</v>
       </c>
-      <c r="E28" s="8" t="s">
+      <c r="H28" s="8" t="s">
         <v>81</v>
       </c>
-      <c r="F28" s="8" t="s">
+      <c r="I28" s="8" t="s">
         <v>33</v>
       </c>
-      <c r="G28" s="10" t="s">
+      <c r="J28" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="H28" s="4"/>
-    </row>
-    <row r="29" spans="1:8" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="K28" s="4"/>
+    </row>
+    <row r="29" spans="1:11" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A29" s="7" t="s">
         <v>109</v>
       </c>
-      <c r="B29" s="8" t="s">
+      <c r="B29" s="7" t="s">
+        <v>276</v>
+      </c>
+      <c r="C29" s="7" t="s">
+        <v>280</v>
+      </c>
+      <c r="D29" s="7" t="s">
+        <v>281</v>
+      </c>
+      <c r="E29" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="C29" s="12" t="s">
+      <c r="F29" s="12" t="s">
         <v>110</v>
       </c>
-      <c r="D29" s="13" t="s">
+      <c r="G29" s="13" t="s">
         <v>111</v>
       </c>
-      <c r="E29" s="14" t="s">
+      <c r="H29" s="14" t="s">
         <v>105</v>
       </c>
-      <c r="F29" s="8" t="s">
+      <c r="I29" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="G29" s="11" t="s">
+      <c r="J29" s="11" t="s">
         <v>28</v>
       </c>
-      <c r="H29" s="4"/>
-    </row>
-    <row r="30" spans="1:8" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="K29" s="4"/>
+    </row>
+    <row r="30" spans="1:11" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A30" s="7" t="s">
         <v>112</v>
       </c>
-      <c r="B30" s="8" t="s">
+      <c r="B30" s="7" t="s">
+        <v>276</v>
+      </c>
+      <c r="C30" s="7" t="s">
+        <v>280</v>
+      </c>
+      <c r="D30" s="7" t="s">
+        <v>281</v>
+      </c>
+      <c r="E30" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="C30" s="12" t="s">
+      <c r="F30" s="12" t="s">
         <v>113</v>
       </c>
-      <c r="D30" s="13" t="s">
+      <c r="G30" s="13" t="s">
         <v>114</v>
       </c>
-      <c r="E30" s="14" t="s">
+      <c r="H30" s="14" t="s">
         <v>105</v>
       </c>
-      <c r="F30" s="8" t="s">
+      <c r="I30" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="G30" s="11" t="s">
+      <c r="J30" s="11" t="s">
         <v>28</v>
       </c>
-      <c r="H30" s="4"/>
-    </row>
-    <row r="31" spans="1:8" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="K30" s="4"/>
+    </row>
+    <row r="31" spans="1:11" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A31" s="7" t="s">
         <v>115</v>
       </c>
-      <c r="B31" s="8" t="s">
+      <c r="B31" s="7" t="s">
+        <v>276</v>
+      </c>
+      <c r="C31" s="7" t="s">
+        <v>280</v>
+      </c>
+      <c r="D31" s="7" t="s">
+        <v>281</v>
+      </c>
+      <c r="E31" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="C31" s="12" t="s">
+      <c r="F31" s="12" t="s">
         <v>116</v>
       </c>
-      <c r="D31" s="13" t="s">
+      <c r="G31" s="13" t="s">
         <v>117</v>
       </c>
-      <c r="E31" s="14" t="s">
+      <c r="H31" s="14" t="s">
         <v>105</v>
       </c>
-      <c r="F31" s="8" t="s">
+      <c r="I31" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="G31" s="11" t="s">
+      <c r="J31" s="11" t="s">
         <v>28</v>
       </c>
-      <c r="H31" s="4"/>
-    </row>
-    <row r="32" spans="1:8" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="K31" s="4"/>
+    </row>
+    <row r="32" spans="1:11" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A32" s="7" t="s">
         <v>118</v>
       </c>
-      <c r="B32" s="8" t="s">
+      <c r="B32" s="7" t="s">
+        <v>276</v>
+      </c>
+      <c r="C32" s="7" t="s">
+        <v>280</v>
+      </c>
+      <c r="D32" s="7" t="s">
+        <v>281</v>
+      </c>
+      <c r="E32" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="C32" s="12" t="s">
+      <c r="F32" s="12" t="s">
         <v>119</v>
       </c>
-      <c r="D32" s="13" t="s">
+      <c r="G32" s="13" t="s">
         <v>120</v>
       </c>
-      <c r="E32" s="14" t="s">
+      <c r="H32" s="14" t="s">
         <v>105</v>
       </c>
-      <c r="F32" s="8" t="s">
+      <c r="I32" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="G32" s="11" t="s">
+      <c r="J32" s="11" t="s">
         <v>28</v>
       </c>
-      <c r="H32" s="4"/>
-    </row>
-    <row r="33" spans="1:8" ht="25.5" x14ac:dyDescent="0.2">
+      <c r="K32" s="4"/>
+    </row>
+    <row r="33" spans="1:11" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A33" s="7" t="s">
         <v>121</v>
       </c>
-      <c r="B33" s="8" t="s">
+      <c r="B33" s="7" t="s">
+        <v>276</v>
+      </c>
+      <c r="C33" s="7" t="s">
+        <v>280</v>
+      </c>
+      <c r="D33" s="7" t="s">
+        <v>281</v>
+      </c>
+      <c r="E33" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="C33" s="12" t="s">
+      <c r="F33" s="12" t="s">
         <v>122</v>
       </c>
-      <c r="D33" s="13" t="s">
+      <c r="G33" s="13" t="s">
         <v>123</v>
       </c>
-      <c r="E33" s="14" t="s">
+      <c r="H33" s="14" t="s">
         <v>124</v>
       </c>
-      <c r="F33" s="8" t="s">
+      <c r="I33" s="8" t="s">
         <v>33</v>
       </c>
-      <c r="G33" s="10" t="s">
+      <c r="J33" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="H33" s="4"/>
-    </row>
-    <row r="34" spans="1:8" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="K33" s="4"/>
+    </row>
+    <row r="34" spans="1:11" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A34" s="7" t="s">
         <v>125</v>
       </c>
-      <c r="B34" s="8" t="s">
+      <c r="B34" s="7" t="s">
+        <v>276</v>
+      </c>
+      <c r="C34" s="7" t="s">
+        <v>280</v>
+      </c>
+      <c r="D34" s="7" t="s">
+        <v>281</v>
+      </c>
+      <c r="E34" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="C34" s="12" t="s">
+      <c r="F34" s="12" t="s">
         <v>126</v>
       </c>
-      <c r="D34" s="13" t="s">
+      <c r="G34" s="13" t="s">
         <v>127</v>
       </c>
-      <c r="E34" s="14" t="s">
+      <c r="H34" s="14" t="s">
         <v>128</v>
       </c>
-      <c r="F34" s="8" t="s">
+      <c r="I34" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="G34" s="11" t="s">
+      <c r="J34" s="11" t="s">
         <v>28</v>
       </c>
-      <c r="H34" s="4"/>
-    </row>
-    <row r="35" spans="1:8" ht="25.5" x14ac:dyDescent="0.2">
+      <c r="K34" s="4"/>
+    </row>
+    <row r="35" spans="1:11" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A35" s="7" t="s">
         <v>129</v>
       </c>
-      <c r="B35" s="8" t="s">
+      <c r="B35" s="7" t="s">
+        <v>276</v>
+      </c>
+      <c r="C35" s="7" t="s">
+        <v>280</v>
+      </c>
+      <c r="D35" s="7" t="s">
+        <v>281</v>
+      </c>
+      <c r="E35" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="C35" s="12" t="s">
+      <c r="F35" s="12" t="s">
         <v>130</v>
       </c>
-      <c r="D35" s="13" t="s">
+      <c r="G35" s="13" t="s">
         <v>131</v>
       </c>
-      <c r="E35" s="14" t="s">
+      <c r="H35" s="14" t="s">
         <v>128</v>
       </c>
-      <c r="F35" s="8" t="s">
+      <c r="I35" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="G35" s="11" t="s">
+      <c r="J35" s="11" t="s">
         <v>28</v>
       </c>
-      <c r="H35" s="4"/>
-    </row>
-    <row r="36" spans="1:8" ht="15" x14ac:dyDescent="0.2">
+      <c r="K35" s="4"/>
+    </row>
+    <row r="36" spans="1:11" ht="15" x14ac:dyDescent="0.2">
       <c r="A36" s="7" t="s">
         <v>132</v>
       </c>
-      <c r="B36" s="8" t="s">
+      <c r="B36" s="7" t="s">
+        <v>276</v>
+      </c>
+      <c r="C36" s="7" t="s">
+        <v>280</v>
+      </c>
+      <c r="D36" s="7" t="s">
+        <v>281</v>
+      </c>
+      <c r="E36" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="C36" s="12" t="s">
+      <c r="F36" s="12" t="s">
         <v>133</v>
       </c>
-      <c r="D36" s="16" t="s">
+      <c r="G36" s="16" t="s">
         <v>134</v>
       </c>
-      <c r="E36" s="14" t="s">
+      <c r="H36" s="14" t="s">
         <v>135</v>
       </c>
-      <c r="F36" s="8" t="s">
+      <c r="I36" s="8" t="s">
         <v>33</v>
       </c>
-      <c r="G36" s="10" t="s">
+      <c r="J36" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="H36" s="4"/>
-    </row>
-    <row r="37" spans="1:8" ht="15" x14ac:dyDescent="0.2">
+      <c r="K36" s="4"/>
+    </row>
+    <row r="37" spans="1:11" ht="15" x14ac:dyDescent="0.2">
       <c r="A37" s="7" t="s">
         <v>136</v>
       </c>
-      <c r="B37" s="8" t="s">
+      <c r="B37" s="7" t="s">
+        <v>276</v>
+      </c>
+      <c r="C37" s="7" t="s">
+        <v>280</v>
+      </c>
+      <c r="D37" s="7" t="s">
+        <v>281</v>
+      </c>
+      <c r="E37" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="C37" s="12" t="s">
+      <c r="F37" s="12" t="s">
         <v>137</v>
       </c>
-      <c r="D37" s="16" t="s">
+      <c r="G37" s="16" t="s">
         <v>138</v>
       </c>
-      <c r="E37" s="14" t="s">
+      <c r="H37" s="14" t="s">
         <v>139</v>
       </c>
-      <c r="F37" s="8" t="s">
+      <c r="I37" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="G37" s="11" t="s">
+      <c r="J37" s="11" t="s">
         <v>28</v>
       </c>
-      <c r="H37" s="4"/>
-    </row>
-    <row r="38" spans="1:8" ht="15" x14ac:dyDescent="0.2">
+      <c r="K37" s="4"/>
+    </row>
+    <row r="38" spans="1:11" ht="15" x14ac:dyDescent="0.2">
       <c r="A38" s="7" t="s">
         <v>140</v>
       </c>
-      <c r="B38" s="8" t="s">
+      <c r="B38" s="7" t="s">
+        <v>276</v>
+      </c>
+      <c r="C38" s="7" t="s">
+        <v>280</v>
+      </c>
+      <c r="D38" s="7" t="s">
+        <v>281</v>
+      </c>
+      <c r="E38" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="C38" s="12" t="s">
+      <c r="F38" s="12" t="s">
         <v>141</v>
       </c>
-      <c r="D38" s="16" t="s">
+      <c r="G38" s="16" t="s">
         <v>142</v>
       </c>
-      <c r="E38" s="14" t="s">
+      <c r="H38" s="14" t="s">
         <v>139</v>
       </c>
-      <c r="F38" s="8" t="s">
+      <c r="I38" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="G38" s="11" t="s">
+      <c r="J38" s="11" t="s">
         <v>28</v>
       </c>
-      <c r="H38" s="4"/>
-    </row>
-    <row r="39" spans="1:8" ht="15" x14ac:dyDescent="0.2">
+      <c r="K38" s="4"/>
+    </row>
+    <row r="39" spans="1:11" ht="15" x14ac:dyDescent="0.2">
       <c r="A39" s="7" t="s">
         <v>143</v>
       </c>
-      <c r="B39" s="8" t="s">
+      <c r="B39" s="7" t="s">
+        <v>276</v>
+      </c>
+      <c r="C39" s="7" t="s">
+        <v>280</v>
+      </c>
+      <c r="D39" s="7" t="s">
+        <v>281</v>
+      </c>
+      <c r="E39" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="C39" s="12" t="s">
+      <c r="F39" s="12" t="s">
         <v>144</v>
       </c>
-      <c r="D39" s="16" t="s">
+      <c r="G39" s="16" t="s">
         <v>145</v>
       </c>
-      <c r="E39" s="12" t="s">
+      <c r="H39" s="12" t="s">
         <v>146</v>
       </c>
-      <c r="F39" s="8" t="s">
+      <c r="I39" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="G39" s="10" t="s">
+      <c r="J39" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="H39" s="4"/>
-    </row>
-    <row r="40" spans="1:8" ht="15" x14ac:dyDescent="0.2">
+      <c r="K39" s="4"/>
+    </row>
+    <row r="40" spans="1:11" ht="15" x14ac:dyDescent="0.2">
       <c r="A40" s="7" t="s">
         <v>147</v>
       </c>
-      <c r="B40" s="8" t="s">
+      <c r="B40" s="7" t="s">
+        <v>276</v>
+      </c>
+      <c r="C40" s="7" t="s">
+        <v>280</v>
+      </c>
+      <c r="D40" s="7" t="s">
+        <v>281</v>
+      </c>
+      <c r="E40" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="C40" s="12" t="s">
+      <c r="F40" s="12" t="s">
         <v>148</v>
       </c>
-      <c r="D40" s="16" t="s">
+      <c r="G40" s="16" t="s">
         <v>149</v>
       </c>
-      <c r="E40" s="12" t="s">
+      <c r="H40" s="12" t="s">
         <v>150</v>
       </c>
-      <c r="F40" s="8" t="s">
+      <c r="I40" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="G40" s="11" t="s">
+      <c r="J40" s="11" t="s">
         <v>28</v>
       </c>
-      <c r="H40" s="4"/>
-    </row>
-    <row r="41" spans="1:8" ht="15" x14ac:dyDescent="0.2">
+      <c r="K40" s="4"/>
+    </row>
+    <row r="41" spans="1:11" ht="15" x14ac:dyDescent="0.2">
       <c r="A41" s="7" t="s">
         <v>151</v>
       </c>
-      <c r="B41" s="8" t="s">
+      <c r="B41" s="7" t="s">
+        <v>276</v>
+      </c>
+      <c r="C41" s="7" t="s">
+        <v>280</v>
+      </c>
+      <c r="D41" s="7" t="s">
+        <v>281</v>
+      </c>
+      <c r="E41" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="C41" s="12" t="s">
+      <c r="F41" s="12" t="s">
         <v>152</v>
       </c>
-      <c r="D41" s="16" t="s">
+      <c r="G41" s="16" t="s">
         <v>153</v>
       </c>
-      <c r="E41" s="12" t="s">
+      <c r="H41" s="12" t="s">
         <v>154</v>
       </c>
-      <c r="F41" s="8" t="s">
+      <c r="I41" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="G41" s="11" t="s">
+      <c r="J41" s="11" t="s">
         <v>28</v>
       </c>
-      <c r="H41" s="4"/>
-    </row>
-    <row r="42" spans="1:8" ht="15" x14ac:dyDescent="0.2">
+      <c r="K41" s="4"/>
+    </row>
+    <row r="42" spans="1:11" ht="15" x14ac:dyDescent="0.2">
       <c r="A42" s="7" t="s">
         <v>155</v>
       </c>
-      <c r="B42" s="8" t="s">
+      <c r="B42" s="7" t="s">
+        <v>276</v>
+      </c>
+      <c r="C42" s="7" t="s">
+        <v>280</v>
+      </c>
+      <c r="D42" s="7" t="s">
+        <v>281</v>
+      </c>
+      <c r="E42" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="C42" s="12" t="s">
+      <c r="F42" s="12" t="s">
         <v>156</v>
       </c>
-      <c r="D42" s="16" t="s">
+      <c r="G42" s="16" t="s">
         <v>157</v>
       </c>
-      <c r="E42" s="8" t="s">
+      <c r="H42" s="8" t="s">
         <v>158</v>
       </c>
-      <c r="F42" s="8" t="s">
+      <c r="I42" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="G42" s="10" t="s">
+      <c r="J42" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="H42" s="4"/>
-    </row>
-    <row r="43" spans="1:8" ht="60" x14ac:dyDescent="0.2">
+      <c r="K42" s="4"/>
+    </row>
+    <row r="43" spans="1:11" ht="60" x14ac:dyDescent="0.2">
       <c r="A43" s="7" t="s">
         <v>159</v>
       </c>
-      <c r="B43" s="8" t="s">
+      <c r="B43" s="7" t="s">
+        <v>276</v>
+      </c>
+      <c r="C43" s="7" t="s">
+        <v>280</v>
+      </c>
+      <c r="D43" s="7" t="s">
+        <v>281</v>
+      </c>
+      <c r="E43" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="C43" s="12" t="s">
+      <c r="F43" s="12" t="s">
         <v>160</v>
       </c>
-      <c r="D43" s="16" t="s">
+      <c r="G43" s="16" t="s">
         <v>161</v>
       </c>
-      <c r="E43" s="8" t="s">
+      <c r="H43" s="8" t="s">
         <v>162</v>
       </c>
-      <c r="F43" s="8" t="s">
+      <c r="I43" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="G43" s="10" t="s">
+      <c r="J43" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="H43" s="4"/>
-    </row>
-    <row r="44" spans="1:8" ht="15" x14ac:dyDescent="0.2">
+      <c r="K43" s="4"/>
+    </row>
+    <row r="44" spans="1:11" ht="15" x14ac:dyDescent="0.2">
       <c r="A44" s="7" t="s">
         <v>163</v>
       </c>
-      <c r="B44" s="8" t="s">
+      <c r="B44" s="7" t="s">
+        <v>276</v>
+      </c>
+      <c r="C44" s="7" t="s">
+        <v>280</v>
+      </c>
+      <c r="D44" s="7" t="s">
+        <v>281</v>
+      </c>
+      <c r="E44" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="C44" s="12" t="s">
+      <c r="F44" s="12" t="s">
         <v>164</v>
       </c>
-      <c r="D44" s="16" t="s">
+      <c r="G44" s="16" t="s">
         <v>165</v>
       </c>
-      <c r="E44" s="14" t="s">
+      <c r="H44" s="14" t="s">
         <v>166</v>
       </c>
-      <c r="F44" s="8" t="s">
+      <c r="I44" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="G44" s="11" t="s">
+      <c r="J44" s="11" t="s">
         <v>28</v>
       </c>
-      <c r="H44" s="4"/>
-    </row>
-    <row r="45" spans="1:8" ht="15" x14ac:dyDescent="0.2">
+      <c r="K44" s="4"/>
+    </row>
+    <row r="45" spans="1:11" ht="15" x14ac:dyDescent="0.2">
       <c r="A45" s="7" t="s">
         <v>167</v>
       </c>
-      <c r="B45" s="8" t="s">
+      <c r="B45" s="7" t="s">
+        <v>276</v>
+      </c>
+      <c r="C45" s="7" t="s">
+        <v>280</v>
+      </c>
+      <c r="D45" s="7" t="s">
+        <v>281</v>
+      </c>
+      <c r="E45" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="C45" s="12" t="s">
+      <c r="F45" s="12" t="s">
         <v>168</v>
       </c>
-      <c r="D45" s="16" t="s">
+      <c r="G45" s="16" t="s">
         <v>169</v>
       </c>
-      <c r="E45" s="12" t="s">
+      <c r="H45" s="12" t="s">
         <v>154</v>
       </c>
-      <c r="F45" s="8" t="s">
+      <c r="I45" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="G45" s="11" t="s">
+      <c r="J45" s="11" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="46" spans="1:8" ht="15" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:11" ht="15" x14ac:dyDescent="0.2">
       <c r="A46" s="7" t="s">
         <v>170</v>
       </c>
-      <c r="B46" s="8" t="s">
+      <c r="B46" s="7" t="s">
+        <v>276</v>
+      </c>
+      <c r="C46" s="7" t="s">
+        <v>280</v>
+      </c>
+      <c r="D46" s="7" t="s">
+        <v>281</v>
+      </c>
+      <c r="E46" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="C46" s="14" t="s">
+      <c r="F46" s="14" t="s">
         <v>171</v>
       </c>
-      <c r="D46" s="16" t="s">
+      <c r="G46" s="16" t="s">
         <v>172</v>
       </c>
-      <c r="E46" s="14" t="s">
+      <c r="H46" s="14" t="s">
         <v>173</v>
       </c>
-      <c r="F46" s="8" t="s">
+      <c r="I46" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="G46" s="11" t="s">
+      <c r="J46" s="11" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="47" spans="1:8" ht="53.25" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:11" ht="53.25" x14ac:dyDescent="0.2">
       <c r="A47" s="7" t="s">
         <v>174</v>
       </c>
-      <c r="B47" s="8" t="s">
+      <c r="B47" s="7" t="s">
+        <v>276</v>
+      </c>
+      <c r="C47" s="7" t="s">
+        <v>280</v>
+      </c>
+      <c r="D47" s="7" t="s">
+        <v>281</v>
+      </c>
+      <c r="E47" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="C47" s="14" t="s">
+      <c r="F47" s="14" t="s">
         <v>175</v>
       </c>
-      <c r="D47" s="16" t="s">
+      <c r="G47" s="16" t="s">
         <v>176</v>
       </c>
-      <c r="E47" s="8" t="s">
+      <c r="H47" s="8" t="s">
         <v>177</v>
       </c>
-      <c r="F47" s="8" t="s">
+      <c r="I47" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="G47" s="10" t="s">
+      <c r="J47" s="10" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="48" spans="1:8" ht="15" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:11" ht="15" x14ac:dyDescent="0.2">
       <c r="A48" s="7" t="s">
         <v>178</v>
       </c>
-      <c r="B48" s="8" t="s">
+      <c r="B48" s="7" t="s">
+        <v>276</v>
+      </c>
+      <c r="C48" s="7" t="s">
+        <v>280</v>
+      </c>
+      <c r="D48" s="7" t="s">
+        <v>281</v>
+      </c>
+      <c r="E48" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="C48" s="14" t="s">
+      <c r="F48" s="14" t="s">
         <v>179</v>
       </c>
-      <c r="D48" s="16" t="s">
+      <c r="G48" s="16" t="s">
         <v>180</v>
       </c>
-      <c r="E48" s="14" t="s">
+      <c r="H48" s="14" t="s">
         <v>181</v>
       </c>
-      <c r="F48" s="8" t="s">
+      <c r="I48" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="G48" s="11" t="s">
+      <c r="J48" s="11" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="49" spans="1:17" ht="15" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:20" ht="15" x14ac:dyDescent="0.2">
       <c r="A49" s="7" t="s">
         <v>182</v>
       </c>
-      <c r="B49" s="8" t="s">
+      <c r="B49" s="7" t="s">
+        <v>276</v>
+      </c>
+      <c r="C49" s="7" t="s">
+        <v>280</v>
+      </c>
+      <c r="D49" s="7" t="s">
+        <v>281</v>
+      </c>
+      <c r="E49" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="C49" s="12" t="s">
+      <c r="F49" s="12" t="s">
         <v>183</v>
       </c>
-      <c r="D49" s="16" t="s">
+      <c r="G49" s="16" t="s">
         <v>184</v>
       </c>
-      <c r="E49" s="12" t="s">
+      <c r="H49" s="12" t="s">
         <v>154</v>
       </c>
-      <c r="F49" s="8" t="s">
+      <c r="I49" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="G49" s="11" t="s">
+      <c r="J49" s="11" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="50" spans="1:17" ht="15" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:20" ht="15" x14ac:dyDescent="0.2">
       <c r="A50" s="7" t="s">
         <v>185</v>
       </c>
-      <c r="B50" s="8" t="s">
+      <c r="B50" s="7" t="s">
+        <v>276</v>
+      </c>
+      <c r="C50" s="7" t="s">
+        <v>280</v>
+      </c>
+      <c r="D50" s="7" t="s">
+        <v>281</v>
+      </c>
+      <c r="E50" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="C50" s="14" t="s">
+      <c r="F50" s="14" t="s">
         <v>186</v>
       </c>
-      <c r="D50" s="16" t="s">
+      <c r="G50" s="16" t="s">
         <v>187</v>
       </c>
-      <c r="E50" s="14" t="s">
+      <c r="H50" s="14" t="s">
         <v>188</v>
       </c>
-      <c r="F50" s="8" t="s">
+      <c r="I50" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="G50" s="11" t="s">
+      <c r="J50" s="11" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="51" spans="1:17" ht="27.75" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:20" ht="27.75" x14ac:dyDescent="0.2">
       <c r="A51" s="7" t="s">
         <v>189</v>
       </c>
-      <c r="B51" s="8" t="s">
+      <c r="B51" s="7" t="s">
+        <v>276</v>
+      </c>
+      <c r="C51" s="7" t="s">
+        <v>280</v>
+      </c>
+      <c r="D51" s="7" t="s">
+        <v>281</v>
+      </c>
+      <c r="E51" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="C51" s="14" t="s">
+      <c r="F51" s="14" t="s">
         <v>190</v>
       </c>
-      <c r="D51" s="16" t="s">
+      <c r="G51" s="16" t="s">
         <v>191</v>
       </c>
-      <c r="E51" s="8" t="s">
+      <c r="H51" s="8" t="s">
         <v>192</v>
       </c>
-      <c r="F51" s="8" t="s">
+      <c r="I51" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="G51" s="10" t="s">
+      <c r="J51" s="10" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="52" spans="1:17" ht="15" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:20" ht="15" x14ac:dyDescent="0.2">
       <c r="A52" s="7" t="s">
         <v>193</v>
       </c>
-      <c r="B52" s="8" t="s">
+      <c r="B52" s="7" t="s">
+        <v>276</v>
+      </c>
+      <c r="C52" s="7" t="s">
+        <v>280</v>
+      </c>
+      <c r="D52" s="7" t="s">
+        <v>281</v>
+      </c>
+      <c r="E52" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="C52" s="12" t="s">
+      <c r="F52" s="12" t="s">
         <v>194</v>
       </c>
-      <c r="D52" s="16" t="s">
+      <c r="G52" s="16" t="s">
         <v>195</v>
       </c>
-      <c r="E52" s="14" t="s">
+      <c r="H52" s="14" t="s">
         <v>196</v>
       </c>
-      <c r="F52" s="8" t="s">
+      <c r="I52" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="G52" s="11" t="s">
+      <c r="J52" s="11" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="53" spans="1:17" ht="15" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:20" ht="15" x14ac:dyDescent="0.2">
       <c r="A53" s="7" t="s">
         <v>197</v>
       </c>
-      <c r="B53" s="8" t="s">
+      <c r="B53" s="7" t="s">
+        <v>276</v>
+      </c>
+      <c r="C53" s="7" t="s">
+        <v>280</v>
+      </c>
+      <c r="D53" s="7" t="s">
+        <v>281</v>
+      </c>
+      <c r="E53" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="C53" s="12" t="s">
+      <c r="F53" s="12" t="s">
         <v>198</v>
       </c>
-      <c r="D53" s="16" t="s">
+      <c r="G53" s="16" t="s">
         <v>199</v>
       </c>
-      <c r="E53" s="12" t="s">
+      <c r="H53" s="12" t="s">
         <v>154</v>
       </c>
-      <c r="F53" s="8" t="s">
+      <c r="I53" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="G53" s="11" t="s">
+      <c r="J53" s="11" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="54" spans="1:17" ht="15" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:20" ht="15" x14ac:dyDescent="0.2">
       <c r="A54" s="7" t="s">
         <v>200</v>
       </c>
-      <c r="B54" s="8" t="s">
+      <c r="B54" s="7" t="s">
+        <v>276</v>
+      </c>
+      <c r="C54" s="7" t="s">
+        <v>280</v>
+      </c>
+      <c r="D54" s="7" t="s">
+        <v>281</v>
+      </c>
+      <c r="E54" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="C54" s="12" t="s">
+      <c r="F54" s="12" t="s">
         <v>201</v>
       </c>
-      <c r="D54" s="16" t="s">
+      <c r="G54" s="16" t="s">
         <v>202</v>
       </c>
-      <c r="E54" s="8" t="s">
+      <c r="H54" s="8" t="s">
         <v>203</v>
       </c>
-      <c r="F54" s="8" t="s">
+      <c r="I54" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="G54" s="10" t="s">
+      <c r="J54" s="10" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="55" spans="1:17" ht="15" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:20" ht="15" x14ac:dyDescent="0.2">
       <c r="A55" s="7" t="s">
         <v>204</v>
       </c>
-      <c r="B55" s="8" t="s">
+      <c r="B55" s="7" t="s">
+        <v>276</v>
+      </c>
+      <c r="C55" s="7" t="s">
+        <v>280</v>
+      </c>
+      <c r="D55" s="7" t="s">
+        <v>281</v>
+      </c>
+      <c r="E55" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="C55" s="12" t="s">
+      <c r="F55" s="12" t="s">
         <v>205</v>
       </c>
-      <c r="D55" s="16" t="s">
+      <c r="G55" s="16" t="s">
         <v>206</v>
       </c>
-      <c r="E55" s="8" t="s">
+      <c r="H55" s="8" t="s">
         <v>207</v>
       </c>
-      <c r="F55" s="8" t="s">
+      <c r="I55" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="G55" s="10" t="s">
+      <c r="J55" s="10" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="56" spans="1:17" ht="15" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:20" ht="15" x14ac:dyDescent="0.2">
       <c r="A56" s="7" t="s">
         <v>208</v>
       </c>
-      <c r="B56" s="8" t="s">
+      <c r="B56" s="7" t="s">
+        <v>276</v>
+      </c>
+      <c r="C56" s="7" t="s">
+        <v>280</v>
+      </c>
+      <c r="D56" s="7" t="s">
+        <v>281</v>
+      </c>
+      <c r="E56" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="C56" s="14" t="s">
+      <c r="F56" s="14" t="s">
         <v>209</v>
       </c>
-      <c r="D56" s="16" t="s">
+      <c r="G56" s="16" t="s">
         <v>210</v>
       </c>
-      <c r="E56" s="14" t="s">
+      <c r="H56" s="14" t="s">
         <v>211</v>
       </c>
-      <c r="F56" s="8" t="s">
+      <c r="I56" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="G56" s="11" t="s">
+      <c r="J56" s="11" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="57" spans="1:17" customFormat="1" ht="15" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:20" customFormat="1" ht="15" x14ac:dyDescent="0.25">
       <c r="A57" s="7" t="s">
         <v>212</v>
       </c>
-      <c r="B57" s="17" t="s">
+      <c r="B57" s="7" t="s">
+        <v>276</v>
+      </c>
+      <c r="C57" s="7" t="s">
+        <v>280</v>
+      </c>
+      <c r="D57" s="7" t="s">
+        <v>281</v>
+      </c>
+      <c r="E57" s="7" t="s">
         <v>213</v>
       </c>
-      <c r="C57" s="12" t="s">
+      <c r="F57" s="12" t="s">
         <v>39</v>
       </c>
-      <c r="D57" s="13" t="s">
+      <c r="G57" s="13" t="s">
         <v>40</v>
       </c>
-      <c r="E57" s="8" t="s">
+      <c r="H57" s="8" t="s">
         <v>41</v>
       </c>
-      <c r="F57" s="8" t="s">
+      <c r="I57" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="G57" s="10" t="s">
+      <c r="J57" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="H57" s="1"/>
-      <c r="I57" s="1"/>
-      <c r="J57" s="1"/>
       <c r="K57" s="1"/>
       <c r="L57" s="1"/>
       <c r="M57" s="1"/>
@@ -3208,32 +3739,41 @@
       <c r="O57" s="1"/>
       <c r="P57" s="1"/>
       <c r="Q57" s="1"/>
-    </row>
-    <row r="58" spans="1:17" customFormat="1" ht="15" x14ac:dyDescent="0.25">
+      <c r="R57" s="1"/>
+      <c r="S57" s="1"/>
+      <c r="T57" s="1"/>
+    </row>
+    <row r="58" spans="1:20" customFormat="1" ht="15" x14ac:dyDescent="0.25">
       <c r="A58" s="7" t="s">
         <v>214</v>
       </c>
-      <c r="B58" s="17" t="s">
+      <c r="B58" s="7" t="s">
+        <v>276</v>
+      </c>
+      <c r="C58" s="7" t="s">
+        <v>280</v>
+      </c>
+      <c r="D58" s="7" t="s">
+        <v>281</v>
+      </c>
+      <c r="E58" s="7" t="s">
         <v>213</v>
       </c>
-      <c r="C58" s="14" t="s">
+      <c r="F58" s="14" t="s">
         <v>43</v>
       </c>
-      <c r="D58" s="13" t="s">
+      <c r="G58" s="13" t="s">
         <v>44</v>
       </c>
-      <c r="E58" s="8" t="s">
+      <c r="H58" s="8" t="s">
         <v>45</v>
       </c>
-      <c r="F58" s="8" t="s">
+      <c r="I58" s="8" t="s">
         <v>33</v>
       </c>
-      <c r="G58" s="10" t="s">
+      <c r="J58" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="H58" s="1"/>
-      <c r="I58" s="1"/>
-      <c r="J58" s="1"/>
       <c r="K58" s="1"/>
       <c r="L58" s="1"/>
       <c r="M58" s="1"/>
@@ -3241,32 +3781,41 @@
       <c r="O58" s="1"/>
       <c r="P58" s="1"/>
       <c r="Q58" s="1"/>
-    </row>
-    <row r="59" spans="1:17" customFormat="1" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="R58" s="1"/>
+      <c r="S58" s="1"/>
+      <c r="T58" s="1"/>
+    </row>
+    <row r="59" spans="1:20" customFormat="1" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A59" s="7" t="s">
         <v>215</v>
       </c>
-      <c r="B59" s="17" t="s">
+      <c r="B59" s="7" t="s">
+        <v>277</v>
+      </c>
+      <c r="C59" s="7" t="s">
+        <v>282</v>
+      </c>
+      <c r="D59" s="7" t="s">
+        <v>283</v>
+      </c>
+      <c r="E59" s="7" t="s">
         <v>213</v>
       </c>
-      <c r="C59" s="14" t="s">
+      <c r="F59" s="14" t="s">
         <v>216</v>
       </c>
-      <c r="D59" s="13" t="s">
+      <c r="G59" s="13" t="s">
         <v>217</v>
       </c>
-      <c r="E59" s="12" t="s">
+      <c r="H59" s="12" t="s">
         <v>218</v>
       </c>
-      <c r="F59" s="8" t="s">
+      <c r="I59" s="8" t="s">
         <v>219</v>
       </c>
-      <c r="G59" s="10" t="s">
+      <c r="J59" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="H59" s="1"/>
-      <c r="I59" s="1"/>
-      <c r="J59" s="1"/>
       <c r="K59" s="1"/>
       <c r="L59" s="1"/>
       <c r="M59" s="1"/>
@@ -3274,32 +3823,41 @@
       <c r="O59" s="1"/>
       <c r="P59" s="1"/>
       <c r="Q59" s="1"/>
-    </row>
-    <row r="60" spans="1:17" customFormat="1" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="R59" s="1"/>
+      <c r="S59" s="1"/>
+      <c r="T59" s="1"/>
+    </row>
+    <row r="60" spans="1:20" customFormat="1" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A60" s="7" t="s">
         <v>220</v>
       </c>
-      <c r="B60" s="17" t="s">
+      <c r="B60" s="7" t="s">
+        <v>277</v>
+      </c>
+      <c r="C60" s="7" t="s">
+        <v>282</v>
+      </c>
+      <c r="D60" s="7" t="s">
+        <v>283</v>
+      </c>
+      <c r="E60" s="7" t="s">
         <v>213</v>
       </c>
-      <c r="C60" s="14" t="s">
+      <c r="F60" s="14" t="s">
         <v>221</v>
       </c>
-      <c r="D60" s="13" t="s">
+      <c r="G60" s="13" t="s">
         <v>48</v>
       </c>
-      <c r="E60" s="12" t="s">
+      <c r="H60" s="12" t="s">
         <v>49</v>
       </c>
-      <c r="F60" s="8" t="s">
+      <c r="I60" s="8" t="s">
         <v>222</v>
       </c>
-      <c r="G60" s="11" t="s">
+      <c r="J60" s="11" t="s">
         <v>28</v>
       </c>
-      <c r="H60" s="1"/>
-      <c r="I60" s="1"/>
-      <c r="J60" s="1"/>
       <c r="K60" s="1"/>
       <c r="L60" s="1"/>
       <c r="M60" s="1"/>
@@ -3307,32 +3865,41 @@
       <c r="O60" s="1"/>
       <c r="P60" s="1"/>
       <c r="Q60" s="1"/>
-    </row>
-    <row r="61" spans="1:17" ht="15" x14ac:dyDescent="0.25">
+      <c r="R60" s="1"/>
+      <c r="S60" s="1"/>
+      <c r="T60" s="1"/>
+    </row>
+    <row r="61" spans="1:20" ht="15" x14ac:dyDescent="0.25">
       <c r="A61" s="7" t="s">
         <v>223</v>
       </c>
-      <c r="B61" s="17" t="s">
+      <c r="B61" s="7" t="s">
+        <v>276</v>
+      </c>
+      <c r="C61" s="7" t="s">
+        <v>280</v>
+      </c>
+      <c r="D61" s="7" t="s">
+        <v>281</v>
+      </c>
+      <c r="E61" s="7" t="s">
         <v>213</v>
       </c>
-      <c r="C61" s="8" t="s">
+      <c r="F61" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="D61" s="9" t="s">
+      <c r="G61" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="E61" s="8" t="s">
+      <c r="H61" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="F61" s="8" t="s">
+      <c r="I61" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="G61" s="10" t="s">
+      <c r="J61" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="H61"/>
-      <c r="I61"/>
-      <c r="J61"/>
       <c r="K61"/>
       <c r="L61"/>
       <c r="M61"/>
@@ -3340,32 +3907,41 @@
       <c r="O61"/>
       <c r="P61"/>
       <c r="Q61"/>
-    </row>
-    <row r="62" spans="1:17" ht="15" x14ac:dyDescent="0.25">
+      <c r="R61"/>
+      <c r="S61"/>
+      <c r="T61"/>
+    </row>
+    <row r="62" spans="1:20" ht="15" x14ac:dyDescent="0.25">
       <c r="A62" s="7" t="s">
         <v>224</v>
       </c>
-      <c r="B62" s="17" t="s">
+      <c r="B62" s="7" t="s">
+        <v>276</v>
+      </c>
+      <c r="C62" s="7" t="s">
+        <v>280</v>
+      </c>
+      <c r="D62" s="7" t="s">
+        <v>281</v>
+      </c>
+      <c r="E62" s="7" t="s">
         <v>213</v>
       </c>
-      <c r="C62" s="8" t="s">
+      <c r="F62" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="D62" s="9" t="s">
+      <c r="G62" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="E62" s="8" t="s">
+      <c r="H62" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="F62" s="8" t="s">
+      <c r="I62" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="G62" s="10" t="s">
+      <c r="J62" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="H62"/>
-      <c r="I62"/>
-      <c r="J62"/>
       <c r="K62"/>
       <c r="L62"/>
       <c r="M62"/>
@@ -3373,251 +3949,341 @@
       <c r="O62"/>
       <c r="P62"/>
       <c r="Q62"/>
-    </row>
-    <row r="63" spans="1:17" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="R62"/>
+      <c r="S62"/>
+      <c r="T62"/>
+    </row>
+    <row r="63" spans="1:20" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A63" s="7" t="s">
         <v>225</v>
       </c>
-      <c r="B63" s="17" t="s">
+      <c r="B63" s="7" t="s">
+        <v>276</v>
+      </c>
+      <c r="C63" s="7" t="s">
+        <v>280</v>
+      </c>
+      <c r="D63" s="7" t="s">
+        <v>281</v>
+      </c>
+      <c r="E63" s="7" t="s">
         <v>213</v>
       </c>
-      <c r="C63" s="8" t="s">
+      <c r="F63" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="D63" s="9" t="s">
+      <c r="G63" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="E63" s="8" t="s">
+      <c r="H63" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="F63" s="8" t="s">
+      <c r="I63" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="G63" s="10" t="s">
+      <c r="J63" s="10" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="64" spans="1:17" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:20" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A64" s="7" t="s">
         <v>226</v>
       </c>
-      <c r="B64" s="17" t="s">
+      <c r="B64" s="7" t="s">
+        <v>276</v>
+      </c>
+      <c r="C64" s="7" t="s">
+        <v>280</v>
+      </c>
+      <c r="D64" s="7" t="s">
+        <v>281</v>
+      </c>
+      <c r="E64" s="7" t="s">
         <v>213</v>
       </c>
-      <c r="C64" s="8" t="s">
+      <c r="F64" s="8" t="s">
         <v>24</v>
       </c>
-      <c r="D64" s="9" t="s">
+      <c r="G64" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="E64" s="8" t="s">
+      <c r="H64" s="8" t="s">
         <v>26</v>
       </c>
-      <c r="F64" s="8" t="s">
+      <c r="I64" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="G64" s="11" t="s">
+      <c r="J64" s="11" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="65" spans="1:7" ht="14.25" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:10" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A65" s="7" t="s">
         <v>227</v>
       </c>
-      <c r="B65" s="17" t="s">
+      <c r="B65" s="7" t="s">
+        <v>276</v>
+      </c>
+      <c r="C65" s="7" t="s">
+        <v>280</v>
+      </c>
+      <c r="D65" s="7" t="s">
+        <v>281</v>
+      </c>
+      <c r="E65" s="7" t="s">
         <v>213</v>
       </c>
-      <c r="C65" s="8" t="s">
+      <c r="F65" s="8" t="s">
         <v>30</v>
       </c>
-      <c r="D65" s="9" t="s">
+      <c r="G65" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="E65" s="8" t="s">
+      <c r="H65" s="8" t="s">
         <v>32</v>
       </c>
-      <c r="F65" s="8" t="s">
+      <c r="I65" s="8" t="s">
         <v>33</v>
       </c>
-      <c r="G65" s="10" t="s">
+      <c r="J65" s="10" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="66" spans="1:7" ht="14.25" x14ac:dyDescent="0.2">
+    <row r="66" spans="1:10" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A66" s="7" t="s">
         <v>228</v>
       </c>
-      <c r="B66" s="17" t="s">
+      <c r="B66" s="7" t="s">
+        <v>276</v>
+      </c>
+      <c r="C66" s="7" t="s">
+        <v>280</v>
+      </c>
+      <c r="D66" s="7" t="s">
+        <v>281</v>
+      </c>
+      <c r="E66" s="7" t="s">
         <v>213</v>
       </c>
-      <c r="C66" s="8" t="s">
+      <c r="F66" s="8" t="s">
         <v>35</v>
       </c>
-      <c r="D66" s="9" t="s">
+      <c r="G66" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="E66" s="8" t="s">
+      <c r="H66" s="8" t="s">
         <v>37</v>
       </c>
-      <c r="F66" s="8" t="s">
+      <c r="I66" s="8" t="s">
         <v>33</v>
       </c>
-      <c r="G66" s="10" t="s">
+      <c r="J66" s="10" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="67" spans="1:7" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:10" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A67" s="7" t="s">
         <v>229</v>
       </c>
-      <c r="B67" s="17" t="s">
+      <c r="B67" s="7" t="s">
+        <v>277</v>
+      </c>
+      <c r="C67" s="7" t="s">
+        <v>282</v>
+      </c>
+      <c r="D67" s="7" t="s">
+        <v>283</v>
+      </c>
+      <c r="E67" s="7" t="s">
         <v>213</v>
       </c>
-      <c r="C67" s="12" t="s">
+      <c r="F67" s="12" t="s">
         <v>230</v>
       </c>
-      <c r="D67" s="9" t="s">
+      <c r="G67" s="9" t="s">
         <v>231</v>
       </c>
-      <c r="E67" s="8" t="s">
+      <c r="H67" s="8" t="s">
         <v>232</v>
       </c>
-      <c r="F67" s="8" t="s">
+      <c r="I67" s="8" t="s">
         <v>219</v>
       </c>
-      <c r="G67" s="10" t="s">
+      <c r="J67" s="10" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="68" spans="1:7" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="68" spans="1:10" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A68" s="7" t="s">
         <v>233</v>
       </c>
-      <c r="B68" s="17" t="s">
+      <c r="B68" s="7" t="s">
+        <v>277</v>
+      </c>
+      <c r="C68" s="7" t="s">
+        <v>282</v>
+      </c>
+      <c r="D68" s="7" t="s">
+        <v>283</v>
+      </c>
+      <c r="E68" s="7" t="s">
         <v>213</v>
       </c>
-      <c r="C68" s="8" t="s">
+      <c r="F68" s="8" t="s">
         <v>234</v>
       </c>
-      <c r="D68" s="9" t="s">
+      <c r="G68" s="9" t="s">
         <v>235</v>
       </c>
-      <c r="E68" s="8" t="s">
+      <c r="H68" s="8" t="s">
         <v>236</v>
       </c>
-      <c r="F68" s="8" t="s">
+      <c r="I68" s="8" t="s">
         <v>237</v>
       </c>
-      <c r="G68" s="11" t="s">
+      <c r="J68" s="11" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="69" spans="1:7" ht="14.25" x14ac:dyDescent="0.2">
+    <row r="69" spans="1:10" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A69" s="17"/>
       <c r="B69" s="17"/>
-      <c r="C69" s="12"/>
-      <c r="D69" s="13"/>
-      <c r="E69" s="12"/>
-      <c r="F69" s="17"/>
-      <c r="G69" s="17"/>
-    </row>
-    <row r="70" spans="1:7" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="C69" s="17"/>
+      <c r="D69" s="17"/>
+      <c r="E69" s="17"/>
+      <c r="F69" s="12"/>
+      <c r="G69" s="13"/>
+      <c r="H69" s="12"/>
+      <c r="I69" s="17"/>
+      <c r="J69" s="17"/>
+    </row>
+    <row r="70" spans="1:10" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A70" s="18"/>
       <c r="B70" s="18"/>
-      <c r="C70" s="19"/>
-      <c r="D70" s="20"/>
-      <c r="E70" s="19"/>
-      <c r="F70" s="18"/>
-      <c r="G70" s="18"/>
-    </row>
-    <row r="71" spans="1:7" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="C70" s="18"/>
+      <c r="D70" s="18"/>
+      <c r="E70" s="18"/>
+      <c r="F70" s="19"/>
+      <c r="G70" s="20"/>
+      <c r="H70" s="19"/>
+      <c r="I70" s="18"/>
+      <c r="J70" s="18"/>
+    </row>
+    <row r="71" spans="1:10" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A71" s="18"/>
       <c r="B71" s="18"/>
-      <c r="C71" s="19"/>
-      <c r="D71" s="20"/>
-      <c r="E71" s="19"/>
-      <c r="F71" s="18"/>
-      <c r="G71" s="18"/>
-    </row>
-    <row r="72" spans="1:7" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="C71" s="18"/>
+      <c r="D71" s="18"/>
+      <c r="E71" s="18"/>
+      <c r="F71" s="19"/>
+      <c r="G71" s="20"/>
+      <c r="H71" s="19"/>
+      <c r="I71" s="18"/>
+      <c r="J71" s="18"/>
+    </row>
+    <row r="72" spans="1:10" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A72" s="18"/>
       <c r="B72" s="18"/>
-      <c r="C72" s="19"/>
-      <c r="D72" s="20"/>
-      <c r="E72" s="19"/>
-      <c r="F72" s="18"/>
-      <c r="G72" s="18"/>
-    </row>
-    <row r="73" spans="1:7" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="C72" s="18"/>
+      <c r="D72" s="18"/>
+      <c r="E72" s="18"/>
+      <c r="F72" s="19"/>
+      <c r="G72" s="20"/>
+      <c r="H72" s="19"/>
+      <c r="I72" s="18"/>
+      <c r="J72" s="18"/>
+    </row>
+    <row r="73" spans="1:10" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A73" s="18"/>
       <c r="B73" s="18"/>
-      <c r="C73" s="19"/>
-      <c r="D73" s="20"/>
-      <c r="E73" s="19"/>
-      <c r="F73" s="18"/>
-      <c r="G73" s="18"/>
-    </row>
-    <row r="74" spans="1:7" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="C73" s="18"/>
+      <c r="D73" s="18"/>
+      <c r="E73" s="18"/>
+      <c r="F73" s="19"/>
+      <c r="G73" s="20"/>
+      <c r="H73" s="19"/>
+      <c r="I73" s="18"/>
+      <c r="J73" s="18"/>
+    </row>
+    <row r="74" spans="1:10" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A74" s="18"/>
       <c r="B74" s="18"/>
-      <c r="C74" s="19"/>
-      <c r="D74" s="20"/>
-      <c r="E74" s="19"/>
-      <c r="F74" s="18"/>
-      <c r="G74" s="18"/>
-    </row>
-    <row r="75" spans="1:7" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="C74" s="18"/>
+      <c r="D74" s="18"/>
+      <c r="E74" s="18"/>
+      <c r="F74" s="19"/>
+      <c r="G74" s="20"/>
+      <c r="H74" s="19"/>
+      <c r="I74" s="18"/>
+      <c r="J74" s="18"/>
+    </row>
+    <row r="75" spans="1:10" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A75" s="18"/>
       <c r="B75" s="18"/>
-      <c r="C75" s="19"/>
-      <c r="D75" s="20"/>
-      <c r="E75" s="19"/>
-      <c r="F75" s="18"/>
-      <c r="G75" s="18"/>
-    </row>
-    <row r="76" spans="1:7" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="C75" s="18"/>
+      <c r="D75" s="18"/>
+      <c r="E75" s="18"/>
+      <c r="F75" s="19"/>
+      <c r="G75" s="20"/>
+      <c r="H75" s="19"/>
+      <c r="I75" s="18"/>
+      <c r="J75" s="18"/>
+    </row>
+    <row r="76" spans="1:10" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A76" s="18"/>
       <c r="B76" s="18"/>
-      <c r="C76" s="19"/>
-      <c r="D76" s="20"/>
-      <c r="E76" s="19"/>
-      <c r="F76" s="18"/>
-      <c r="G76" s="18"/>
-    </row>
-    <row r="77" spans="1:7" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="C76" s="18"/>
+      <c r="D76" s="18"/>
+      <c r="E76" s="18"/>
+      <c r="F76" s="19"/>
+      <c r="G76" s="20"/>
+      <c r="H76" s="19"/>
+      <c r="I76" s="18"/>
+      <c r="J76" s="18"/>
+    </row>
+    <row r="77" spans="1:10" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A77" s="18"/>
       <c r="B77" s="18"/>
-      <c r="C77" s="19"/>
-      <c r="D77" s="20"/>
-      <c r="E77" s="19"/>
-      <c r="F77" s="18"/>
-      <c r="G77" s="18"/>
-    </row>
-    <row r="78" spans="1:7" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="C77" s="18"/>
+      <c r="D77" s="18"/>
+      <c r="E77" s="18"/>
+      <c r="F77" s="19"/>
+      <c r="G77" s="20"/>
+      <c r="H77" s="19"/>
+      <c r="I77" s="18"/>
+      <c r="J77" s="18"/>
+    </row>
+    <row r="78" spans="1:10" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A78" s="18"/>
       <c r="B78" s="18"/>
-      <c r="C78" s="19"/>
-      <c r="D78" s="20"/>
-      <c r="E78" s="19"/>
-      <c r="F78" s="18"/>
-      <c r="G78" s="18"/>
-    </row>
-    <row r="79" spans="1:7" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="C78" s="18"/>
+      <c r="D78" s="18"/>
+      <c r="E78" s="18"/>
+      <c r="F78" s="19"/>
+      <c r="G78" s="20"/>
+      <c r="H78" s="19"/>
+      <c r="I78" s="18"/>
+      <c r="J78" s="18"/>
+    </row>
+    <row r="79" spans="1:10" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A79" s="18"/>
       <c r="B79" s="18"/>
-      <c r="C79" s="19"/>
-      <c r="D79" s="20"/>
-      <c r="E79" s="19"/>
-      <c r="F79" s="18"/>
-      <c r="G79" s="18"/>
+      <c r="C79" s="18"/>
+      <c r="D79" s="18"/>
+      <c r="E79" s="18"/>
+      <c r="F79" s="19"/>
+      <c r="G79" s="20"/>
+      <c r="H79" s="19"/>
+      <c r="I79" s="18"/>
+      <c r="J79" s="18"/>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="A2:J2"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation operator="equal" sqref="D1:D35 D57:D1068" xr:uid="{00000000-0002-0000-0000-000000000000}">
+    <dataValidation operator="equal" sqref="G1:G35 G57:G1068" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>0</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -3633,10 +4299,10 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:J3"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.5703125" defaultRowHeight="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:7" ht="19.350000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" ht="19.350000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="21" t="s">
         <v>0</v>
       </c>
@@ -3646,8 +4312,11 @@
       <c r="E1" s="21"/>
       <c r="F1" s="21"/>
       <c r="G1" s="21"/>
-    </row>
-    <row r="2" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="H1" s="21"/>
+      <c r="I1" s="21"/>
+      <c r="J1" s="21"/>
+    </row>
+    <row r="2" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="22" t="s">
         <v>239</v>
       </c>
@@ -3658,36 +4327,45 @@
       <c r="F2" s="22"/>
       <c r="G2" s="22"/>
     </row>
-    <row r="3" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:10" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
         <v>2</v>
       </c>
       <c r="B3" s="5" t="s">
+        <v>275</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>278</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>279</v>
+      </c>
+      <c r="E3" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="C3" s="5" t="s">
+      <c r="F3" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="D3" s="6" t="s">
+      <c r="G3" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="E3" s="5" t="s">
+      <c r="H3" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="F3" s="5" t="s">
+      <c r="I3" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="G3" s="5" t="s">
+      <c r="J3" s="5" t="s">
         <v>8</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A1:G1"/>
     <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A1:J1"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation operator="equal" sqref="D1:D3" xr:uid="{00000000-0002-0000-0900-000000000000}">
+    <dataValidation operator="equal" sqref="G3 D2 G1" xr:uid="{00000000-0002-0000-0900-000000000000}">
       <formula1>0</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -3703,19 +4381,19 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:G10"/>
+  <dimension ref="A1:J10"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.5703125" defaultRowHeight="53.25" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="11.5703125" style="16"/>
-    <col min="2" max="2" width="21.7109375" style="16" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="44" style="16" customWidth="1"/>
-    <col min="4" max="4" width="48.28515625" style="16" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="38.42578125" style="16" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="13.28515625" style="16" bestFit="1" customWidth="1"/>
-    <col min="7" max="16384" width="11.5703125" style="16"/>
+    <col min="1" max="4" width="11.5703125" style="16"/>
+    <col min="5" max="5" width="21.7109375" style="16" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="44" style="16" customWidth="1"/>
+    <col min="7" max="7" width="48.28515625" style="16" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="38.42578125" style="16" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="13.28515625" style="16" bestFit="1" customWidth="1"/>
+    <col min="10" max="16384" width="11.5703125" style="16"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="53.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" ht="53.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="21" t="s">
         <v>0</v>
       </c>
@@ -3725,8 +4403,11 @@
       <c r="E1" s="21"/>
       <c r="F1" s="21"/>
       <c r="G1" s="21"/>
-    </row>
-    <row r="2" spans="1:7" ht="53.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="H1" s="21"/>
+      <c r="I1" s="21"/>
+      <c r="J1" s="21"/>
+    </row>
+    <row r="2" spans="1:10" ht="53.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="22" t="s">
         <v>240</v>
       </c>
@@ -3736,205 +4417,280 @@
       <c r="E2" s="22"/>
       <c r="F2" s="22"/>
       <c r="G2" s="22"/>
-    </row>
-    <row r="3" spans="1:7" ht="53.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="H2" s="22"/>
+      <c r="I2" s="22"/>
+      <c r="J2" s="22"/>
+    </row>
+    <row r="3" spans="1:10" ht="53.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
         <v>2</v>
       </c>
       <c r="B3" s="5" t="s">
+        <v>275</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>278</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>279</v>
+      </c>
+      <c r="E3" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="C3" s="5" t="s">
+      <c r="F3" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="D3" s="6" t="s">
+      <c r="G3" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="E3" s="5" t="s">
+      <c r="H3" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="F3" s="5" t="s">
+      <c r="I3" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="G3" s="5" t="s">
+      <c r="J3" s="5" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:7" ht="53.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:10" ht="53.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="7" t="s">
+        <v>246</v>
+      </c>
+      <c r="B4" s="7" t="s">
+        <v>276</v>
+      </c>
+      <c r="C4" s="7" t="s">
+        <v>280</v>
+      </c>
+      <c r="D4" s="7" t="s">
+        <v>281</v>
+      </c>
+      <c r="E4" s="12" t="s">
         <v>247</v>
       </c>
-      <c r="B4" s="12" t="s">
+      <c r="F4" s="16" t="s">
         <v>248</v>
       </c>
-      <c r="C4" s="16" t="s">
+      <c r="G4" s="16" t="s">
+        <v>269</v>
+      </c>
+      <c r="H4" s="16" t="s">
+        <v>274</v>
+      </c>
+      <c r="I4" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="J4" s="10" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" ht="53.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="7" t="s">
+        <v>253</v>
+      </c>
+      <c r="B5" s="7" t="s">
+        <v>277</v>
+      </c>
+      <c r="C5" s="7" t="s">
+        <v>282</v>
+      </c>
+      <c r="D5" s="7" t="s">
+        <v>283</v>
+      </c>
+      <c r="E5" s="12" t="s">
+        <v>247</v>
+      </c>
+      <c r="F5" s="16" t="s">
         <v>249</v>
       </c>
-      <c r="D4" s="16" t="s">
+      <c r="G5" s="16" t="s">
+        <v>259</v>
+      </c>
+      <c r="H5" s="16" t="s">
+        <v>274</v>
+      </c>
+      <c r="I5" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="J5" s="10" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" ht="53.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="7" t="s">
+        <v>254</v>
+      </c>
+      <c r="B6" s="7" t="s">
+        <v>277</v>
+      </c>
+      <c r="C6" s="7" t="s">
+        <v>282</v>
+      </c>
+      <c r="D6" s="7" t="s">
+        <v>283</v>
+      </c>
+      <c r="E6" s="12" t="s">
+        <v>247</v>
+      </c>
+      <c r="F6" s="16" t="s">
+        <v>250</v>
+      </c>
+      <c r="G6" s="16" t="s">
+        <v>260</v>
+      </c>
+      <c r="H6" s="16" t="s">
+        <v>265</v>
+      </c>
+      <c r="I6" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="J6" s="11" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" ht="53.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="7" t="s">
+        <v>255</v>
+      </c>
+      <c r="B7" s="7" t="s">
+        <v>277</v>
+      </c>
+      <c r="C7" s="7" t="s">
+        <v>282</v>
+      </c>
+      <c r="D7" s="7" t="s">
+        <v>283</v>
+      </c>
+      <c r="E7" s="12" t="s">
+        <v>247</v>
+      </c>
+      <c r="F7" s="16" t="s">
+        <v>251</v>
+      </c>
+      <c r="G7" s="16" t="s">
+        <v>261</v>
+      </c>
+      <c r="H7" s="16" t="s">
+        <v>266</v>
+      </c>
+      <c r="I7" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="J7" s="11" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" ht="53.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="7" t="s">
+        <v>256</v>
+      </c>
+      <c r="B8" s="7" t="s">
+        <v>277</v>
+      </c>
+      <c r="C8" s="7" t="s">
+        <v>282</v>
+      </c>
+      <c r="D8" s="7" t="s">
+        <v>283</v>
+      </c>
+      <c r="E8" s="12" t="s">
+        <v>247</v>
+      </c>
+      <c r="F8" s="16" t="s">
+        <v>268</v>
+      </c>
+      <c r="G8" s="16" t="s">
+        <v>262</v>
+      </c>
+      <c r="H8" s="16" t="s">
+        <v>263</v>
+      </c>
+      <c r="I8" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="J8" s="11" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" ht="53.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="7" t="s">
+        <v>257</v>
+      </c>
+      <c r="B9" s="7" t="s">
+        <v>277</v>
+      </c>
+      <c r="C9" s="7" t="s">
+        <v>282</v>
+      </c>
+      <c r="D9" s="7" t="s">
+        <v>283</v>
+      </c>
+      <c r="E9" s="12" t="s">
+        <v>247</v>
+      </c>
+      <c r="F9" s="16" t="s">
+        <v>252</v>
+      </c>
+      <c r="G9" s="16" t="s">
+        <v>264</v>
+      </c>
+      <c r="H9" s="16" t="s">
+        <v>267</v>
+      </c>
+      <c r="I9" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="J9" s="11" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" ht="53.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="7" t="s">
+        <v>258</v>
+      </c>
+      <c r="B10" s="7" t="s">
+        <v>277</v>
+      </c>
+      <c r="C10" s="7" t="s">
+        <v>285</v>
+      </c>
+      <c r="D10" s="7" t="s">
+        <v>286</v>
+      </c>
+      <c r="E10" s="12" t="s">
+        <v>247</v>
+      </c>
+      <c r="F10" s="16" t="s">
+        <v>272</v>
+      </c>
+      <c r="G10" s="16" t="s">
+        <v>271</v>
+      </c>
+      <c r="H10" s="16" t="s">
+        <v>273</v>
+      </c>
+      <c r="I10" s="8" t="s">
         <v>270</v>
       </c>
-      <c r="E4" s="16" t="s">
-        <v>275</v>
-      </c>
-      <c r="F4" s="8" t="s">
-        <v>14</v>
-      </c>
-      <c r="G4" s="10" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" ht="53.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="7" t="s">
-        <v>254</v>
-      </c>
-      <c r="B5" s="12" t="s">
-        <v>248</v>
-      </c>
-      <c r="C5" s="16" t="s">
-        <v>250</v>
-      </c>
-      <c r="D5" s="16" t="s">
-        <v>260</v>
-      </c>
-      <c r="E5" s="16" t="s">
-        <v>275</v>
-      </c>
-      <c r="F5" s="8" t="s">
-        <v>14</v>
-      </c>
-      <c r="G5" s="10" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" ht="53.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="7" t="s">
-        <v>255</v>
-      </c>
-      <c r="B6" s="12" t="s">
-        <v>248</v>
-      </c>
-      <c r="C6" s="16" t="s">
-        <v>251</v>
-      </c>
-      <c r="D6" s="16" t="s">
-        <v>261</v>
-      </c>
-      <c r="E6" s="16" t="s">
-        <v>266</v>
-      </c>
-      <c r="F6" s="8" t="s">
-        <v>27</v>
-      </c>
-      <c r="G6" s="11" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" ht="53.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="7" t="s">
-        <v>256</v>
-      </c>
-      <c r="B7" s="12" t="s">
-        <v>248</v>
-      </c>
-      <c r="C7" s="16" t="s">
-        <v>252</v>
-      </c>
-      <c r="D7" s="16" t="s">
-        <v>262</v>
-      </c>
-      <c r="E7" s="16" t="s">
-        <v>267</v>
-      </c>
-      <c r="F7" s="8" t="s">
-        <v>27</v>
-      </c>
-      <c r="G7" s="11" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" ht="53.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="7" t="s">
-        <v>257</v>
-      </c>
-      <c r="B8" s="12" t="s">
-        <v>248</v>
-      </c>
-      <c r="C8" s="16" t="s">
-        <v>269</v>
-      </c>
-      <c r="D8" s="16" t="s">
-        <v>263</v>
-      </c>
-      <c r="E8" s="16" t="s">
-        <v>264</v>
-      </c>
-      <c r="F8" s="8" t="s">
-        <v>27</v>
-      </c>
-      <c r="G8" s="11" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" ht="53.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="7" t="s">
-        <v>258</v>
-      </c>
-      <c r="B9" s="12" t="s">
-        <v>248</v>
-      </c>
-      <c r="C9" s="16" t="s">
-        <v>253</v>
-      </c>
-      <c r="D9" s="16" t="s">
-        <v>265</v>
-      </c>
-      <c r="E9" s="16" t="s">
-        <v>268</v>
-      </c>
-      <c r="F9" s="8" t="s">
-        <v>27</v>
-      </c>
-      <c r="G9" s="11" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" ht="53.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="7" t="s">
-        <v>259</v>
-      </c>
-      <c r="B10" s="12" t="s">
-        <v>248</v>
-      </c>
-      <c r="C10" s="16" t="s">
-        <v>273</v>
-      </c>
-      <c r="D10" s="16" t="s">
-        <v>272</v>
-      </c>
-      <c r="E10" s="16" t="s">
-        <v>274</v>
-      </c>
-      <c r="F10" s="8" t="s">
-        <v>271</v>
-      </c>
-      <c r="G10" s="10" t="s">
+      <c r="J10" s="10" t="s">
         <v>15</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="A2:J2"/>
   </mergeCells>
   <phoneticPr fontId="9" type="noConversion"/>
   <dataValidations count="1">
-    <dataValidation operator="equal" sqref="D1:D3" xr:uid="{00000000-0002-0000-0100-000000000000}">
+    <dataValidation operator="equal" sqref="G1:G3" xr:uid="{00000000-0002-0000-0100-000000000000}">
       <formula1>0</formula1>
       <formula2>0</formula2>
     </dataValidation>
   </dataValidations>
   <hyperlinks>
-    <hyperlink ref="D10" r:id="rId1" display="search?q=@#&lt;?&amp;+!&amp;limit=10" xr:uid="{B2B6A10A-6BD0-48FE-82FC-898BF2336482}"/>
+    <hyperlink ref="G10" r:id="rId1" display="search?q=@#&lt;?&amp;+!&amp;limit=10" xr:uid="{B2B6A10A-6BD0-48FE-82FC-898BF2336482}"/>
   </hyperlinks>
   <pageMargins left="0.78749999999999998" right="0.78749999999999998" top="1.05277777777778" bottom="1.05277777777778" header="0.78749999999999998" footer="0.78749999999999998"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
@@ -3947,10 +4703,10 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:J3"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.5703125" defaultRowHeight="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:7" ht="19.350000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" ht="19.350000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="21" t="s">
         <v>0</v>
       </c>
@@ -3960,8 +4716,11 @@
       <c r="E1" s="21"/>
       <c r="F1" s="21"/>
       <c r="G1" s="21"/>
-    </row>
-    <row r="2" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="H1" s="21"/>
+      <c r="I1" s="21"/>
+      <c r="J1" s="21"/>
+    </row>
+    <row r="2" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="22" t="s">
         <v>241</v>
       </c>
@@ -3971,37 +4730,49 @@
       <c r="E2" s="22"/>
       <c r="F2" s="22"/>
       <c r="G2" s="22"/>
-    </row>
-    <row r="3" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="H2" s="22"/>
+      <c r="I2" s="22"/>
+      <c r="J2" s="22"/>
+    </row>
+    <row r="3" spans="1:10" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
         <v>2</v>
       </c>
       <c r="B3" s="5" t="s">
+        <v>275</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>278</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>279</v>
+      </c>
+      <c r="E3" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="C3" s="5" t="s">
+      <c r="F3" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="D3" s="6" t="s">
+      <c r="G3" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="E3" s="5" t="s">
+      <c r="H3" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="F3" s="5" t="s">
+      <c r="I3" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="G3" s="5" t="s">
+      <c r="J3" s="5" t="s">
         <v>8</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="A2:J2"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation operator="equal" sqref="D1:D3" xr:uid="{00000000-0002-0000-0200-000000000000}">
+    <dataValidation operator="equal" sqref="G1:G3" xr:uid="{00000000-0002-0000-0200-000000000000}">
       <formula1>0</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -4017,10 +4788,10 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:J3"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.5703125" defaultRowHeight="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:7" ht="19.350000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" ht="19.350000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="21" t="s">
         <v>0</v>
       </c>
@@ -4030,10 +4801,13 @@
       <c r="E1" s="21"/>
       <c r="F1" s="21"/>
       <c r="G1" s="21"/>
-    </row>
-    <row r="2" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="H1" s="21"/>
+      <c r="I1" s="21"/>
+      <c r="J1" s="21"/>
+    </row>
+    <row r="2" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="22" t="s">
-        <v>246</v>
+        <v>284</v>
       </c>
       <c r="B2" s="22"/>
       <c r="C2" s="22"/>
@@ -4042,36 +4816,45 @@
       <c r="F2" s="22"/>
       <c r="G2" s="22"/>
     </row>
-    <row r="3" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:10" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
         <v>2</v>
       </c>
       <c r="B3" s="5" t="s">
+        <v>275</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>278</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>279</v>
+      </c>
+      <c r="E3" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="C3" s="5" t="s">
+      <c r="F3" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="D3" s="6" t="s">
+      <c r="G3" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="E3" s="5" t="s">
+      <c r="H3" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="F3" s="5" t="s">
+      <c r="I3" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="G3" s="5" t="s">
+      <c r="J3" s="5" t="s">
         <v>8</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A1:G1"/>
     <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A1:J1"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation operator="equal" sqref="D1:D3" xr:uid="{00000000-0002-0000-0300-000000000000}">
+    <dataValidation operator="equal" sqref="G3 D2 G1" xr:uid="{00000000-0002-0000-0300-000000000000}">
       <formula1>0</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -4087,10 +4870,10 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:J3"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.5703125" defaultRowHeight="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:7" ht="19.350000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" ht="19.350000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="21" t="s">
         <v>0</v>
       </c>
@@ -4100,8 +4883,11 @@
       <c r="E1" s="21"/>
       <c r="F1" s="21"/>
       <c r="G1" s="21"/>
-    </row>
-    <row r="2" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="H1" s="21"/>
+      <c r="I1" s="21"/>
+      <c r="J1" s="21"/>
+    </row>
+    <row r="2" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="22" t="s">
         <v>245</v>
       </c>
@@ -4112,36 +4898,45 @@
       <c r="F2" s="22"/>
       <c r="G2" s="22"/>
     </row>
-    <row r="3" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:10" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
         <v>2</v>
       </c>
       <c r="B3" s="5" t="s">
+        <v>275</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>278</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>279</v>
+      </c>
+      <c r="E3" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="C3" s="5" t="s">
+      <c r="F3" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="D3" s="6" t="s">
+      <c r="G3" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="E3" s="5" t="s">
+      <c r="H3" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="F3" s="5" t="s">
+      <c r="I3" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="G3" s="5" t="s">
+      <c r="J3" s="5" t="s">
         <v>8</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A1:G1"/>
     <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A1:J1"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation operator="equal" sqref="D1:D3" xr:uid="{00000000-0002-0000-0400-000000000000}">
+    <dataValidation operator="equal" sqref="G3 D2 G1" xr:uid="{00000000-0002-0000-0400-000000000000}">
       <formula1>0</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -4157,10 +4952,10 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:J3"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.5703125" defaultRowHeight="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:7" ht="19.350000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" ht="19.350000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="21" t="s">
         <v>0</v>
       </c>
@@ -4170,8 +4965,11 @@
       <c r="E1" s="21"/>
       <c r="F1" s="21"/>
       <c r="G1" s="21"/>
-    </row>
-    <row r="2" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="H1" s="21"/>
+      <c r="I1" s="21"/>
+      <c r="J1" s="21"/>
+    </row>
+    <row r="2" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="22" t="s">
         <v>244</v>
       </c>
@@ -4182,36 +4980,45 @@
       <c r="F2" s="22"/>
       <c r="G2" s="22"/>
     </row>
-    <row r="3" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:10" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
         <v>2</v>
       </c>
       <c r="B3" s="5" t="s">
+        <v>275</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>278</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>279</v>
+      </c>
+      <c r="E3" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="C3" s="5" t="s">
+      <c r="F3" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="D3" s="6" t="s">
+      <c r="G3" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="E3" s="5" t="s">
+      <c r="H3" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="F3" s="5" t="s">
+      <c r="I3" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="G3" s="5" t="s">
+      <c r="J3" s="5" t="s">
         <v>8</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A1:G1"/>
     <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A1:J1"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation operator="equal" sqref="D1:D3" xr:uid="{00000000-0002-0000-0500-000000000000}">
+    <dataValidation operator="equal" sqref="G3 D2 G1" xr:uid="{00000000-0002-0000-0500-000000000000}">
       <formula1>0</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -4227,10 +5034,10 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:J3"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.5703125" defaultRowHeight="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:7" ht="19.350000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" ht="19.350000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="21" t="s">
         <v>0</v>
       </c>
@@ -4240,8 +5047,11 @@
       <c r="E1" s="21"/>
       <c r="F1" s="21"/>
       <c r="G1" s="21"/>
-    </row>
-    <row r="2" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="H1" s="21"/>
+      <c r="I1" s="21"/>
+      <c r="J1" s="21"/>
+    </row>
+    <row r="2" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="22" t="s">
         <v>243</v>
       </c>
@@ -4252,36 +5062,45 @@
       <c r="F2" s="22"/>
       <c r="G2" s="22"/>
     </row>
-    <row r="3" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:10" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
         <v>2</v>
       </c>
       <c r="B3" s="5" t="s">
+        <v>275</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>278</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>279</v>
+      </c>
+      <c r="E3" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="C3" s="5" t="s">
+      <c r="F3" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="D3" s="6" t="s">
+      <c r="G3" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="E3" s="5" t="s">
+      <c r="H3" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="F3" s="5" t="s">
+      <c r="I3" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="G3" s="5" t="s">
+      <c r="J3" s="5" t="s">
         <v>8</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A1:G1"/>
     <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A1:J1"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation operator="equal" sqref="D1:D3" xr:uid="{00000000-0002-0000-0600-000000000000}">
+    <dataValidation operator="equal" sqref="G3 D2 G1" xr:uid="{00000000-0002-0000-0600-000000000000}">
       <formula1>0</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -4297,10 +5116,10 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:J3"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.5703125" defaultRowHeight="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:7" ht="19.350000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" ht="19.350000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="21" t="s">
         <v>0</v>
       </c>
@@ -4310,8 +5129,11 @@
       <c r="E1" s="21"/>
       <c r="F1" s="21"/>
       <c r="G1" s="21"/>
-    </row>
-    <row r="2" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="H1" s="21"/>
+      <c r="I1" s="21"/>
+      <c r="J1" s="21"/>
+    </row>
+    <row r="2" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="22" t="s">
         <v>242</v>
       </c>
@@ -4322,36 +5144,45 @@
       <c r="F2" s="22"/>
       <c r="G2" s="22"/>
     </row>
-    <row r="3" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:10" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
         <v>2</v>
       </c>
       <c r="B3" s="5" t="s">
+        <v>275</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>278</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>279</v>
+      </c>
+      <c r="E3" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="C3" s="5" t="s">
+      <c r="F3" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="D3" s="6" t="s">
+      <c r="G3" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="E3" s="5" t="s">
+      <c r="H3" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="F3" s="5" t="s">
+      <c r="I3" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="G3" s="5" t="s">
+      <c r="J3" s="5" t="s">
         <v>8</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A1:G1"/>
     <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A1:J1"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation operator="equal" sqref="D1:D3" xr:uid="{00000000-0002-0000-0700-000000000000}">
+    <dataValidation operator="equal" sqref="G3 D2 G1" xr:uid="{00000000-0002-0000-0700-000000000000}">
       <formula1>0</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -4367,10 +5198,10 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:J3"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.5703125" defaultRowHeight="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:7" ht="19.350000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" ht="19.350000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="21" t="s">
         <v>0</v>
       </c>
@@ -4380,8 +5211,11 @@
       <c r="E1" s="21"/>
       <c r="F1" s="21"/>
       <c r="G1" s="21"/>
-    </row>
-    <row r="2" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="H1" s="21"/>
+      <c r="I1" s="21"/>
+      <c r="J1" s="21"/>
+    </row>
+    <row r="2" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="22" t="s">
         <v>238</v>
       </c>
@@ -4392,36 +5226,45 @@
       <c r="F2" s="22"/>
       <c r="G2" s="22"/>
     </row>
-    <row r="3" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:10" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
         <v>2</v>
       </c>
       <c r="B3" s="5" t="s">
+        <v>275</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>278</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>279</v>
+      </c>
+      <c r="E3" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="C3" s="5" t="s">
+      <c r="F3" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="D3" s="6" t="s">
+      <c r="G3" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="E3" s="5" t="s">
+      <c r="H3" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="F3" s="5" t="s">
+      <c r="I3" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="G3" s="5" t="s">
+      <c r="J3" s="5" t="s">
         <v>8</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A1:G1"/>
     <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A1:J1"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation operator="equal" sqref="D1:D3" xr:uid="{00000000-0002-0000-0800-000000000000}">
+    <dataValidation operator="equal" sqref="G3 D2 G1" xr:uid="{00000000-0002-0000-0800-000000000000}">
       <formula1>0</formula1>
       <formula2>0</formula2>
     </dataValidation>

</xml_diff>

<commit_message>
test: unit story 2
</commit_message>
<xml_diff>
--- a/docs/tests/breco - cas de test.xlsx
+++ b/docs/tests/breco - cas de test.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\wamp\www\breco_v2_0_0\docs\tests\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{64AF3231-CEA9-452F-82AB-0FB9701476E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B1397359-ADE9-427B-A99E-FF655B7339E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="770" uniqueCount="273">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="770" uniqueCount="277">
   <si>
     <t>Plan de test Breco, cas de test</t>
   </si>
@@ -1021,9 +1021,6 @@
   </si>
   <si>
     <t>S2 - Autocomplétion ville</t>
-  </si>
-  <si>
-    <t>n'entre pas de chaîne (champ vide)</t>
   </si>
   <si>
     <t>entre deux lettres qui correspondent aux premières lettres d'une ville avec une seule réponse</t>
@@ -1094,9 +1091,6 @@
     <t>entre deux lettres qui ne correspondent à aucune premières lettres d'une ville</t>
   </si>
   <si>
-    <t>search?limit=10</t>
-  </si>
-  <si>
     <t>Équivalence</t>
   </si>
   <si>
@@ -1361,13 +1355,31 @@
     <t>Erreur "Le nombre de places ne peut pas dépasser 8"</t>
   </si>
   <si>
-    <t>entre une lettre</t>
-  </si>
-  <si>
-    <t>Erreur : "La recherche doit contenir au moins 2 caractères"</t>
-  </si>
-  <si>
-    <t>S2 - appel API direct avec une lettre (bypass frontend)</t>
+    <t>q=""</t>
+  </si>
+  <si>
+    <t>q='r'</t>
+  </si>
+  <si>
+    <t>q='@#&lt;&gt;?&amp;+!'</t>
+  </si>
+  <si>
+    <t>appel API direct avec une lettre (bypass frontend)</t>
+  </si>
+  <si>
+    <t>n'entre pas de chaîne (champ vide) pour la ville</t>
+  </si>
+  <si>
+    <t>entre une ville avec une seule lettre</t>
+  </si>
+  <si>
+    <t>Erreur "La ville est requise"</t>
+  </si>
+  <si>
+    <t>Erreur "Au moins 2 caractères"</t>
+  </si>
+  <si>
+    <t>Erreur "Caractères non autorisés"</t>
   </si>
 </sst>
 </file>
@@ -1751,13 +1763,13 @@
         <v>2</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="E3" s="1" t="s">
         <v>3</v>
@@ -1783,13 +1795,13 @@
         <v>9</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="E4" s="3" t="s">
         <v>10</v>
@@ -1801,7 +1813,7 @@
         <v>12</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="I4" s="3" t="s">
         <v>13</v>
@@ -1815,13 +1827,13 @@
         <v>15</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="E5" s="3" t="s">
         <v>10</v>
@@ -1833,7 +1845,7 @@
         <v>17</v>
       </c>
       <c r="H5" s="3" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="I5" s="3" t="s">
         <v>13</v>
@@ -1847,13 +1859,13 @@
         <v>18</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="E6" s="3" t="s">
         <v>10</v>
@@ -1865,7 +1877,7 @@
         <v>20</v>
       </c>
       <c r="H6" s="3" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="I6" s="3" t="s">
         <v>13</v>
@@ -1879,13 +1891,13 @@
         <v>21</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="E7" s="3" t="s">
         <v>10</v>
@@ -1911,13 +1923,13 @@
         <v>27</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="E8" s="3" t="s">
         <v>10</v>
@@ -1929,7 +1941,7 @@
         <v>29</v>
       </c>
       <c r="H8" s="3" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="I8" s="3" t="s">
         <v>30</v>
@@ -1943,13 +1955,13 @@
         <v>31</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="E9" s="3" t="s">
         <v>10</v>
@@ -1961,7 +1973,7 @@
         <v>33</v>
       </c>
       <c r="H9" s="3" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="I9" s="3" t="s">
         <v>30</v>
@@ -1975,13 +1987,13 @@
         <v>34</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="E10" s="3" t="s">
         <v>10</v>
@@ -1993,7 +2005,7 @@
         <v>36</v>
       </c>
       <c r="H10" s="3" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="I10" s="3" t="s">
         <v>13</v>
@@ -2007,13 +2019,13 @@
         <v>37</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="E11" s="3" t="s">
         <v>10</v>
@@ -2025,7 +2037,7 @@
         <v>39</v>
       </c>
       <c r="H11" s="3" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
       <c r="I11" s="3" t="s">
         <v>30</v>
@@ -2039,13 +2051,13 @@
         <v>40</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="E12" s="3" t="s">
         <v>10</v>
@@ -2071,13 +2083,13 @@
         <v>44</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="E13" s="3" t="s">
         <v>10</v>
@@ -2089,7 +2101,7 @@
         <v>46</v>
       </c>
       <c r="H13" s="3" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="I13" s="3" t="s">
         <v>13</v>
@@ -2103,13 +2115,13 @@
         <v>47</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="E14" s="3" t="s">
         <v>10</v>
@@ -2121,7 +2133,7 @@
         <v>49</v>
       </c>
       <c r="H14" s="3" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="I14" s="3" t="s">
         <v>13</v>
@@ -2135,13 +2147,13 @@
         <v>50</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="D15" s="3" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="E15" s="3" t="s">
         <v>10</v>
@@ -2153,7 +2165,7 @@
         <v>52</v>
       </c>
       <c r="H15" s="3" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="I15" s="3" t="s">
         <v>30</v>
@@ -2167,13 +2179,13 @@
         <v>53</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="D16" s="3" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="E16" s="3" t="s">
         <v>10</v>
@@ -2199,13 +2211,13 @@
         <v>57</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="D17" s="3" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="E17" s="3" t="s">
         <v>10</v>
@@ -2217,7 +2229,7 @@
         <v>59</v>
       </c>
       <c r="H17" s="3" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="I17" s="3" t="s">
         <v>13</v>
@@ -2231,13 +2243,13 @@
         <v>60</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="D18" s="3" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="E18" s="3" t="s">
         <v>10</v>
@@ -2249,7 +2261,7 @@
         <v>62</v>
       </c>
       <c r="H18" s="3" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="I18" s="3" t="s">
         <v>13</v>
@@ -2263,13 +2275,13 @@
         <v>63</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="C19" s="3" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="D19" s="3" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="E19" s="3" t="s">
         <v>10</v>
@@ -2295,13 +2307,13 @@
         <v>67</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="C20" s="3" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="D20" s="3" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="E20" s="3" t="s">
         <v>10</v>
@@ -2313,7 +2325,7 @@
         <v>69</v>
       </c>
       <c r="H20" s="3" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="I20" s="3" t="s">
         <v>30</v>
@@ -2327,13 +2339,13 @@
         <v>70</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="C21" s="3" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="D21" s="3" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="E21" s="3" t="s">
         <v>10</v>
@@ -2359,13 +2371,13 @@
         <v>73</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="C22" s="3" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="D22" s="3" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="E22" s="3" t="s">
         <v>10</v>
@@ -2391,13 +2403,13 @@
         <v>76</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="C23" s="3" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="D23" s="3" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="E23" s="3" t="s">
         <v>10</v>
@@ -2423,13 +2435,13 @@
         <v>79</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="C24" s="3" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="D24" s="3" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="E24" s="3" t="s">
         <v>10</v>
@@ -2455,13 +2467,13 @@
         <v>82</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="C25" s="3" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="D25" s="3" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="E25" s="3" t="s">
         <v>10</v>
@@ -2473,7 +2485,7 @@
         <v>84</v>
       </c>
       <c r="H25" s="3" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="I25" s="3" t="s">
         <v>13</v>
@@ -2487,13 +2499,13 @@
         <v>85</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="C26" s="3" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="D26" s="3" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="E26" s="3" t="s">
         <v>10</v>
@@ -2505,7 +2517,7 @@
         <v>87</v>
       </c>
       <c r="H26" s="3" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="I26" s="3" t="s">
         <v>13</v>
@@ -2519,13 +2531,13 @@
         <v>88</v>
       </c>
       <c r="B27" s="3" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="C27" s="3" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="D27" s="3" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="E27" s="3" t="s">
         <v>10</v>
@@ -2551,13 +2563,13 @@
         <v>92</v>
       </c>
       <c r="B28" s="3" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="C28" s="3" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="D28" s="3" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="E28" s="3" t="s">
         <v>10</v>
@@ -2569,7 +2581,7 @@
         <v>94</v>
       </c>
       <c r="H28" s="3" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="I28" s="3" t="s">
         <v>30</v>
@@ -2583,13 +2595,13 @@
         <v>95</v>
       </c>
       <c r="B29" s="3" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="C29" s="3" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="D29" s="3" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="E29" s="3" t="s">
         <v>10</v>
@@ -2615,13 +2627,13 @@
         <v>98</v>
       </c>
       <c r="B30" s="3" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="C30" s="3" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="D30" s="3" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="E30" s="3" t="s">
         <v>10</v>
@@ -2630,7 +2642,7 @@
         <v>99</v>
       </c>
       <c r="G30" s="16" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="H30" s="17" t="s">
         <v>91</v>
@@ -2647,13 +2659,13 @@
         <v>100</v>
       </c>
       <c r="B31" s="3" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="C31" s="3" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="D31" s="3" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="E31" s="3" t="s">
         <v>10</v>
@@ -2662,7 +2674,7 @@
         <v>101</v>
       </c>
       <c r="G31" s="16" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="H31" s="17" t="s">
         <v>91</v>
@@ -2679,13 +2691,13 @@
         <v>102</v>
       </c>
       <c r="B32" s="3" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="C32" s="3" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="D32" s="3" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="E32" s="3" t="s">
         <v>10</v>
@@ -2694,7 +2706,7 @@
         <v>103</v>
       </c>
       <c r="G32" s="16" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="H32" s="17" t="s">
         <v>91</v>
@@ -2711,13 +2723,13 @@
         <v>104</v>
       </c>
       <c r="B33" s="3" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="C33" s="3" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="D33" s="3" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="E33" s="3" t="s">
         <v>10</v>
@@ -2729,7 +2741,7 @@
         <v>106</v>
       </c>
       <c r="H33" s="15" t="s">
-        <v>257</v>
+        <v>255</v>
       </c>
       <c r="I33" s="3" t="s">
         <v>30</v>
@@ -2743,13 +2755,13 @@
         <v>107</v>
       </c>
       <c r="B34" s="3" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="C34" s="3" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="D34" s="3" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="E34" s="3" t="s">
         <v>10</v>
@@ -2775,19 +2787,19 @@
         <v>111</v>
       </c>
       <c r="B35" s="3" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="C35" s="3" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="D35" s="3" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="E35" s="3" t="s">
         <v>10</v>
       </c>
       <c r="F35" s="15" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="G35" s="16" t="s">
         <v>112</v>
@@ -2807,13 +2819,13 @@
         <v>113</v>
       </c>
       <c r="B36" s="3" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="C36" s="3" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="D36" s="3" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="E36" s="3" t="s">
         <v>10</v>
@@ -2822,10 +2834,10 @@
         <v>114</v>
       </c>
       <c r="G36" s="19" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="H36" s="15" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="I36" s="3" t="s">
         <v>30</v>
@@ -2839,13 +2851,13 @@
         <v>115</v>
       </c>
       <c r="B37" s="3" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="C37" s="3" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="D37" s="3" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="E37" s="3" t="s">
         <v>10</v>
@@ -2871,13 +2883,13 @@
         <v>119</v>
       </c>
       <c r="B38" s="3" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="C38" s="3" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="D38" s="3" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="E38" s="3" t="s">
         <v>10</v>
@@ -2903,13 +2915,13 @@
         <v>122</v>
       </c>
       <c r="B39" s="3" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="C39" s="3" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="D39" s="3" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="E39" s="3" t="s">
         <v>10</v>
@@ -2935,22 +2947,22 @@
         <v>123</v>
       </c>
       <c r="B40" s="3" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="C40" s="3" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="D40" s="3" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="E40" s="3" t="s">
         <v>10</v>
       </c>
       <c r="F40" s="15" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="G40" s="19" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
       <c r="H40" s="15" t="s">
         <v>128</v>
@@ -2967,13 +2979,13 @@
         <v>127</v>
       </c>
       <c r="B41" s="3" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="C41" s="3" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="D41" s="3" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="E41" s="3" t="s">
         <v>10</v>
@@ -2985,7 +2997,7 @@
         <v>131</v>
       </c>
       <c r="H41" s="3" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
       <c r="I41" s="3" t="s">
         <v>13</v>
@@ -2999,13 +3011,13 @@
         <v>129</v>
       </c>
       <c r="B42" s="3" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="C42" s="3" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="D42" s="3" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="E42" s="3" t="s">
         <v>10</v>
@@ -3014,10 +3026,10 @@
         <v>133</v>
       </c>
       <c r="G42" s="19" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="H42" s="3" t="s">
-        <v>256</v>
+        <v>254</v>
       </c>
       <c r="I42" s="3" t="s">
         <v>13</v>
@@ -3031,13 +3043,13 @@
         <v>132</v>
       </c>
       <c r="B43" s="3" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="C43" s="3" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="D43" s="3" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="E43" s="3" t="s">
         <v>10</v>
@@ -3063,19 +3075,19 @@
         <v>134</v>
       </c>
       <c r="B44" s="3" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="C44" s="3" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="D44" s="3" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="E44" s="3" t="s">
         <v>10</v>
       </c>
       <c r="F44" s="15" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="G44" s="19" t="s">
         <v>139</v>
@@ -3095,13 +3107,13 @@
         <v>138</v>
       </c>
       <c r="B45" s="3" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="C45" s="3" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="D45" s="3" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="E45" s="3" t="s">
         <v>10</v>
@@ -3127,13 +3139,13 @@
         <v>140</v>
       </c>
       <c r="B46" s="3" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="C46" s="3" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="D46" s="3" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="E46" s="3" t="s">
         <v>10</v>
@@ -3142,10 +3154,10 @@
         <v>145</v>
       </c>
       <c r="G46" s="19" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="H46" s="3" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
       <c r="I46" s="3" t="s">
         <v>13</v>
@@ -3159,13 +3171,13 @@
         <v>144</v>
       </c>
       <c r="B47" s="3" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="C47" s="3" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="D47" s="3" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="E47" s="3" t="s">
         <v>10</v>
@@ -3174,7 +3186,7 @@
         <v>147</v>
       </c>
       <c r="G47" s="19" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="H47" s="17" t="s">
         <v>148</v>
@@ -3191,22 +3203,22 @@
         <v>146</v>
       </c>
       <c r="B48" s="3" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="C48" s="3" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="D48" s="3" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="E48" s="3" t="s">
         <v>10</v>
       </c>
       <c r="F48" s="15" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="G48" s="19" t="s">
-        <v>266</v>
+        <v>264</v>
       </c>
       <c r="H48" s="15" t="s">
         <v>128</v>
@@ -3223,13 +3235,13 @@
         <v>149</v>
       </c>
       <c r="B49" s="3" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="C49" s="3" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="D49" s="3" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="E49" s="3" t="s">
         <v>10</v>
@@ -3255,13 +3267,13 @@
         <v>150</v>
       </c>
       <c r="B50" s="3" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="C50" s="3" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="D50" s="3" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="E50" s="3" t="s">
         <v>10</v>
@@ -3270,10 +3282,10 @@
         <v>155</v>
       </c>
       <c r="G50" s="19" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="H50" s="3" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="I50" s="3" t="s">
         <v>13</v>
@@ -3287,13 +3299,13 @@
         <v>154</v>
       </c>
       <c r="B51" s="3" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="C51" s="3" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="D51" s="3" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="E51" s="3" t="s">
         <v>10</v>
@@ -3319,13 +3331,13 @@
         <v>156</v>
       </c>
       <c r="B52" s="3" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="C52" s="3" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="D52" s="3" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="E52" s="3" t="s">
         <v>10</v>
@@ -3334,7 +3346,7 @@
         <v>161</v>
       </c>
       <c r="G52" s="19" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
       <c r="H52" s="15" t="s">
         <v>128</v>
@@ -3351,13 +3363,13 @@
         <v>160</v>
       </c>
       <c r="B53" s="3" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="C53" s="3" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="D53" s="3" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="E53" s="3" t="s">
         <v>10</v>
@@ -3369,7 +3381,7 @@
         <v>164</v>
       </c>
       <c r="H53" s="3" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
       <c r="I53" s="3" t="s">
         <v>13</v>
@@ -3383,13 +3395,13 @@
         <v>162</v>
       </c>
       <c r="B54" s="3" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="C54" s="3" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="D54" s="3" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="E54" s="3" t="s">
         <v>10</v>
@@ -3401,7 +3413,7 @@
         <v>167</v>
       </c>
       <c r="H54" s="3" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="I54" s="3" t="s">
         <v>13</v>
@@ -3415,13 +3427,13 @@
         <v>165</v>
       </c>
       <c r="B55" s="3" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="C55" s="3" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="D55" s="3" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="E55" s="3" t="s">
         <v>10</v>
@@ -3447,13 +3459,13 @@
         <v>168</v>
       </c>
       <c r="B56" s="3" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="C56" s="3" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="D56" s="3" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="E56" s="3" t="s">
         <v>173</v>
@@ -3489,13 +3501,13 @@
         <v>172</v>
       </c>
       <c r="B57" s="3" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="C57" s="3" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="D57" s="3" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="E57" s="3" t="s">
         <v>173</v>
@@ -3531,13 +3543,13 @@
         <v>174</v>
       </c>
       <c r="B58" s="3" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="C58" s="3" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="D58" s="3" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="E58" s="3" t="s">
         <v>173</v>
@@ -3563,13 +3575,13 @@
         <v>175</v>
       </c>
       <c r="B59" s="3" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="C59" s="3" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="D59" s="3" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="E59" s="3" t="s">
         <v>173</v>
@@ -3778,13 +3790,13 @@
         <v>2</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="E3" s="1" t="s">
         <v>3</v>
@@ -3872,13 +3884,13 @@
         <v>2</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="E3" s="1" t="s">
         <v>3</v>
@@ -3904,25 +3916,25 @@
         <v>180</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="E4" s="7" t="s">
         <v>206</v>
       </c>
       <c r="F4" s="8" t="s">
-        <v>207</v>
+        <v>272</v>
       </c>
       <c r="G4" s="8" t="s">
-        <v>221</v>
+        <v>268</v>
       </c>
       <c r="H4" s="8" t="s">
-        <v>271</v>
+        <v>274</v>
       </c>
       <c r="I4" s="4" t="s">
         <v>13</v>
@@ -3936,25 +3948,25 @@
         <v>183</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="E5" s="7" t="s">
         <v>206</v>
       </c>
       <c r="F5" s="8" t="s">
-        <v>270</v>
+        <v>273</v>
       </c>
       <c r="G5" s="8" t="s">
-        <v>211</v>
+        <v>269</v>
       </c>
       <c r="H5" s="8" t="s">
-        <v>271</v>
+        <v>275</v>
       </c>
       <c r="I5" s="4" t="s">
         <v>13</v>
@@ -3968,28 +3980,28 @@
         <v>184</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="E6" s="7" t="s">
         <v>206</v>
       </c>
       <c r="F6" s="8" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="G6" s="8" t="s">
-        <v>223</v>
+        <v>270</v>
       </c>
       <c r="H6" s="8" t="s">
-        <v>225</v>
+        <v>276</v>
       </c>
       <c r="I6" s="4" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="J6" s="5" t="s">
         <v>14</v>
@@ -4000,25 +4012,25 @@
         <v>185</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="E7" s="7" t="s">
-        <v>272</v>
-      </c>
-      <c r="F7" s="8" t="s">
-        <v>270</v>
+        <v>206</v>
+      </c>
+      <c r="F7" s="7" t="s">
+        <v>271</v>
       </c>
       <c r="G7" s="8" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="H7" s="8" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="I7" s="4" t="s">
         <v>13</v>
@@ -4032,25 +4044,25 @@
         <v>186</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="E8" s="7" t="s">
         <v>206</v>
       </c>
       <c r="F8" s="8" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="G8" s="8" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="H8" s="8" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="I8" s="4" t="s">
         <v>25</v>
@@ -4064,25 +4076,25 @@
         <v>187</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="E9" s="7" t="s">
         <v>206</v>
       </c>
       <c r="F9" s="8" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="G9" s="8" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="H9" s="8" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="I9" s="4" t="s">
         <v>25</v>
@@ -4096,25 +4108,25 @@
         <v>188</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="E10" s="7" t="s">
         <v>206</v>
       </c>
       <c r="F10" s="8" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="G10" s="8" t="s">
+        <v>213</v>
+      </c>
+      <c r="H10" s="8" t="s">
         <v>214</v>
-      </c>
-      <c r="H10" s="8" t="s">
-        <v>215</v>
       </c>
       <c r="I10" s="4" t="s">
         <v>25</v>
@@ -4128,25 +4140,25 @@
         <v>189</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="E11" s="7" t="s">
         <v>206</v>
       </c>
       <c r="F11" s="8" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="G11" s="8" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="H11" s="8" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="I11" s="4" t="s">
         <v>25</v>
@@ -4160,28 +4172,28 @@
         <v>193</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>237</v>
+        <v>235</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
       <c r="E12" s="7" t="s">
         <v>206</v>
       </c>
       <c r="F12" s="8" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="G12" s="8" t="s">
+        <v>221</v>
+      </c>
+      <c r="H12" s="8" t="s">
         <v>223</v>
       </c>
-      <c r="H12" s="8" t="s">
-        <v>225</v>
-      </c>
       <c r="I12" s="4" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="J12" s="5" t="s">
         <v>14</v>
@@ -4250,13 +4262,13 @@
         <v>2</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="E3" s="1" t="s">
         <v>3</v>
@@ -4318,7 +4330,7 @@
     </row>
     <row r="2" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="10" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="B2" s="10"/>
       <c r="C2" s="10"/>
@@ -4332,13 +4344,13 @@
         <v>2</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="E3" s="1" t="s">
         <v>3</v>
@@ -4414,13 +4426,13 @@
         <v>2</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="E3" s="1" t="s">
         <v>3</v>
@@ -4496,13 +4508,13 @@
         <v>2</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="E3" s="1" t="s">
         <v>3</v>
@@ -4578,13 +4590,13 @@
         <v>2</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="E3" s="1" t="s">
         <v>3</v>
@@ -4660,13 +4672,13 @@
         <v>2</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="E3" s="1" t="s">
         <v>3</v>
@@ -4742,13 +4754,13 @@
         <v>2</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="E3" s="1" t="s">
         <v>3</v>

</xml_diff>

<commit_message>
test: TC-53 & TC-54
</commit_message>
<xml_diff>
--- a/docs/tests/breco - cas de test.xlsx
+++ b/docs/tests/breco - cas de test.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\wamp\www\breco_v2_0_0\docs\tests\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FEBCC166-BB5D-4C89-8A58-19CB9D5C715A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DE4690BC-4B45-40E5-B371-0138CB530B31}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1173" uniqueCount="413">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1175" uniqueCount="414">
   <si>
     <t>Plan de test Breco, cas de test</t>
   </si>
@@ -1795,6 +1795,9 @@
   </si>
   <si>
     <t>register.integration.spec.ts + AuthServiceTest.php</t>
+  </si>
+  <si>
+    <t>login.integration.spec.ts + AuthServiceTest.php</t>
   </si>
 </sst>
 </file>
@@ -2002,20 +2005,20 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="10" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2161,34 +2164,34 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="19.350000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="15" t="s">
+      <c r="A1" s="17" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="15"/>
-      <c r="C1" s="15"/>
-      <c r="D1" s="15"/>
-      <c r="E1" s="15"/>
-      <c r="F1" s="15"/>
-      <c r="G1" s="15"/>
-      <c r="H1" s="15"/>
-      <c r="I1" s="15"/>
-      <c r="J1" s="15"/>
-      <c r="K1" s="15"/>
+      <c r="B1" s="17"/>
+      <c r="C1" s="17"/>
+      <c r="D1" s="17"/>
+      <c r="E1" s="17"/>
+      <c r="F1" s="17"/>
+      <c r="G1" s="17"/>
+      <c r="H1" s="17"/>
+      <c r="I1" s="17"/>
+      <c r="J1" s="17"/>
+      <c r="K1" s="17"/>
     </row>
     <row r="2" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="17" t="s">
+      <c r="A2" s="18" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="17"/>
-      <c r="C2" s="17"/>
-      <c r="D2" s="17"/>
-      <c r="E2" s="17"/>
-      <c r="F2" s="17"/>
-      <c r="G2" s="17"/>
-      <c r="H2" s="17"/>
-      <c r="I2" s="17"/>
-      <c r="J2" s="17"/>
-      <c r="K2" s="17"/>
+      <c r="B2" s="18"/>
+      <c r="C2" s="18"/>
+      <c r="D2" s="18"/>
+      <c r="E2" s="18"/>
+      <c r="F2" s="18"/>
+      <c r="G2" s="18"/>
+      <c r="H2" s="18"/>
+      <c r="I2" s="18"/>
+      <c r="J2" s="18"/>
+      <c r="K2" s="18"/>
     </row>
     <row r="3" spans="1:11" ht="14.25" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
@@ -2226,7 +2229,7 @@
       </c>
     </row>
     <row r="4" spans="1:11" ht="14.25" x14ac:dyDescent="0.25">
-      <c r="A4" s="19" t="s">
+      <c r="A4" s="16" t="s">
         <v>9</v>
       </c>
       <c r="B4" s="3" t="s">
@@ -2261,7 +2264,7 @@
       </c>
     </row>
     <row r="5" spans="1:11" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="A5" s="19" t="s">
+      <c r="A5" s="16" t="s">
         <v>15</v>
       </c>
       <c r="B5" s="3" t="s">
@@ -2296,7 +2299,7 @@
       </c>
     </row>
     <row r="6" spans="1:11" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="A6" s="19" t="s">
+      <c r="A6" s="16" t="s">
         <v>18</v>
       </c>
       <c r="B6" s="3" t="s">
@@ -2331,7 +2334,7 @@
       </c>
     </row>
     <row r="7" spans="1:11" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="A7" s="19" t="s">
+      <c r="A7" s="16" t="s">
         <v>21</v>
       </c>
       <c r="B7" s="3" t="s">
@@ -2366,7 +2369,7 @@
       </c>
     </row>
     <row r="8" spans="1:11" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="A8" s="19" t="s">
+      <c r="A8" s="16" t="s">
         <v>27</v>
       </c>
       <c r="B8" s="3" t="s">
@@ -2401,7 +2404,7 @@
       </c>
     </row>
     <row r="9" spans="1:11" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="A9" s="19" t="s">
+      <c r="A9" s="16" t="s">
         <v>291</v>
       </c>
       <c r="B9" s="3" t="s">
@@ -2436,7 +2439,7 @@
       </c>
     </row>
     <row r="10" spans="1:11" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="A10" s="19" t="s">
+      <c r="A10" s="16" t="s">
         <v>292</v>
       </c>
       <c r="B10" s="3" t="s">
@@ -2471,7 +2474,7 @@
       </c>
     </row>
     <row r="11" spans="1:11" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="A11" s="19" t="s">
+      <c r="A11" s="16" t="s">
         <v>293</v>
       </c>
       <c r="B11" s="3" t="s">
@@ -2506,7 +2509,7 @@
       </c>
     </row>
     <row r="12" spans="1:11" ht="14.25" x14ac:dyDescent="0.25">
-      <c r="A12" s="19" t="s">
+      <c r="A12" s="16" t="s">
         <v>33</v>
       </c>
       <c r="B12" s="3" t="s">
@@ -2541,7 +2544,7 @@
       </c>
     </row>
     <row r="13" spans="1:11" ht="14.25" x14ac:dyDescent="0.25">
-      <c r="A13" s="19" t="s">
+      <c r="A13" s="16" t="s">
         <v>36</v>
       </c>
       <c r="B13" s="3" t="s">
@@ -2576,7 +2579,7 @@
       </c>
     </row>
     <row r="14" spans="1:11" ht="14.25" x14ac:dyDescent="0.25">
-      <c r="A14" s="19" t="s">
+      <c r="A14" s="16" t="s">
         <v>39</v>
       </c>
       <c r="B14" s="3" t="s">
@@ -2611,7 +2614,7 @@
       </c>
     </row>
     <row r="15" spans="1:11" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="A15" s="19" t="s">
+      <c r="A15" s="16" t="s">
         <v>43</v>
       </c>
       <c r="B15" s="3" t="s">
@@ -2646,7 +2649,7 @@
       </c>
     </row>
     <row r="16" spans="1:11" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="A16" s="19" t="s">
+      <c r="A16" s="16" t="s">
         <v>46</v>
       </c>
       <c r="B16" s="3" t="s">
@@ -2681,7 +2684,7 @@
       </c>
     </row>
     <row r="17" spans="1:11" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="A17" s="19" t="s">
+      <c r="A17" s="16" t="s">
         <v>49</v>
       </c>
       <c r="B17" s="3" t="s">
@@ -2716,7 +2719,7 @@
       </c>
     </row>
     <row r="18" spans="1:11" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="A18" s="19" t="s">
+      <c r="A18" s="16" t="s">
         <v>51</v>
       </c>
       <c r="B18" s="3" t="s">
@@ -2751,7 +2754,7 @@
       </c>
     </row>
     <row r="19" spans="1:11" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="A19" s="19" t="s">
+      <c r="A19" s="16" t="s">
         <v>55</v>
       </c>
       <c r="B19" s="3" t="s">
@@ -2786,7 +2789,7 @@
       </c>
     </row>
     <row r="20" spans="1:11" ht="38.25" x14ac:dyDescent="0.25">
-      <c r="A20" s="19" t="s">
+      <c r="A20" s="16" t="s">
         <v>58</v>
       </c>
       <c r="B20" s="3" t="s">
@@ -2821,7 +2824,7 @@
       </c>
     </row>
     <row r="21" spans="1:11" ht="14.25" x14ac:dyDescent="0.25">
-      <c r="A21" s="19" t="s">
+      <c r="A21" s="16" t="s">
         <v>61</v>
       </c>
       <c r="B21" s="3" t="s">
@@ -2856,7 +2859,7 @@
       </c>
     </row>
     <row r="22" spans="1:11" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="A22" s="19" t="s">
+      <c r="A22" s="16" t="s">
         <v>65</v>
       </c>
       <c r="B22" s="3" t="s">
@@ -2891,7 +2894,7 @@
       </c>
     </row>
     <row r="23" spans="1:11" ht="14.25" x14ac:dyDescent="0.25">
-      <c r="A23" s="19" t="s">
+      <c r="A23" s="16" t="s">
         <v>68</v>
       </c>
       <c r="B23" s="3" t="s">
@@ -2926,7 +2929,7 @@
       </c>
     </row>
     <row r="24" spans="1:11" ht="14.25" x14ac:dyDescent="0.25">
-      <c r="A24" s="19" t="s">
+      <c r="A24" s="16" t="s">
         <v>71</v>
       </c>
       <c r="B24" s="3" t="s">
@@ -2961,7 +2964,7 @@
       </c>
     </row>
     <row r="25" spans="1:11" ht="14.25" x14ac:dyDescent="0.25">
-      <c r="A25" s="19" t="s">
+      <c r="A25" s="16" t="s">
         <v>74</v>
       </c>
       <c r="B25" s="3" t="s">
@@ -2996,7 +2999,7 @@
       </c>
     </row>
     <row r="26" spans="1:11" ht="14.25" x14ac:dyDescent="0.25">
-      <c r="A26" s="19" t="s">
+      <c r="A26" s="16" t="s">
         <v>77</v>
       </c>
       <c r="B26" s="3" t="s">
@@ -3031,7 +3034,7 @@
       </c>
     </row>
     <row r="27" spans="1:11" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="A27" s="19" t="s">
+      <c r="A27" s="16" t="s">
         <v>80</v>
       </c>
       <c r="B27" s="3" t="s">
@@ -3066,7 +3069,7 @@
       </c>
     </row>
     <row r="28" spans="1:11" ht="38.25" x14ac:dyDescent="0.25">
-      <c r="A28" s="19" t="s">
+      <c r="A28" s="16" t="s">
         <v>83</v>
       </c>
       <c r="B28" s="3" t="s">
@@ -3101,7 +3104,7 @@
       </c>
     </row>
     <row r="29" spans="1:11" ht="14.25" x14ac:dyDescent="0.25">
-      <c r="A29" s="19" t="s">
+      <c r="A29" s="16" t="s">
         <v>86</v>
       </c>
       <c r="B29" s="3" t="s">
@@ -3136,7 +3139,7 @@
       </c>
     </row>
     <row r="30" spans="1:11" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="A30" s="19" t="s">
+      <c r="A30" s="16" t="s">
         <v>90</v>
       </c>
       <c r="B30" s="3" t="s">
@@ -3171,7 +3174,7 @@
       </c>
     </row>
     <row r="31" spans="1:11" ht="14.25" x14ac:dyDescent="0.25">
-      <c r="A31" s="19" t="s">
+      <c r="A31" s="16" t="s">
         <v>93</v>
       </c>
       <c r="B31" s="3" t="s">
@@ -3206,7 +3209,7 @@
       </c>
     </row>
     <row r="32" spans="1:11" ht="14.25" x14ac:dyDescent="0.25">
-      <c r="A32" s="19" t="s">
+      <c r="A32" s="16" t="s">
         <v>96</v>
       </c>
       <c r="B32" s="3" t="s">
@@ -3241,7 +3244,7 @@
       </c>
     </row>
     <row r="33" spans="1:11" ht="14.25" x14ac:dyDescent="0.25">
-      <c r="A33" s="19" t="s">
+      <c r="A33" s="16" t="s">
         <v>98</v>
       </c>
       <c r="B33" s="3" t="s">
@@ -3276,7 +3279,7 @@
       </c>
     </row>
     <row r="34" spans="1:11" ht="14.25" x14ac:dyDescent="0.25">
-      <c r="A34" s="19" t="s">
+      <c r="A34" s="16" t="s">
         <v>100</v>
       </c>
       <c r="B34" s="3" t="s">
@@ -3311,7 +3314,7 @@
       </c>
     </row>
     <row r="35" spans="1:11" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="A35" s="19" t="s">
+      <c r="A35" s="16" t="s">
         <v>102</v>
       </c>
       <c r="B35" s="3" t="s">
@@ -3346,7 +3349,7 @@
       </c>
     </row>
     <row r="36" spans="1:11" ht="14.25" x14ac:dyDescent="0.25">
-      <c r="A36" s="19" t="s">
+      <c r="A36" s="16" t="s">
         <v>282</v>
       </c>
       <c r="B36" s="3" t="s">
@@ -3381,7 +3384,7 @@
       </c>
     </row>
     <row r="37" spans="1:11" ht="14.25" x14ac:dyDescent="0.25">
-      <c r="A37" s="19" t="s">
+      <c r="A37" s="16" t="s">
         <v>283</v>
       </c>
       <c r="B37" s="3" t="s">
@@ -3416,7 +3419,7 @@
       </c>
     </row>
     <row r="38" spans="1:11" ht="14.25" x14ac:dyDescent="0.25">
-      <c r="A38" s="19" t="s">
+      <c r="A38" s="16" t="s">
         <v>284</v>
       </c>
       <c r="B38" s="3" t="s">
@@ -3451,7 +3454,7 @@
       </c>
     </row>
     <row r="39" spans="1:11" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="A39" s="19" t="s">
+      <c r="A39" s="16" t="s">
         <v>108</v>
       </c>
       <c r="B39" s="3" t="s">
@@ -3486,7 +3489,7 @@
       </c>
     </row>
     <row r="40" spans="1:11" ht="15" x14ac:dyDescent="0.25">
-      <c r="A40" s="19" t="s">
+      <c r="A40" s="16" t="s">
         <v>281</v>
       </c>
       <c r="B40" s="3" t="s">
@@ -3521,7 +3524,7 @@
       </c>
     </row>
     <row r="41" spans="1:11" ht="15" x14ac:dyDescent="0.25">
-      <c r="A41" s="19" t="s">
+      <c r="A41" s="16" t="s">
         <v>280</v>
       </c>
       <c r="B41" s="3" t="s">
@@ -3556,7 +3559,7 @@
       </c>
     </row>
     <row r="42" spans="1:11" ht="15" x14ac:dyDescent="0.25">
-      <c r="A42" s="19" t="s">
+      <c r="A42" s="16" t="s">
         <v>279</v>
       </c>
       <c r="B42" s="3" t="s">
@@ -3591,7 +3594,7 @@
       </c>
     </row>
     <row r="43" spans="1:11" ht="15" x14ac:dyDescent="0.25">
-      <c r="A43" s="19" t="s">
+      <c r="A43" s="16" t="s">
         <v>110</v>
       </c>
       <c r="B43" s="3" t="s">
@@ -3626,7 +3629,7 @@
       </c>
     </row>
     <row r="44" spans="1:11" ht="15" x14ac:dyDescent="0.25">
-      <c r="A44" s="19" t="s">
+      <c r="A44" s="16" t="s">
         <v>114</v>
       </c>
       <c r="B44" s="3" t="s">
@@ -3661,7 +3664,7 @@
       </c>
     </row>
     <row r="45" spans="1:11" ht="15" x14ac:dyDescent="0.25">
-      <c r="A45" s="19" t="s">
+      <c r="A45" s="16" t="s">
         <v>117</v>
       </c>
       <c r="B45" s="3" t="s">
@@ -3696,7 +3699,7 @@
       </c>
     </row>
     <row r="46" spans="1:11" ht="15" x14ac:dyDescent="0.25">
-      <c r="A46" s="19" t="s">
+      <c r="A46" s="16" t="s">
         <v>118</v>
       </c>
       <c r="B46" s="3" t="s">
@@ -3731,7 +3734,7 @@
       </c>
     </row>
     <row r="47" spans="1:11" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="A47" s="19" t="s">
+      <c r="A47" s="16" t="s">
         <v>122</v>
       </c>
       <c r="B47" s="3" t="s">
@@ -3766,7 +3769,7 @@
       </c>
     </row>
     <row r="48" spans="1:11" ht="60" x14ac:dyDescent="0.25">
-      <c r="A48" s="19" t="s">
+      <c r="A48" s="16" t="s">
         <v>124</v>
       </c>
       <c r="B48" s="3" t="s">
@@ -3801,7 +3804,7 @@
       </c>
     </row>
     <row r="49" spans="1:21" ht="15" x14ac:dyDescent="0.25">
-      <c r="A49" s="19" t="s">
+      <c r="A49" s="16" t="s">
         <v>127</v>
       </c>
       <c r="B49" s="3" t="s">
@@ -3836,7 +3839,7 @@
       </c>
     </row>
     <row r="50" spans="1:21" ht="15" x14ac:dyDescent="0.25">
-      <c r="A50" s="19" t="s">
+      <c r="A50" s="16" t="s">
         <v>129</v>
       </c>
       <c r="B50" s="3" t="s">
@@ -3871,7 +3874,7 @@
       </c>
     </row>
     <row r="51" spans="1:21" ht="15" x14ac:dyDescent="0.25">
-      <c r="A51" s="19" t="s">
+      <c r="A51" s="16" t="s">
         <v>133</v>
       </c>
       <c r="B51" s="3" t="s">
@@ -3906,7 +3909,7 @@
       </c>
     </row>
     <row r="52" spans="1:21" ht="40.5" x14ac:dyDescent="0.25">
-      <c r="A52" s="19" t="s">
+      <c r="A52" s="16" t="s">
         <v>135</v>
       </c>
       <c r="B52" s="3" t="s">
@@ -3941,7 +3944,7 @@
       </c>
     </row>
     <row r="53" spans="1:21" ht="15" x14ac:dyDescent="0.25">
-      <c r="A53" s="19" t="s">
+      <c r="A53" s="16" t="s">
         <v>139</v>
       </c>
       <c r="B53" s="3" t="s">
@@ -3976,7 +3979,7 @@
       </c>
     </row>
     <row r="54" spans="1:21" ht="15" x14ac:dyDescent="0.25">
-      <c r="A54" s="19" t="s">
+      <c r="A54" s="16" t="s">
         <v>141</v>
       </c>
       <c r="B54" s="3" t="s">
@@ -4011,7 +4014,7 @@
       </c>
     </row>
     <row r="55" spans="1:21" ht="15" x14ac:dyDescent="0.25">
-      <c r="A55" s="19" t="s">
+      <c r="A55" s="16" t="s">
         <v>144</v>
       </c>
       <c r="B55" s="3" t="s">
@@ -4046,7 +4049,7 @@
       </c>
     </row>
     <row r="56" spans="1:21" ht="27.75" x14ac:dyDescent="0.25">
-      <c r="A56" s="19" t="s">
+      <c r="A56" s="16" t="s">
         <v>145</v>
       </c>
       <c r="B56" s="3" t="s">
@@ -4081,7 +4084,7 @@
       </c>
     </row>
     <row r="57" spans="1:21" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A57" s="19" t="s">
+      <c r="A57" s="16" t="s">
         <v>149</v>
       </c>
       <c r="B57" s="3" t="s">
@@ -4116,7 +4119,7 @@
       </c>
     </row>
     <row r="58" spans="1:21" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A58" s="19" t="s">
+      <c r="A58" s="16" t="s">
         <v>151</v>
       </c>
       <c r="B58" s="3" t="s">
@@ -4151,7 +4154,7 @@
       </c>
     </row>
     <row r="59" spans="1:21" ht="15" x14ac:dyDescent="0.25">
-      <c r="A59" s="19" t="s">
+      <c r="A59" s="16" t="s">
         <v>155</v>
       </c>
       <c r="B59" s="3" t="s">
@@ -4186,7 +4189,7 @@
       </c>
     </row>
     <row r="60" spans="1:21" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="A60" s="19" t="s">
+      <c r="A60" s="16" t="s">
         <v>157</v>
       </c>
       <c r="B60" s="3" t="s">
@@ -4221,7 +4224,7 @@
       </c>
     </row>
     <row r="61" spans="1:21" ht="15" x14ac:dyDescent="0.25">
-      <c r="A61" s="19" t="s">
+      <c r="A61" s="16" t="s">
         <v>160</v>
       </c>
       <c r="B61" s="3" t="s">
@@ -4256,7 +4259,7 @@
       </c>
     </row>
     <row r="62" spans="1:21" ht="38.25" x14ac:dyDescent="0.25">
-      <c r="A62" s="19" t="s">
+      <c r="A62" s="16" t="s">
         <v>270</v>
       </c>
       <c r="B62" s="3" t="s">
@@ -4291,7 +4294,7 @@
       </c>
     </row>
     <row r="63" spans="1:21" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="A63" s="19" t="s">
+      <c r="A63" s="16" t="s">
         <v>271</v>
       </c>
       <c r="B63" s="3" t="s">
@@ -4326,7 +4329,7 @@
       </c>
     </row>
     <row r="64" spans="1:21" s="12" customFormat="1" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="A64" s="3" t="s">
+      <c r="A64" s="16" t="s">
         <v>163</v>
       </c>
       <c r="B64" s="3" t="s">
@@ -4338,7 +4341,9 @@
       <c r="D64" s="3" t="s">
         <v>225</v>
       </c>
-      <c r="E64" s="3"/>
+      <c r="E64" s="3" t="s">
+        <v>413</v>
+      </c>
       <c r="F64" s="3" t="s">
         <v>168</v>
       </c>
@@ -4369,7 +4374,7 @@
       <c r="U64" s="13"/>
     </row>
     <row r="65" spans="1:21" s="12" customFormat="1" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="A65" s="3" t="s">
+      <c r="A65" s="16" t="s">
         <v>167</v>
       </c>
       <c r="B65" s="3" t="s">
@@ -4381,7 +4386,9 @@
       <c r="D65" s="3" t="s">
         <v>225</v>
       </c>
-      <c r="E65" s="3"/>
+      <c r="E65" s="3" t="s">
+        <v>413</v>
+      </c>
       <c r="F65" s="3" t="s">
         <v>168</v>
       </c>
@@ -4704,7 +4711,7 @@
       <c r="J74" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="K74" s="18" t="s">
+      <c r="K74" s="15" t="s">
         <v>359</v>
       </c>
     </row>
@@ -5100,7 +5107,7 @@
       <c r="J86" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="K86" s="18" t="s">
+      <c r="K86" s="15" t="s">
         <v>359</v>
       </c>
     </row>
@@ -5199,7 +5206,7 @@
       <c r="J89" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="K89" s="18" t="s">
+      <c r="K89" s="15" t="s">
         <v>359</v>
       </c>
     </row>
@@ -5473,30 +5480,30 @@
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.5703125" defaultRowHeight="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:11" ht="19.350000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="15" t="s">
+      <c r="A1" s="17" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="15"/>
-      <c r="C1" s="15"/>
-      <c r="D1" s="15"/>
-      <c r="E1" s="15"/>
-      <c r="F1" s="15"/>
-      <c r="G1" s="15"/>
-      <c r="H1" s="15"/>
-      <c r="I1" s="15"/>
-      <c r="J1" s="15"/>
-      <c r="K1" s="15"/>
+      <c r="B1" s="17"/>
+      <c r="C1" s="17"/>
+      <c r="D1" s="17"/>
+      <c r="E1" s="17"/>
+      <c r="F1" s="17"/>
+      <c r="G1" s="17"/>
+      <c r="H1" s="17"/>
+      <c r="I1" s="17"/>
+      <c r="J1" s="17"/>
+      <c r="K1" s="17"/>
     </row>
     <row r="2" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="16" t="s">
+      <c r="A2" s="19" t="s">
         <v>191</v>
       </c>
-      <c r="B2" s="16"/>
-      <c r="C2" s="16"/>
-      <c r="D2" s="16"/>
-      <c r="E2" s="16"/>
-      <c r="F2" s="16"/>
-      <c r="G2" s="16"/>
+      <c r="B2" s="19"/>
+      <c r="C2" s="19"/>
+      <c r="D2" s="19"/>
+      <c r="E2" s="19"/>
+      <c r="F2" s="19"/>
+      <c r="G2" s="19"/>
     </row>
     <row r="3" spans="1:11" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
@@ -5568,34 +5575,34 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="53.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="15" t="s">
+      <c r="A1" s="17" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="15"/>
-      <c r="C1" s="15"/>
-      <c r="D1" s="15"/>
-      <c r="E1" s="15"/>
-      <c r="F1" s="15"/>
-      <c r="G1" s="15"/>
-      <c r="H1" s="15"/>
-      <c r="I1" s="15"/>
-      <c r="J1" s="15"/>
-      <c r="K1" s="15"/>
+      <c r="B1" s="17"/>
+      <c r="C1" s="17"/>
+      <c r="D1" s="17"/>
+      <c r="E1" s="17"/>
+      <c r="F1" s="17"/>
+      <c r="G1" s="17"/>
+      <c r="H1" s="17"/>
+      <c r="I1" s="17"/>
+      <c r="J1" s="17"/>
+      <c r="K1" s="17"/>
     </row>
     <row r="2" spans="1:11" ht="53.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="16" t="s">
+      <c r="A2" s="19" t="s">
         <v>192</v>
       </c>
-      <c r="B2" s="16"/>
-      <c r="C2" s="16"/>
-      <c r="D2" s="16"/>
-      <c r="E2" s="16"/>
-      <c r="F2" s="16"/>
-      <c r="G2" s="16"/>
-      <c r="H2" s="16"/>
-      <c r="I2" s="16"/>
-      <c r="J2" s="16"/>
-      <c r="K2" s="16"/>
+      <c r="B2" s="19"/>
+      <c r="C2" s="19"/>
+      <c r="D2" s="19"/>
+      <c r="E2" s="19"/>
+      <c r="F2" s="19"/>
+      <c r="G2" s="19"/>
+      <c r="H2" s="19"/>
+      <c r="I2" s="19"/>
+      <c r="J2" s="19"/>
+      <c r="K2" s="19"/>
     </row>
     <row r="3" spans="1:11" ht="53.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
@@ -5633,7 +5640,7 @@
       </c>
     </row>
     <row r="4" spans="1:11" ht="53.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="19" t="s">
+      <c r="A4" s="16" t="s">
         <v>398</v>
       </c>
       <c r="B4" s="3" t="s">
@@ -5668,7 +5675,7 @@
       </c>
     </row>
     <row r="5" spans="1:11" ht="53.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="19" t="s">
+      <c r="A5" s="16" t="s">
         <v>399</v>
       </c>
       <c r="B5" s="3" t="s">
@@ -5703,7 +5710,7 @@
       </c>
     </row>
     <row r="6" spans="1:11" ht="53.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="19" t="s">
+      <c r="A6" s="16" t="s">
         <v>400</v>
       </c>
       <c r="B6" s="3" t="s">
@@ -5966,33 +5973,33 @@
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.5703125" defaultRowHeight="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:11" ht="19.350000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="15" t="s">
+      <c r="A1" s="17" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="15"/>
-      <c r="C1" s="15"/>
-      <c r="D1" s="15"/>
-      <c r="E1" s="15"/>
-      <c r="F1" s="15"/>
-      <c r="G1" s="15"/>
-      <c r="H1" s="15"/>
-      <c r="I1" s="15"/>
-      <c r="J1" s="15"/>
-      <c r="K1" s="15"/>
+      <c r="B1" s="17"/>
+      <c r="C1" s="17"/>
+      <c r="D1" s="17"/>
+      <c r="E1" s="17"/>
+      <c r="F1" s="17"/>
+      <c r="G1" s="17"/>
+      <c r="H1" s="17"/>
+      <c r="I1" s="17"/>
+      <c r="J1" s="17"/>
+      <c r="K1" s="17"/>
     </row>
     <row r="2" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="16" t="s">
+      <c r="A2" s="19" t="s">
         <v>193</v>
       </c>
-      <c r="B2" s="16"/>
-      <c r="C2" s="16"/>
-      <c r="D2" s="16"/>
-      <c r="E2" s="16"/>
-      <c r="F2" s="16"/>
-      <c r="G2" s="16"/>
-      <c r="H2" s="16"/>
-      <c r="I2" s="16"/>
-      <c r="J2" s="16"/>
+      <c r="B2" s="19"/>
+      <c r="C2" s="19"/>
+      <c r="D2" s="19"/>
+      <c r="E2" s="19"/>
+      <c r="F2" s="19"/>
+      <c r="G2" s="19"/>
+      <c r="H2" s="19"/>
+      <c r="I2" s="19"/>
+      <c r="J2" s="19"/>
     </row>
     <row r="3" spans="1:11" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
@@ -6055,30 +6062,30 @@
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.5703125" defaultRowHeight="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:11" ht="19.350000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="15" t="s">
+      <c r="A1" s="17" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="15"/>
-      <c r="C1" s="15"/>
-      <c r="D1" s="15"/>
-      <c r="E1" s="15"/>
-      <c r="F1" s="15"/>
-      <c r="G1" s="15"/>
-      <c r="H1" s="15"/>
-      <c r="I1" s="15"/>
-      <c r="J1" s="15"/>
-      <c r="K1" s="15"/>
+      <c r="B1" s="17"/>
+      <c r="C1" s="17"/>
+      <c r="D1" s="17"/>
+      <c r="E1" s="17"/>
+      <c r="F1" s="17"/>
+      <c r="G1" s="17"/>
+      <c r="H1" s="17"/>
+      <c r="I1" s="17"/>
+      <c r="J1" s="17"/>
+      <c r="K1" s="17"/>
     </row>
     <row r="2" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="16" t="s">
+      <c r="A2" s="19" t="s">
         <v>226</v>
       </c>
-      <c r="B2" s="16"/>
-      <c r="C2" s="16"/>
-      <c r="D2" s="16"/>
-      <c r="E2" s="16"/>
-      <c r="F2" s="16"/>
-      <c r="G2" s="16"/>
+      <c r="B2" s="19"/>
+      <c r="C2" s="19"/>
+      <c r="D2" s="19"/>
+      <c r="E2" s="19"/>
+      <c r="F2" s="19"/>
+      <c r="G2" s="19"/>
     </row>
     <row r="3" spans="1:11" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
@@ -6141,30 +6148,30 @@
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.5703125" defaultRowHeight="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:11" ht="19.350000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="15" t="s">
+      <c r="A1" s="17" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="15"/>
-      <c r="C1" s="15"/>
-      <c r="D1" s="15"/>
-      <c r="E1" s="15"/>
-      <c r="F1" s="15"/>
-      <c r="G1" s="15"/>
-      <c r="H1" s="15"/>
-      <c r="I1" s="15"/>
-      <c r="J1" s="15"/>
-      <c r="K1" s="15"/>
+      <c r="B1" s="17"/>
+      <c r="C1" s="17"/>
+      <c r="D1" s="17"/>
+      <c r="E1" s="17"/>
+      <c r="F1" s="17"/>
+      <c r="G1" s="17"/>
+      <c r="H1" s="17"/>
+      <c r="I1" s="17"/>
+      <c r="J1" s="17"/>
+      <c r="K1" s="17"/>
     </row>
     <row r="2" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="16" t="s">
+      <c r="A2" s="19" t="s">
         <v>197</v>
       </c>
-      <c r="B2" s="16"/>
-      <c r="C2" s="16"/>
-      <c r="D2" s="16"/>
-      <c r="E2" s="16"/>
-      <c r="F2" s="16"/>
-      <c r="G2" s="16"/>
+      <c r="B2" s="19"/>
+      <c r="C2" s="19"/>
+      <c r="D2" s="19"/>
+      <c r="E2" s="19"/>
+      <c r="F2" s="19"/>
+      <c r="G2" s="19"/>
     </row>
     <row r="3" spans="1:11" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
@@ -6227,30 +6234,30 @@
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.5703125" defaultRowHeight="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:11" ht="19.350000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="15" t="s">
+      <c r="A1" s="17" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="15"/>
-      <c r="C1" s="15"/>
-      <c r="D1" s="15"/>
-      <c r="E1" s="15"/>
-      <c r="F1" s="15"/>
-      <c r="G1" s="15"/>
-      <c r="H1" s="15"/>
-      <c r="I1" s="15"/>
-      <c r="J1" s="15"/>
-      <c r="K1" s="15"/>
+      <c r="B1" s="17"/>
+      <c r="C1" s="17"/>
+      <c r="D1" s="17"/>
+      <c r="E1" s="17"/>
+      <c r="F1" s="17"/>
+      <c r="G1" s="17"/>
+      <c r="H1" s="17"/>
+      <c r="I1" s="17"/>
+      <c r="J1" s="17"/>
+      <c r="K1" s="17"/>
     </row>
     <row r="2" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="16" t="s">
+      <c r="A2" s="19" t="s">
         <v>196</v>
       </c>
-      <c r="B2" s="16"/>
-      <c r="C2" s="16"/>
-      <c r="D2" s="16"/>
-      <c r="E2" s="16"/>
-      <c r="F2" s="16"/>
-      <c r="G2" s="16"/>
+      <c r="B2" s="19"/>
+      <c r="C2" s="19"/>
+      <c r="D2" s="19"/>
+      <c r="E2" s="19"/>
+      <c r="F2" s="19"/>
+      <c r="G2" s="19"/>
     </row>
     <row r="3" spans="1:11" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
@@ -6313,30 +6320,30 @@
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.5703125" defaultRowHeight="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:11" ht="19.350000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="15" t="s">
+      <c r="A1" s="17" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="15"/>
-      <c r="C1" s="15"/>
-      <c r="D1" s="15"/>
-      <c r="E1" s="15"/>
-      <c r="F1" s="15"/>
-      <c r="G1" s="15"/>
-      <c r="H1" s="15"/>
-      <c r="I1" s="15"/>
-      <c r="J1" s="15"/>
-      <c r="K1" s="15"/>
+      <c r="B1" s="17"/>
+      <c r="C1" s="17"/>
+      <c r="D1" s="17"/>
+      <c r="E1" s="17"/>
+      <c r="F1" s="17"/>
+      <c r="G1" s="17"/>
+      <c r="H1" s="17"/>
+      <c r="I1" s="17"/>
+      <c r="J1" s="17"/>
+      <c r="K1" s="17"/>
     </row>
     <row r="2" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="16" t="s">
+      <c r="A2" s="19" t="s">
         <v>195</v>
       </c>
-      <c r="B2" s="16"/>
-      <c r="C2" s="16"/>
-      <c r="D2" s="16"/>
-      <c r="E2" s="16"/>
-      <c r="F2" s="16"/>
-      <c r="G2" s="16"/>
+      <c r="B2" s="19"/>
+      <c r="C2" s="19"/>
+      <c r="D2" s="19"/>
+      <c r="E2" s="19"/>
+      <c r="F2" s="19"/>
+      <c r="G2" s="19"/>
     </row>
     <row r="3" spans="1:11" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
@@ -6399,30 +6406,30 @@
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.5703125" defaultRowHeight="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:11" ht="19.350000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="15" t="s">
+      <c r="A1" s="17" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="15"/>
-      <c r="C1" s="15"/>
-      <c r="D1" s="15"/>
-      <c r="E1" s="15"/>
-      <c r="F1" s="15"/>
-      <c r="G1" s="15"/>
-      <c r="H1" s="15"/>
-      <c r="I1" s="15"/>
-      <c r="J1" s="15"/>
-      <c r="K1" s="15"/>
+      <c r="B1" s="17"/>
+      <c r="C1" s="17"/>
+      <c r="D1" s="17"/>
+      <c r="E1" s="17"/>
+      <c r="F1" s="17"/>
+      <c r="G1" s="17"/>
+      <c r="H1" s="17"/>
+      <c r="I1" s="17"/>
+      <c r="J1" s="17"/>
+      <c r="K1" s="17"/>
     </row>
     <row r="2" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="16" t="s">
+      <c r="A2" s="19" t="s">
         <v>194</v>
       </c>
-      <c r="B2" s="16"/>
-      <c r="C2" s="16"/>
-      <c r="D2" s="16"/>
-      <c r="E2" s="16"/>
-      <c r="F2" s="16"/>
-      <c r="G2" s="16"/>
+      <c r="B2" s="19"/>
+      <c r="C2" s="19"/>
+      <c r="D2" s="19"/>
+      <c r="E2" s="19"/>
+      <c r="F2" s="19"/>
+      <c r="G2" s="19"/>
     </row>
     <row r="3" spans="1:11" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
@@ -6485,30 +6492,30 @@
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.5703125" defaultRowHeight="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:11" ht="19.350000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="15" t="s">
+      <c r="A1" s="17" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="15"/>
-      <c r="C1" s="15"/>
-      <c r="D1" s="15"/>
-      <c r="E1" s="15"/>
-      <c r="F1" s="15"/>
-      <c r="G1" s="15"/>
-      <c r="H1" s="15"/>
-      <c r="I1" s="15"/>
-      <c r="J1" s="15"/>
-      <c r="K1" s="15"/>
+      <c r="B1" s="17"/>
+      <c r="C1" s="17"/>
+      <c r="D1" s="17"/>
+      <c r="E1" s="17"/>
+      <c r="F1" s="17"/>
+      <c r="G1" s="17"/>
+      <c r="H1" s="17"/>
+      <c r="I1" s="17"/>
+      <c r="J1" s="17"/>
+      <c r="K1" s="17"/>
     </row>
     <row r="2" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="16" t="s">
+      <c r="A2" s="19" t="s">
         <v>190</v>
       </c>
-      <c r="B2" s="16"/>
-      <c r="C2" s="16"/>
-      <c r="D2" s="16"/>
-      <c r="E2" s="16"/>
-      <c r="F2" s="16"/>
-      <c r="G2" s="16"/>
+      <c r="B2" s="19"/>
+      <c r="C2" s="19"/>
+      <c r="D2" s="19"/>
+      <c r="E2" s="19"/>
+      <c r="F2" s="19"/>
+      <c r="G2" s="19"/>
     </row>
     <row r="3" spans="1:11" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">

</xml_diff>

<commit_message>
test: integration TC 61, 62, 64, 72, 73
</commit_message>
<xml_diff>
--- a/docs/tests/breco - cas de test.xlsx
+++ b/docs/tests/breco - cas de test.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\wamp\www\breco_v2_0_0\docs\tests\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DECB4F73-BE77-4725-9CC8-401017F498B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2B63C162-626F-46EC-A219-EC68C4F5A701}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Story1 - Auth" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1184" uniqueCount="421">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1188" uniqueCount="421">
   <si>
     <t>Plan de test Breco, cas de test</t>
   </si>
@@ -1977,7 +1977,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -2040,15 +2040,6 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2177,6 +2168,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:U103"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.5703125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
@@ -2258,7 +2250,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:11" ht="14.25" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:11" ht="14.25" hidden="1" x14ac:dyDescent="0.25">
       <c r="A4" s="16" t="s">
         <v>9</v>
       </c>
@@ -2293,7 +2285,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:11" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:11" ht="25.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A5" s="16" t="s">
         <v>15</v>
       </c>
@@ -2328,7 +2320,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="6" spans="1:11" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:11" ht="25.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A6" s="16" t="s">
         <v>18</v>
       </c>
@@ -2363,7 +2355,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="7" spans="1:11" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:11" ht="25.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A7" s="16" t="s">
         <v>21</v>
       </c>
@@ -2398,7 +2390,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="8" spans="1:11" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:11" ht="25.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A8" s="16" t="s">
         <v>27</v>
       </c>
@@ -2433,7 +2425,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="9" spans="1:11" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:11" ht="25.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A9" s="16" t="s">
         <v>287</v>
       </c>
@@ -2468,7 +2460,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="10" spans="1:11" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:11" ht="25.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A10" s="16" t="s">
         <v>288</v>
       </c>
@@ -2503,7 +2495,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="11" spans="1:11" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:11" ht="25.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A11" s="16" t="s">
         <v>289</v>
       </c>
@@ -2538,7 +2530,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:11" ht="14.25" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:11" ht="14.25" hidden="1" x14ac:dyDescent="0.25">
       <c r="A12" s="16" t="s">
         <v>33</v>
       </c>
@@ -2573,7 +2565,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="13" spans="1:11" ht="14.25" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:11" ht="14.25" hidden="1" x14ac:dyDescent="0.25">
       <c r="A13" s="16" t="s">
         <v>36</v>
       </c>
@@ -2608,7 +2600,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="14" spans="1:11" ht="14.25" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:11" ht="14.25" hidden="1" x14ac:dyDescent="0.25">
       <c r="A14" s="16" t="s">
         <v>39</v>
       </c>
@@ -2643,7 +2635,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="15" spans="1:11" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:11" ht="25.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A15" s="16" t="s">
         <v>43</v>
       </c>
@@ -2678,7 +2670,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="16" spans="1:11" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:11" ht="25.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A16" s="16" t="s">
         <v>46</v>
       </c>
@@ -2713,7 +2705,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="17" spans="1:11" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:11" ht="25.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A17" s="16" t="s">
         <v>49</v>
       </c>
@@ -2748,7 +2740,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="18" spans="1:11" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:11" ht="25.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A18" s="16" t="s">
         <v>51</v>
       </c>
@@ -2773,7 +2765,7 @@
       <c r="H18" s="11" t="s">
         <v>53</v>
       </c>
-      <c r="I18" s="21" t="s">
+      <c r="I18" s="8" t="s">
         <v>54</v>
       </c>
       <c r="J18" s="3" t="s">
@@ -2783,7 +2775,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="19" spans="1:11" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:11" ht="25.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A19" s="16" t="s">
         <v>55</v>
       </c>
@@ -2818,7 +2810,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="20" spans="1:11" ht="38.25" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:11" ht="38.25" hidden="1" x14ac:dyDescent="0.25">
       <c r="A20" s="16" t="s">
         <v>58</v>
       </c>
@@ -2853,7 +2845,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="21" spans="1:11" ht="14.25" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:11" ht="14.25" hidden="1" x14ac:dyDescent="0.25">
       <c r="A21" s="16" t="s">
         <v>61</v>
       </c>
@@ -2888,7 +2880,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="22" spans="1:11" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:11" ht="25.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A22" s="16" t="s">
         <v>65</v>
       </c>
@@ -2923,7 +2915,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="23" spans="1:11" ht="14.25" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:11" ht="14.25" hidden="1" x14ac:dyDescent="0.25">
       <c r="A23" s="16" t="s">
         <v>68</v>
       </c>
@@ -2958,7 +2950,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="24" spans="1:11" ht="14.25" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:11" ht="14.25" hidden="1" x14ac:dyDescent="0.25">
       <c r="A24" s="16" t="s">
         <v>71</v>
       </c>
@@ -2993,7 +2985,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="25" spans="1:11" ht="14.25" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:11" ht="14.25" hidden="1" x14ac:dyDescent="0.25">
       <c r="A25" s="16" t="s">
         <v>74</v>
       </c>
@@ -3028,7 +3020,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="26" spans="1:11" ht="14.25" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:11" ht="14.25" hidden="1" x14ac:dyDescent="0.25">
       <c r="A26" s="16" t="s">
         <v>77</v>
       </c>
@@ -3063,7 +3055,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="27" spans="1:11" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:11" ht="25.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A27" s="16" t="s">
         <v>80</v>
       </c>
@@ -3098,7 +3090,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="28" spans="1:11" ht="38.25" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:11" ht="38.25" hidden="1" x14ac:dyDescent="0.25">
       <c r="A28" s="16" t="s">
         <v>83</v>
       </c>
@@ -3133,7 +3125,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="29" spans="1:11" ht="14.25" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:11" ht="14.25" hidden="1" x14ac:dyDescent="0.25">
       <c r="A29" s="16" t="s">
         <v>86</v>
       </c>
@@ -3168,7 +3160,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="30" spans="1:11" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:11" ht="25.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A30" s="16" t="s">
         <v>90</v>
       </c>
@@ -3203,7 +3195,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="31" spans="1:11" ht="14.25" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:11" ht="14.25" hidden="1" x14ac:dyDescent="0.25">
       <c r="A31" s="16" t="s">
         <v>93</v>
       </c>
@@ -3238,7 +3230,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="32" spans="1:11" ht="14.25" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:11" ht="14.25" hidden="1" x14ac:dyDescent="0.25">
       <c r="A32" s="16" t="s">
         <v>96</v>
       </c>
@@ -3273,7 +3265,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="33" spans="1:11" ht="14.25" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:11" ht="14.25" hidden="1" x14ac:dyDescent="0.25">
       <c r="A33" s="16" t="s">
         <v>98</v>
       </c>
@@ -3308,7 +3300,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="34" spans="1:11" ht="14.25" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:11" ht="14.25" hidden="1" x14ac:dyDescent="0.25">
       <c r="A34" s="16" t="s">
         <v>100</v>
       </c>
@@ -3343,7 +3335,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="35" spans="1:11" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:11" ht="25.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A35" s="16" t="s">
         <v>102</v>
       </c>
@@ -3368,7 +3360,7 @@
       <c r="H35" s="9" t="s">
         <v>104</v>
       </c>
-      <c r="I35" s="21" t="s">
+      <c r="I35" s="8" t="s">
         <v>246</v>
       </c>
       <c r="J35" s="3" t="s">
@@ -3378,7 +3370,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="36" spans="1:11" ht="14.25" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:11" ht="14.25" hidden="1" x14ac:dyDescent="0.25">
       <c r="A36" s="16" t="s">
         <v>278</v>
       </c>
@@ -3403,7 +3395,7 @@
       <c r="H36" s="9" t="s">
         <v>106</v>
       </c>
-      <c r="I36" s="20" t="s">
+      <c r="I36" s="10" t="s">
         <v>107</v>
       </c>
       <c r="J36" s="3" t="s">
@@ -3413,7 +3405,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="37" spans="1:11" ht="14.25" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:11" ht="14.25" hidden="1" x14ac:dyDescent="0.25">
       <c r="A37" s="16" t="s">
         <v>279</v>
       </c>
@@ -3448,7 +3440,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="38" spans="1:11" ht="14.25" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:11" ht="14.25" hidden="1" x14ac:dyDescent="0.25">
       <c r="A38" s="16" t="s">
         <v>280</v>
       </c>
@@ -3483,7 +3475,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="39" spans="1:11" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:11" ht="25.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A39" s="16" t="s">
         <v>108</v>
       </c>
@@ -3518,7 +3510,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="40" spans="1:11" ht="15" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:11" ht="15" hidden="1" x14ac:dyDescent="0.25">
       <c r="A40" s="16" t="s">
         <v>277</v>
       </c>
@@ -3543,7 +3535,7 @@
       <c r="H40" s="12" t="s">
         <v>240</v>
       </c>
-      <c r="I40" s="21" t="s">
+      <c r="I40" s="8" t="s">
         <v>247</v>
       </c>
       <c r="J40" s="3" t="s">
@@ -3553,7 +3545,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="41" spans="1:11" ht="15" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:11" ht="15" hidden="1" x14ac:dyDescent="0.25">
       <c r="A41" s="16" t="s">
         <v>276</v>
       </c>
@@ -3588,7 +3580,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="42" spans="1:11" ht="15" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:11" ht="15" hidden="1" x14ac:dyDescent="0.25">
       <c r="A42" s="16" t="s">
         <v>275</v>
       </c>
@@ -3623,7 +3615,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="43" spans="1:11" ht="15" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:11" ht="15" hidden="1" x14ac:dyDescent="0.25">
       <c r="A43" s="16" t="s">
         <v>110</v>
       </c>
@@ -3658,7 +3650,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="44" spans="1:11" ht="15" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:11" ht="15" hidden="1" x14ac:dyDescent="0.25">
       <c r="A44" s="16" t="s">
         <v>114</v>
       </c>
@@ -3683,7 +3675,7 @@
       <c r="H44" s="12" t="s">
         <v>116</v>
       </c>
-      <c r="I44" s="20" t="s">
+      <c r="I44" s="10" t="s">
         <v>113</v>
       </c>
       <c r="J44" s="3" t="s">
@@ -3693,7 +3685,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="45" spans="1:11" ht="15" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:11" ht="15" hidden="1" x14ac:dyDescent="0.25">
       <c r="A45" s="16" t="s">
         <v>117</v>
       </c>
@@ -3728,7 +3720,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="46" spans="1:11" ht="15" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:11" ht="15" hidden="1" x14ac:dyDescent="0.25">
       <c r="A46" s="16" t="s">
         <v>118</v>
       </c>
@@ -3763,7 +3755,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="47" spans="1:11" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:11" ht="25.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A47" s="16" t="s">
         <v>122</v>
       </c>
@@ -3798,7 +3790,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="48" spans="1:11" ht="60" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:11" ht="60" hidden="1" x14ac:dyDescent="0.25">
       <c r="A48" s="16" t="s">
         <v>124</v>
       </c>
@@ -3833,7 +3825,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="49" spans="1:21" ht="15" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:21" ht="15" hidden="1" x14ac:dyDescent="0.25">
       <c r="A49" s="16" t="s">
         <v>127</v>
       </c>
@@ -3868,7 +3860,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="50" spans="1:21" ht="15" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:21" ht="15" hidden="1" x14ac:dyDescent="0.25">
       <c r="A50" s="16" t="s">
         <v>129</v>
       </c>
@@ -3887,13 +3879,13 @@
       <c r="F50" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="G50" s="21" t="s">
+      <c r="G50" s="8" t="s">
         <v>249</v>
       </c>
-      <c r="H50" s="22" t="s">
+      <c r="H50" s="12" t="s">
         <v>134</v>
       </c>
-      <c r="I50" s="21" t="s">
+      <c r="I50" s="8" t="s">
         <v>123</v>
       </c>
       <c r="J50" s="3" t="s">
@@ -3903,7 +3895,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="51" spans="1:21" ht="15" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:21" ht="15" hidden="1" x14ac:dyDescent="0.25">
       <c r="A51" s="16" t="s">
         <v>133</v>
       </c>
@@ -3922,13 +3914,13 @@
       <c r="F51" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="G51" s="20" t="s">
+      <c r="G51" s="10" t="s">
         <v>136</v>
       </c>
-      <c r="H51" s="22" t="s">
+      <c r="H51" s="12" t="s">
         <v>137</v>
       </c>
-      <c r="I51" s="20" t="s">
+      <c r="I51" s="10" t="s">
         <v>138</v>
       </c>
       <c r="J51" s="3" t="s">
@@ -3938,7 +3930,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="52" spans="1:21" ht="40.5" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:21" ht="40.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A52" s="16" t="s">
         <v>135</v>
       </c>
@@ -3957,10 +3949,10 @@
       <c r="F52" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="G52" s="20" t="s">
+      <c r="G52" s="10" t="s">
         <v>140</v>
       </c>
-      <c r="H52" s="22" t="s">
+      <c r="H52" s="12" t="s">
         <v>248</v>
       </c>
       <c r="I52" s="3" t="s">
@@ -3973,7 +3965,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="53" spans="1:21" ht="15" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:21" ht="15" hidden="1" x14ac:dyDescent="0.25">
       <c r="A53" s="16" t="s">
         <v>139</v>
       </c>
@@ -3992,13 +3984,13 @@
       <c r="F53" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="G53" s="20" t="s">
+      <c r="G53" s="10" t="s">
         <v>142</v>
       </c>
-      <c r="H53" s="22" t="s">
+      <c r="H53" s="12" t="s">
         <v>252</v>
       </c>
-      <c r="I53" s="20" t="s">
+      <c r="I53" s="10" t="s">
         <v>143</v>
       </c>
       <c r="J53" s="3" t="s">
@@ -4008,7 +4000,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="54" spans="1:21" ht="15" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:21" ht="15" hidden="1" x14ac:dyDescent="0.25">
       <c r="A54" s="16" t="s">
         <v>141</v>
       </c>
@@ -4027,13 +4019,13 @@
       <c r="F54" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="G54" s="21" t="s">
+      <c r="G54" s="8" t="s">
         <v>250</v>
       </c>
-      <c r="H54" s="22" t="s">
+      <c r="H54" s="12" t="s">
         <v>255</v>
       </c>
-      <c r="I54" s="21" t="s">
+      <c r="I54" s="8" t="s">
         <v>123</v>
       </c>
       <c r="J54" s="3" t="s">
@@ -4043,7 +4035,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="55" spans="1:21" ht="15" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:21" ht="15" hidden="1" x14ac:dyDescent="0.25">
       <c r="A55" s="16" t="s">
         <v>144</v>
       </c>
@@ -4062,13 +4054,13 @@
       <c r="F55" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="G55" s="20" t="s">
+      <c r="G55" s="10" t="s">
         <v>146</v>
       </c>
-      <c r="H55" s="22" t="s">
+      <c r="H55" s="12" t="s">
         <v>147</v>
       </c>
-      <c r="I55" s="20" t="s">
+      <c r="I55" s="10" t="s">
         <v>148</v>
       </c>
       <c r="J55" s="3" t="s">
@@ -4078,7 +4070,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="56" spans="1:21" ht="27.75" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:21" ht="27.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A56" s="16" t="s">
         <v>145</v>
       </c>
@@ -4097,10 +4089,10 @@
       <c r="F56" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="G56" s="20" t="s">
+      <c r="G56" s="10" t="s">
         <v>150</v>
       </c>
-      <c r="H56" s="22" t="s">
+      <c r="H56" s="12" t="s">
         <v>253</v>
       </c>
       <c r="I56" s="3" t="s">
@@ -4113,7 +4105,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="57" spans="1:21" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:21" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A57" s="16" t="s">
         <v>149</v>
       </c>
@@ -4132,13 +4124,13 @@
       <c r="F57" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="G57" s="21" t="s">
+      <c r="G57" s="8" t="s">
         <v>152</v>
       </c>
-      <c r="H57" s="22" t="s">
+      <c r="H57" s="12" t="s">
         <v>153</v>
       </c>
-      <c r="I57" s="20" t="s">
+      <c r="I57" s="10" t="s">
         <v>154</v>
       </c>
       <c r="J57" s="3" t="s">
@@ -4148,7 +4140,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="58" spans="1:21" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:21" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A58" s="16" t="s">
         <v>151</v>
       </c>
@@ -4167,13 +4159,13 @@
       <c r="F58" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="G58" s="21" t="s">
+      <c r="G58" s="8" t="s">
         <v>156</v>
       </c>
-      <c r="H58" s="22" t="s">
+      <c r="H58" s="12" t="s">
         <v>256</v>
       </c>
-      <c r="I58" s="21" t="s">
+      <c r="I58" s="8" t="s">
         <v>123</v>
       </c>
       <c r="J58" s="3" t="s">
@@ -4183,7 +4175,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="59" spans="1:21" ht="15" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:21" ht="15" hidden="1" x14ac:dyDescent="0.25">
       <c r="A59" s="16" t="s">
         <v>155</v>
       </c>
@@ -4202,10 +4194,10 @@
       <c r="F59" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="G59" s="21" t="s">
+      <c r="G59" s="8" t="s">
         <v>158</v>
       </c>
-      <c r="H59" s="22" t="s">
+      <c r="H59" s="12" t="s">
         <v>159</v>
       </c>
       <c r="I59" s="3" t="s">
@@ -4218,7 +4210,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="60" spans="1:21" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:21" ht="25.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A60" s="16" t="s">
         <v>157</v>
       </c>
@@ -4237,10 +4229,10 @@
       <c r="F60" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="G60" s="21" t="s">
+      <c r="G60" s="8" t="s">
         <v>161</v>
       </c>
-      <c r="H60" s="22" t="s">
+      <c r="H60" s="12" t="s">
         <v>162</v>
       </c>
       <c r="I60" s="3" t="s">
@@ -4253,7 +4245,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="61" spans="1:21" ht="15" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:21" ht="15" hidden="1" x14ac:dyDescent="0.25">
       <c r="A61" s="16" t="s">
         <v>160</v>
       </c>
@@ -4272,13 +4264,13 @@
       <c r="F61" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="G61" s="20" t="s">
+      <c r="G61" s="10" t="s">
         <v>164</v>
       </c>
-      <c r="H61" s="22" t="s">
+      <c r="H61" s="12" t="s">
         <v>165</v>
       </c>
-      <c r="I61" s="20" t="s">
+      <c r="I61" s="10" t="s">
         <v>166</v>
       </c>
       <c r="J61" s="3" t="s">
@@ -4659,7 +4651,7 @@
       </c>
     </row>
     <row r="72" spans="1:21" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="A72" s="3" t="s">
+      <c r="A72" s="16" t="s">
         <v>180</v>
       </c>
       <c r="B72" s="3" t="s">
@@ -4671,7 +4663,9 @@
       <c r="D72" s="3" t="s">
         <v>227</v>
       </c>
-      <c r="E72" s="3"/>
+      <c r="E72" s="3" t="s">
+        <v>412</v>
+      </c>
       <c r="F72" s="3" t="s">
         <v>415</v>
       </c>
@@ -4692,7 +4686,7 @@
       </c>
     </row>
     <row r="73" spans="1:21" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="A73" s="3" t="s">
+      <c r="A73" s="16" t="s">
         <v>181</v>
       </c>
       <c r="B73" s="3" t="s">
@@ -4704,7 +4698,9 @@
       <c r="D73" s="3" t="s">
         <v>227</v>
       </c>
-      <c r="E73" s="3"/>
+      <c r="E73" s="3" t="s">
+        <v>412</v>
+      </c>
       <c r="F73" s="3" t="s">
         <v>415</v>
       </c>
@@ -4757,18 +4753,18 @@
         <v>353</v>
       </c>
     </row>
-    <row r="75" spans="1:21" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:21" ht="25.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A75" s="3" t="s">
         <v>183</v>
       </c>
       <c r="B75" s="3" t="s">
-        <v>218</v>
+        <v>335</v>
       </c>
       <c r="C75" s="3" t="s">
-        <v>226</v>
+        <v>336</v>
       </c>
       <c r="D75" s="3" t="s">
-        <v>227</v>
+        <v>222</v>
       </c>
       <c r="E75" s="3"/>
       <c r="F75" s="3" t="s">
@@ -4790,7 +4786,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="76" spans="1:21" ht="14.25" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:21" ht="14.25" hidden="1" x14ac:dyDescent="0.25">
       <c r="A76" s="3" t="s">
         <v>186</v>
       </c>
@@ -4823,7 +4819,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="77" spans="1:21" ht="14.25" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:21" ht="14.25" hidden="1" x14ac:dyDescent="0.25">
       <c r="A77" s="3" t="s">
         <v>324</v>
       </c>
@@ -4856,7 +4852,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="78" spans="1:21" ht="14.25" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:21" ht="14.25" hidden="1" x14ac:dyDescent="0.25">
       <c r="A78" s="3" t="s">
         <v>328</v>
       </c>
@@ -4889,7 +4885,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="79" spans="1:21" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:21" ht="25.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A79" s="3" t="s">
         <v>337</v>
       </c>
@@ -4922,7 +4918,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="80" spans="1:21" ht="14.25" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:21" ht="14.25" hidden="1" x14ac:dyDescent="0.25">
       <c r="A80" s="3" t="s">
         <v>341</v>
       </c>
@@ -4955,7 +4951,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="81" spans="1:11" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:11" ht="25.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A81" s="3" t="s">
         <v>345</v>
       </c>
@@ -4988,7 +4984,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="82" spans="1:11" ht="14.25" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:11" ht="14.25" hidden="1" x14ac:dyDescent="0.25">
       <c r="A82" s="3" t="s">
         <v>348</v>
       </c>
@@ -5022,7 +5018,7 @@
       </c>
     </row>
     <row r="83" spans="1:11" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="A83" s="3" t="s">
+      <c r="A83" s="16" t="s">
         <v>354</v>
       </c>
       <c r="B83" s="3" t="s">
@@ -5034,7 +5030,9 @@
       <c r="D83" s="3" t="s">
         <v>227</v>
       </c>
-      <c r="E83" s="3"/>
+      <c r="E83" s="3" t="s">
+        <v>412</v>
+      </c>
       <c r="F83" s="3" t="s">
         <v>10</v>
       </c>
@@ -5055,7 +5053,7 @@
       </c>
     </row>
     <row r="84" spans="1:11" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="A84" s="3" t="s">
+      <c r="A84" s="16" t="s">
         <v>355</v>
       </c>
       <c r="B84" s="3" t="s">
@@ -5067,7 +5065,9 @@
       <c r="D84" s="3" t="s">
         <v>227</v>
       </c>
-      <c r="E84" s="3"/>
+      <c r="E84" s="3" t="s">
+        <v>412</v>
+      </c>
       <c r="F84" s="3" t="s">
         <v>10</v>
       </c>
@@ -5258,7 +5258,7 @@
         <v>353</v>
       </c>
     </row>
-    <row r="90" spans="1:11" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:11" ht="25.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A90" s="3" t="s">
         <v>384</v>
       </c>
@@ -5291,7 +5291,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="91" spans="1:11" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:11" ht="25.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A91" s="3" t="s">
         <v>385</v>
       </c>
@@ -5324,7 +5324,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="92" spans="1:11" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:11" ht="25.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A92" s="3" t="s">
         <v>386</v>
       </c>
@@ -5502,6 +5502,11 @@
     </row>
   </sheetData>
   <autoFilter ref="A3:U92" xr:uid="{00000000-0001-0000-0000-000000000000}">
+    <filterColumn colId="1">
+      <filters>
+        <filter val="Intégration"/>
+      </filters>
+    </filterColumn>
     <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A4:U92">
       <sortCondition ref="A3:A92"/>
     </sortState>
@@ -6011,7 +6016,7 @@
     <hyperlink ref="H6" r:id="rId2" display="search?q=@#&lt;?&amp;+!&amp;limit=10" xr:uid="{66C64D42-70A2-4593-9DF3-48F475D7EB46}"/>
   </hyperlinks>
   <pageMargins left="0.78749999999999998" right="0.78749999999999998" top="1.05277777777778" bottom="1.05277777777778" header="0.78749999999999998" footer="0.78749999999999998"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId3"/>
   <headerFooter>
     <oddHeader>&amp;C&amp;"Times New Roman,Normal"&amp;12&amp;Kffffff&amp;A</oddHeader>
     <oddFooter>&amp;C&amp;"Times New Roman,Normal"&amp;12&amp;KffffffPage &amp;P</oddFooter>

</xml_diff>

<commit_message>
test(auth): add PHPUnit test TC-63 and implement login rate limiting
</commit_message>
<xml_diff>
--- a/docs/tests/breco - cas de test.xlsx
+++ b/docs/tests/breco - cas de test.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\wamp\www\breco_v2_0_0\docs\tests\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2B63C162-626F-46EC-A219-EC68C4F5A701}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{49B79A27-3673-471C-A768-9512C41D62D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -4721,7 +4721,7 @@
       </c>
     </row>
     <row r="74" spans="1:21" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="A74" s="3" t="s">
+      <c r="A74" s="16" t="s">
         <v>182</v>
       </c>
       <c r="B74" s="3" t="s">
@@ -4749,8 +4749,8 @@
       <c r="J74" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="K74" s="15" t="s">
-        <v>353</v>
+      <c r="K74" s="4" t="s">
+        <v>14</v>
       </c>
     </row>
     <row r="75" spans="1:21" ht="25.5" hidden="1" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
test(auth): implement account lockout (TC-75) with locked_at migration and AccountLockedException
</commit_message>
<xml_diff>
--- a/docs/tests/breco - cas de test.xlsx
+++ b/docs/tests/breco - cas de test.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\wamp\www\breco_v2_0_0\docs\tests\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{49B79A27-3673-471C-A768-9512C41D62D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B17CE178-4ECD-4ED5-B495-94E583CEA5C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1188" uniqueCount="421">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1190" uniqueCount="421">
   <si>
     <t>Plan de test Breco, cas de test</t>
   </si>
@@ -4733,7 +4733,9 @@
       <c r="D74" s="3" t="s">
         <v>227</v>
       </c>
-      <c r="E74" s="3"/>
+      <c r="E74" s="3" t="s">
+        <v>412</v>
+      </c>
       <c r="F74" s="3" t="s">
         <v>168</v>
       </c>
@@ -5123,7 +5125,7 @@
       </c>
     </row>
     <row r="86" spans="1:11" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="A86" s="3" t="s">
+      <c r="A86" s="16" t="s">
         <v>357</v>
       </c>
       <c r="B86" s="3" t="s">
@@ -5135,7 +5137,9 @@
       <c r="D86" s="3" t="s">
         <v>227</v>
       </c>
-      <c r="E86" s="3"/>
+      <c r="E86" s="3" t="s">
+        <v>412</v>
+      </c>
       <c r="F86" s="3" t="s">
         <v>168</v>
       </c>
@@ -5151,8 +5155,8 @@
       <c r="J86" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="K86" s="15" t="s">
-        <v>353</v>
+      <c r="K86" s="4" t="s">
+        <v>14</v>
       </c>
     </row>
     <row r="87" spans="1:11" ht="14.25" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
test: UI - TC 64, 65, 66, 67, 68
</commit_message>
<xml_diff>
--- a/docs/tests/breco - cas de test.xlsx
+++ b/docs/tests/breco - cas de test.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\wamp\www\breco_v2_0_0\docs\tests\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B17CE178-4ECD-4ED5-B495-94E583CEA5C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8B4A3F02-CE33-4DAF-A5F3-F8F7C531FE42}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1190" uniqueCount="421">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1196" uniqueCount="423">
   <si>
     <t>Plan de test Breco, cas de test</t>
   </si>
@@ -1548,9 +1548,6 @@
     <t>Affichage messages d'erreur Zod en UI</t>
   </si>
   <si>
-    <t>email = "" soumis via formulaire</t>
-  </si>
-  <si>
     <t>Message d'erreur affiché dans le DOM</t>
   </si>
   <si>
@@ -1590,9 +1587,6 @@
     <t>Tous champs étape 1 valides</t>
   </si>
   <si>
-    <t>Étape 2 affichée, barre de progression à 50%</t>
-  </si>
-  <si>
     <t>TC-70</t>
   </si>
   <si>
@@ -1819,6 +1813,18 @@
   </si>
   <si>
     <t>Autocomplétion non déclenchée, liste vide</t>
+  </si>
+  <si>
+    <t>(Rate limiting global à implémenter au niveau middleware CakePHP, hors périmètre AuthService. Nécessite un système de cache, Redis ou CakePHP Cache, pour comptabiliser les requêtes par IP. Non prioritaire pour la v1)</t>
+  </si>
+  <si>
+    <t>RegisterPage.spec.ts</t>
+  </si>
+  <si>
+    <t>E-mail vide soumis via formulaire</t>
+  </si>
+  <si>
+    <t>Étape 2 affichée</t>
   </si>
 </sst>
 </file>
@@ -2168,7 +2174,6 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <sheetPr filterMode="1"/>
   <dimension ref="A1:U103"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.5703125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
@@ -2229,7 +2234,7 @@
         <v>220</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>396</v>
+        <v>394</v>
       </c>
       <c r="F3" s="1" t="s">
         <v>3</v>
@@ -2250,7 +2255,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:11" ht="14.25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:11" ht="14.25" x14ac:dyDescent="0.25">
       <c r="A4" s="16" t="s">
         <v>9</v>
       </c>
@@ -2264,7 +2269,7 @@
         <v>222</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
       <c r="F4" s="3" t="s">
         <v>10</v>
@@ -2285,7 +2290,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:11" ht="25.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:11" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A5" s="16" t="s">
         <v>15</v>
       </c>
@@ -2299,7 +2304,7 @@
         <v>222</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
       <c r="F5" s="3" t="s">
         <v>10</v>
@@ -2320,7 +2325,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="6" spans="1:11" ht="25.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:11" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A6" s="16" t="s">
         <v>18</v>
       </c>
@@ -2334,7 +2339,7 @@
         <v>222</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
       <c r="F6" s="3" t="s">
         <v>10</v>
@@ -2355,7 +2360,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="7" spans="1:11" ht="25.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:11" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A7" s="16" t="s">
         <v>21</v>
       </c>
@@ -2369,7 +2374,7 @@
         <v>222</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
       <c r="F7" s="3" t="s">
         <v>10</v>
@@ -2390,7 +2395,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="8" spans="1:11" ht="25.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:11" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A8" s="16" t="s">
         <v>27</v>
       </c>
@@ -2404,7 +2409,7 @@
         <v>222</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
       <c r="F8" s="3" t="s">
         <v>10</v>
@@ -2425,7 +2430,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="9" spans="1:11" ht="25.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:11" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A9" s="16" t="s">
         <v>287</v>
       </c>
@@ -2439,7 +2444,7 @@
         <v>222</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
       <c r="F9" s="3" t="s">
         <v>10</v>
@@ -2460,7 +2465,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="10" spans="1:11" ht="25.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:11" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A10" s="16" t="s">
         <v>288</v>
       </c>
@@ -2474,7 +2479,7 @@
         <v>222</v>
       </c>
       <c r="E10" s="3" t="s">
-        <v>399</v>
+        <v>397</v>
       </c>
       <c r="F10" s="3" t="s">
         <v>10</v>
@@ -2495,7 +2500,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="11" spans="1:11" ht="25.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:11" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A11" s="16" t="s">
         <v>289</v>
       </c>
@@ -2509,7 +2514,7 @@
         <v>222</v>
       </c>
       <c r="E11" s="3" t="s">
-        <v>399</v>
+        <v>397</v>
       </c>
       <c r="F11" s="3" t="s">
         <v>10</v>
@@ -2530,7 +2535,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:11" ht="14.25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:11" ht="14.25" x14ac:dyDescent="0.25">
       <c r="A12" s="16" t="s">
         <v>33</v>
       </c>
@@ -2544,7 +2549,7 @@
         <v>222</v>
       </c>
       <c r="E12" s="3" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
       <c r="F12" s="3" t="s">
         <v>10</v>
@@ -2565,7 +2570,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="13" spans="1:11" ht="14.25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:11" ht="14.25" x14ac:dyDescent="0.25">
       <c r="A13" s="16" t="s">
         <v>36</v>
       </c>
@@ -2579,7 +2584,7 @@
         <v>222</v>
       </c>
       <c r="E13" s="3" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
       <c r="F13" s="3" t="s">
         <v>10</v>
@@ -2600,7 +2605,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="14" spans="1:11" ht="14.25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:11" ht="14.25" x14ac:dyDescent="0.25">
       <c r="A14" s="16" t="s">
         <v>39</v>
       </c>
@@ -2614,7 +2619,7 @@
         <v>222</v>
       </c>
       <c r="E14" s="3" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
       <c r="F14" s="3" t="s">
         <v>10</v>
@@ -2635,7 +2640,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="15" spans="1:11" ht="25.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:11" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A15" s="16" t="s">
         <v>43</v>
       </c>
@@ -2649,7 +2654,7 @@
         <v>222</v>
       </c>
       <c r="E15" s="3" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
       <c r="F15" s="3" t="s">
         <v>10</v>
@@ -2670,7 +2675,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="16" spans="1:11" ht="25.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:11" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A16" s="16" t="s">
         <v>46</v>
       </c>
@@ -2684,7 +2689,7 @@
         <v>222</v>
       </c>
       <c r="E16" s="3" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
       <c r="F16" s="3" t="s">
         <v>10</v>
@@ -2705,7 +2710,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="17" spans="1:11" ht="25.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:11" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A17" s="16" t="s">
         <v>49</v>
       </c>
@@ -2719,7 +2724,7 @@
         <v>222</v>
       </c>
       <c r="E17" s="3" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
       <c r="F17" s="3" t="s">
         <v>10</v>
@@ -2740,7 +2745,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="18" spans="1:11" ht="25.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:11" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A18" s="16" t="s">
         <v>51</v>
       </c>
@@ -2754,7 +2759,7 @@
         <v>222</v>
       </c>
       <c r="E18" s="3" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
       <c r="F18" s="3" t="s">
         <v>10</v>
@@ -2775,7 +2780,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="19" spans="1:11" ht="25.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:11" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A19" s="16" t="s">
         <v>55</v>
       </c>
@@ -2789,7 +2794,7 @@
         <v>222</v>
       </c>
       <c r="E19" s="3" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
       <c r="F19" s="3" t="s">
         <v>10</v>
@@ -2810,7 +2815,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="20" spans="1:11" ht="38.25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:11" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A20" s="16" t="s">
         <v>58</v>
       </c>
@@ -2824,7 +2829,7 @@
         <v>222</v>
       </c>
       <c r="E20" s="3" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
       <c r="F20" s="3" t="s">
         <v>10</v>
@@ -2845,7 +2850,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="21" spans="1:11" ht="14.25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:11" ht="14.25" x14ac:dyDescent="0.25">
       <c r="A21" s="16" t="s">
         <v>61</v>
       </c>
@@ -2859,7 +2864,7 @@
         <v>222</v>
       </c>
       <c r="E21" s="3" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
       <c r="F21" s="3" t="s">
         <v>10</v>
@@ -2880,7 +2885,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="22" spans="1:11" ht="25.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:11" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A22" s="16" t="s">
         <v>65</v>
       </c>
@@ -2894,7 +2899,7 @@
         <v>222</v>
       </c>
       <c r="E22" s="3" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
       <c r="F22" s="3" t="s">
         <v>10</v>
@@ -2915,7 +2920,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="23" spans="1:11" ht="14.25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:11" ht="14.25" x14ac:dyDescent="0.25">
       <c r="A23" s="16" t="s">
         <v>68</v>
       </c>
@@ -2929,7 +2934,7 @@
         <v>222</v>
       </c>
       <c r="E23" s="3" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
       <c r="F23" s="3" t="s">
         <v>10</v>
@@ -2950,7 +2955,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="24" spans="1:11" ht="14.25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:11" ht="14.25" x14ac:dyDescent="0.25">
       <c r="A24" s="16" t="s">
         <v>71</v>
       </c>
@@ -2964,7 +2969,7 @@
         <v>222</v>
       </c>
       <c r="E24" s="3" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
       <c r="F24" s="3" t="s">
         <v>10</v>
@@ -2985,7 +2990,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="25" spans="1:11" ht="14.25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:11" ht="14.25" x14ac:dyDescent="0.25">
       <c r="A25" s="16" t="s">
         <v>74</v>
       </c>
@@ -2999,7 +3004,7 @@
         <v>222</v>
       </c>
       <c r="E25" s="3" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
       <c r="F25" s="3" t="s">
         <v>10</v>
@@ -3020,7 +3025,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="26" spans="1:11" ht="14.25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:11" ht="14.25" x14ac:dyDescent="0.25">
       <c r="A26" s="16" t="s">
         <v>77</v>
       </c>
@@ -3034,7 +3039,7 @@
         <v>222</v>
       </c>
       <c r="E26" s="3" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
       <c r="F26" s="3" t="s">
         <v>10</v>
@@ -3055,7 +3060,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="27" spans="1:11" ht="25.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:11" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A27" s="16" t="s">
         <v>80</v>
       </c>
@@ -3069,7 +3074,7 @@
         <v>222</v>
       </c>
       <c r="E27" s="3" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
       <c r="F27" s="3" t="s">
         <v>10</v>
@@ -3090,7 +3095,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="28" spans="1:11" ht="38.25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:11" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A28" s="16" t="s">
         <v>83</v>
       </c>
@@ -3104,7 +3109,7 @@
         <v>222</v>
       </c>
       <c r="E28" s="3" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
       <c r="F28" s="3" t="s">
         <v>10</v>
@@ -3125,7 +3130,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="29" spans="1:11" ht="14.25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:11" ht="14.25" x14ac:dyDescent="0.25">
       <c r="A29" s="16" t="s">
         <v>86</v>
       </c>
@@ -3139,7 +3144,7 @@
         <v>222</v>
       </c>
       <c r="E29" s="3" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
       <c r="F29" s="3" t="s">
         <v>10</v>
@@ -3160,7 +3165,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="30" spans="1:11" ht="25.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:11" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A30" s="16" t="s">
         <v>90</v>
       </c>
@@ -3174,7 +3179,7 @@
         <v>222</v>
       </c>
       <c r="E30" s="3" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
       <c r="F30" s="3" t="s">
         <v>10</v>
@@ -3195,7 +3200,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="31" spans="1:11" ht="14.25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:11" ht="14.25" x14ac:dyDescent="0.25">
       <c r="A31" s="16" t="s">
         <v>93</v>
       </c>
@@ -3209,7 +3214,7 @@
         <v>222</v>
       </c>
       <c r="E31" s="3" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
       <c r="F31" s="3" t="s">
         <v>10</v>
@@ -3230,7 +3235,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="32" spans="1:11" ht="14.25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:11" ht="14.25" x14ac:dyDescent="0.25">
       <c r="A32" s="16" t="s">
         <v>96</v>
       </c>
@@ -3244,7 +3249,7 @@
         <v>222</v>
       </c>
       <c r="E32" s="3" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
       <c r="F32" s="3" t="s">
         <v>10</v>
@@ -3265,7 +3270,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="33" spans="1:11" ht="14.25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:11" ht="14.25" x14ac:dyDescent="0.25">
       <c r="A33" s="16" t="s">
         <v>98</v>
       </c>
@@ -3279,7 +3284,7 @@
         <v>222</v>
       </c>
       <c r="E33" s="3" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
       <c r="F33" s="3" t="s">
         <v>10</v>
@@ -3300,7 +3305,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="34" spans="1:11" ht="14.25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:11" ht="14.25" x14ac:dyDescent="0.25">
       <c r="A34" s="16" t="s">
         <v>100</v>
       </c>
@@ -3314,7 +3319,7 @@
         <v>222</v>
       </c>
       <c r="E34" s="3" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
       <c r="F34" s="3" t="s">
         <v>10</v>
@@ -3335,7 +3340,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="35" spans="1:11" ht="25.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:11" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A35" s="16" t="s">
         <v>102</v>
       </c>
@@ -3349,7 +3354,7 @@
         <v>222</v>
       </c>
       <c r="E35" s="3" t="s">
-        <v>397</v>
+        <v>395</v>
       </c>
       <c r="F35" s="3" t="s">
         <v>10</v>
@@ -3370,7 +3375,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="36" spans="1:11" ht="14.25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:11" ht="14.25" x14ac:dyDescent="0.25">
       <c r="A36" s="16" t="s">
         <v>278</v>
       </c>
@@ -3384,7 +3389,7 @@
         <v>222</v>
       </c>
       <c r="E36" s="3" t="s">
-        <v>397</v>
+        <v>395</v>
       </c>
       <c r="F36" s="3" t="s">
         <v>10</v>
@@ -3405,7 +3410,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="37" spans="1:11" ht="14.25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:11" ht="14.25" x14ac:dyDescent="0.25">
       <c r="A37" s="16" t="s">
         <v>279</v>
       </c>
@@ -3419,7 +3424,7 @@
         <v>222</v>
       </c>
       <c r="E37" s="3" t="s">
-        <v>397</v>
+        <v>395</v>
       </c>
       <c r="F37" s="3" t="s">
         <v>10</v>
@@ -3440,7 +3445,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="38" spans="1:11" ht="14.25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:11" ht="14.25" x14ac:dyDescent="0.25">
       <c r="A38" s="16" t="s">
         <v>280</v>
       </c>
@@ -3454,7 +3459,7 @@
         <v>222</v>
       </c>
       <c r="E38" s="3" t="s">
-        <v>397</v>
+        <v>395</v>
       </c>
       <c r="F38" s="3" t="s">
         <v>10</v>
@@ -3475,7 +3480,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="39" spans="1:11" ht="25.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:11" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A39" s="16" t="s">
         <v>108</v>
       </c>
@@ -3489,7 +3494,7 @@
         <v>222</v>
       </c>
       <c r="E39" s="3" t="s">
-        <v>397</v>
+        <v>395</v>
       </c>
       <c r="F39" s="3" t="s">
         <v>10</v>
@@ -3510,7 +3515,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="40" spans="1:11" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:11" ht="15" x14ac:dyDescent="0.25">
       <c r="A40" s="16" t="s">
         <v>277</v>
       </c>
@@ -3524,7 +3529,7 @@
         <v>222</v>
       </c>
       <c r="E40" s="3" t="s">
-        <v>397</v>
+        <v>395</v>
       </c>
       <c r="F40" s="3" t="s">
         <v>10</v>
@@ -3545,7 +3550,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="41" spans="1:11" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:11" ht="15" x14ac:dyDescent="0.25">
       <c r="A41" s="16" t="s">
         <v>276</v>
       </c>
@@ -3559,7 +3564,7 @@
         <v>222</v>
       </c>
       <c r="E41" s="3" t="s">
-        <v>397</v>
+        <v>395</v>
       </c>
       <c r="F41" s="3" t="s">
         <v>10</v>
@@ -3580,7 +3585,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="42" spans="1:11" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:11" ht="15" x14ac:dyDescent="0.25">
       <c r="A42" s="16" t="s">
         <v>275</v>
       </c>
@@ -3594,7 +3599,7 @@
         <v>222</v>
       </c>
       <c r="E42" s="3" t="s">
-        <v>397</v>
+        <v>395</v>
       </c>
       <c r="F42" s="3" t="s">
         <v>10</v>
@@ -3615,7 +3620,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="43" spans="1:11" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:11" ht="15" x14ac:dyDescent="0.25">
       <c r="A43" s="16" t="s">
         <v>110</v>
       </c>
@@ -3629,7 +3634,7 @@
         <v>222</v>
       </c>
       <c r="E43" s="3" t="s">
-        <v>397</v>
+        <v>395</v>
       </c>
       <c r="F43" s="3" t="s">
         <v>10</v>
@@ -3650,7 +3655,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="44" spans="1:11" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:11" ht="15" x14ac:dyDescent="0.25">
       <c r="A44" s="16" t="s">
         <v>114</v>
       </c>
@@ -3664,7 +3669,7 @@
         <v>222</v>
       </c>
       <c r="E44" s="3" t="s">
-        <v>397</v>
+        <v>395</v>
       </c>
       <c r="F44" s="3" t="s">
         <v>10</v>
@@ -3685,7 +3690,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="45" spans="1:11" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:11" ht="15" x14ac:dyDescent="0.25">
       <c r="A45" s="16" t="s">
         <v>117</v>
       </c>
@@ -3699,7 +3704,7 @@
         <v>222</v>
       </c>
       <c r="E45" s="3" t="s">
-        <v>397</v>
+        <v>395</v>
       </c>
       <c r="F45" s="3" t="s">
         <v>10</v>
@@ -3720,7 +3725,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="46" spans="1:11" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:11" ht="15" x14ac:dyDescent="0.25">
       <c r="A46" s="16" t="s">
         <v>118</v>
       </c>
@@ -3734,7 +3739,7 @@
         <v>222</v>
       </c>
       <c r="E46" s="3" t="s">
-        <v>397</v>
+        <v>395</v>
       </c>
       <c r="F46" s="3" t="s">
         <v>10</v>
@@ -3755,7 +3760,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="47" spans="1:11" ht="25.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:11" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A47" s="16" t="s">
         <v>122</v>
       </c>
@@ -3769,7 +3774,7 @@
         <v>222</v>
       </c>
       <c r="E47" s="3" t="s">
-        <v>397</v>
+        <v>395</v>
       </c>
       <c r="F47" s="3" t="s">
         <v>10</v>
@@ -3790,7 +3795,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="48" spans="1:11" ht="60" hidden="1" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:11" ht="60" x14ac:dyDescent="0.25">
       <c r="A48" s="16" t="s">
         <v>124</v>
       </c>
@@ -3804,7 +3809,7 @@
         <v>222</v>
       </c>
       <c r="E48" s="3" t="s">
-        <v>397</v>
+        <v>395</v>
       </c>
       <c r="F48" s="3" t="s">
         <v>10</v>
@@ -3825,7 +3830,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="49" spans="1:21" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:21" ht="15" x14ac:dyDescent="0.25">
       <c r="A49" s="16" t="s">
         <v>127</v>
       </c>
@@ -3839,7 +3844,7 @@
         <v>222</v>
       </c>
       <c r="E49" s="3" t="s">
-        <v>397</v>
+        <v>395</v>
       </c>
       <c r="F49" s="3" t="s">
         <v>10</v>
@@ -3860,7 +3865,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="50" spans="1:21" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:21" ht="15" x14ac:dyDescent="0.25">
       <c r="A50" s="16" t="s">
         <v>129</v>
       </c>
@@ -3874,7 +3879,7 @@
         <v>222</v>
       </c>
       <c r="E50" s="3" t="s">
-        <v>397</v>
+        <v>395</v>
       </c>
       <c r="F50" s="3" t="s">
         <v>10</v>
@@ -3895,7 +3900,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="51" spans="1:21" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:21" ht="15" x14ac:dyDescent="0.25">
       <c r="A51" s="16" t="s">
         <v>133</v>
       </c>
@@ -3909,7 +3914,7 @@
         <v>222</v>
       </c>
       <c r="E51" s="3" t="s">
-        <v>397</v>
+        <v>395</v>
       </c>
       <c r="F51" s="3" t="s">
         <v>10</v>
@@ -3930,7 +3935,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="52" spans="1:21" ht="40.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:21" ht="40.5" x14ac:dyDescent="0.25">
       <c r="A52" s="16" t="s">
         <v>135</v>
       </c>
@@ -3944,7 +3949,7 @@
         <v>222</v>
       </c>
       <c r="E52" s="3" t="s">
-        <v>397</v>
+        <v>395</v>
       </c>
       <c r="F52" s="3" t="s">
         <v>10</v>
@@ -3965,7 +3970,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="53" spans="1:21" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:21" ht="15" x14ac:dyDescent="0.25">
       <c r="A53" s="16" t="s">
         <v>139</v>
       </c>
@@ -3979,7 +3984,7 @@
         <v>222</v>
       </c>
       <c r="E53" s="3" t="s">
-        <v>397</v>
+        <v>395</v>
       </c>
       <c r="F53" s="3" t="s">
         <v>10</v>
@@ -4000,7 +4005,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="54" spans="1:21" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:21" ht="15" x14ac:dyDescent="0.25">
       <c r="A54" s="16" t="s">
         <v>141</v>
       </c>
@@ -4014,7 +4019,7 @@
         <v>222</v>
       </c>
       <c r="E54" s="3" t="s">
-        <v>397</v>
+        <v>395</v>
       </c>
       <c r="F54" s="3" t="s">
         <v>10</v>
@@ -4035,7 +4040,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="55" spans="1:21" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:21" ht="15" x14ac:dyDescent="0.25">
       <c r="A55" s="16" t="s">
         <v>144</v>
       </c>
@@ -4049,7 +4054,7 @@
         <v>222</v>
       </c>
       <c r="E55" s="3" t="s">
-        <v>397</v>
+        <v>395</v>
       </c>
       <c r="F55" s="3" t="s">
         <v>10</v>
@@ -4070,7 +4075,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="56" spans="1:21" ht="27.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:21" ht="27.75" x14ac:dyDescent="0.25">
       <c r="A56" s="16" t="s">
         <v>145</v>
       </c>
@@ -4084,7 +4089,7 @@
         <v>222</v>
       </c>
       <c r="E56" s="3" t="s">
-        <v>397</v>
+        <v>395</v>
       </c>
       <c r="F56" s="3" t="s">
         <v>10</v>
@@ -4105,7 +4110,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="57" spans="1:21" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:21" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A57" s="16" t="s">
         <v>149</v>
       </c>
@@ -4119,7 +4124,7 @@
         <v>222</v>
       </c>
       <c r="E57" s="3" t="s">
-        <v>397</v>
+        <v>395</v>
       </c>
       <c r="F57" s="3" t="s">
         <v>10</v>
@@ -4140,7 +4145,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="58" spans="1:21" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:21" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A58" s="16" t="s">
         <v>151</v>
       </c>
@@ -4154,7 +4159,7 @@
         <v>222</v>
       </c>
       <c r="E58" s="3" t="s">
-        <v>397</v>
+        <v>395</v>
       </c>
       <c r="F58" s="3" t="s">
         <v>10</v>
@@ -4175,7 +4180,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="59" spans="1:21" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:21" ht="15" x14ac:dyDescent="0.25">
       <c r="A59" s="16" t="s">
         <v>155</v>
       </c>
@@ -4189,7 +4194,7 @@
         <v>222</v>
       </c>
       <c r="E59" s="3" t="s">
-        <v>397</v>
+        <v>395</v>
       </c>
       <c r="F59" s="3" t="s">
         <v>10</v>
@@ -4210,7 +4215,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="60" spans="1:21" ht="25.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:21" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A60" s="16" t="s">
         <v>157</v>
       </c>
@@ -4224,7 +4229,7 @@
         <v>222</v>
       </c>
       <c r="E60" s="3" t="s">
-        <v>397</v>
+        <v>395</v>
       </c>
       <c r="F60" s="3" t="s">
         <v>10</v>
@@ -4245,7 +4250,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="61" spans="1:21" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:21" ht="15" x14ac:dyDescent="0.25">
       <c r="A61" s="16" t="s">
         <v>160</v>
       </c>
@@ -4259,7 +4264,7 @@
         <v>222</v>
       </c>
       <c r="E61" s="3" t="s">
-        <v>397</v>
+        <v>395</v>
       </c>
       <c r="F61" s="3" t="s">
         <v>10</v>
@@ -4294,7 +4299,7 @@
         <v>224</v>
       </c>
       <c r="E62" s="3" t="s">
-        <v>401</v>
+        <v>399</v>
       </c>
       <c r="F62" s="3" t="s">
         <v>10</v>
@@ -4303,10 +4308,10 @@
         <v>265</v>
       </c>
       <c r="H62" s="3" t="s">
-        <v>410</v>
+        <v>408</v>
       </c>
       <c r="I62" s="3" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="J62" s="3" t="s">
         <v>285</v>
@@ -4329,7 +4334,7 @@
         <v>224</v>
       </c>
       <c r="E63" s="3" t="s">
-        <v>401</v>
+        <v>399</v>
       </c>
       <c r="F63" s="3" t="s">
         <v>10</v>
@@ -4338,10 +4343,10 @@
         <v>268</v>
       </c>
       <c r="H63" s="3" t="s">
-        <v>411</v>
+        <v>409</v>
       </c>
       <c r="I63" s="3" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="J63" s="3" t="s">
         <v>285</v>
@@ -4364,7 +4369,7 @@
         <v>224</v>
       </c>
       <c r="E64" s="3" t="s">
-        <v>402</v>
+        <v>400</v>
       </c>
       <c r="F64" s="3" t="s">
         <v>168</v>
@@ -4409,7 +4414,7 @@
         <v>224</v>
       </c>
       <c r="E65" s="3" t="s">
-        <v>402</v>
+        <v>400</v>
       </c>
       <c r="F65" s="3" t="s">
         <v>168</v>
@@ -4454,7 +4459,7 @@
         <v>224</v>
       </c>
       <c r="E66" s="3" t="s">
-        <v>402</v>
+        <v>400</v>
       </c>
       <c r="F66" s="3" t="s">
         <v>168</v>
@@ -4466,7 +4471,7 @@
         <v>185</v>
       </c>
       <c r="I66" s="3" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="J66" s="3" t="s">
         <v>174</v>
@@ -4489,7 +4494,7 @@
         <v>224</v>
       </c>
       <c r="E67" s="3" t="s">
-        <v>409</v>
+        <v>407</v>
       </c>
       <c r="F67" s="3" t="s">
         <v>168</v>
@@ -4524,10 +4529,10 @@
         <v>227</v>
       </c>
       <c r="E68" s="3" t="s">
+        <v>410</v>
+      </c>
+      <c r="F68" s="3" t="s">
         <v>412</v>
-      </c>
-      <c r="F68" s="3" t="s">
-        <v>414</v>
       </c>
       <c r="G68" s="3" t="s">
         <v>296</v>
@@ -4559,10 +4564,10 @@
         <v>227</v>
       </c>
       <c r="E69" s="3" t="s">
+        <v>410</v>
+      </c>
+      <c r="F69" s="3" t="s">
         <v>412</v>
-      </c>
-      <c r="F69" s="3" t="s">
-        <v>414</v>
       </c>
       <c r="G69" s="3" t="s">
         <v>299</v>
@@ -4594,10 +4599,10 @@
         <v>227</v>
       </c>
       <c r="E70" s="3" t="s">
-        <v>413</v>
+        <v>411</v>
       </c>
       <c r="F70" s="3" t="s">
-        <v>414</v>
+        <v>412</v>
       </c>
       <c r="G70" s="3" t="s">
         <v>302</v>
@@ -4629,7 +4634,7 @@
         <v>224</v>
       </c>
       <c r="E71" s="3" t="s">
-        <v>402</v>
+        <v>400</v>
       </c>
       <c r="F71" s="3" t="s">
         <v>168</v>
@@ -4664,10 +4669,10 @@
         <v>227</v>
       </c>
       <c r="E72" s="3" t="s">
-        <v>412</v>
+        <v>410</v>
       </c>
       <c r="F72" s="3" t="s">
-        <v>415</v>
+        <v>413</v>
       </c>
       <c r="G72" s="3" t="s">
         <v>308</v>
@@ -4699,10 +4704,10 @@
         <v>227</v>
       </c>
       <c r="E73" s="3" t="s">
-        <v>412</v>
+        <v>410</v>
       </c>
       <c r="F73" s="3" t="s">
-        <v>415</v>
+        <v>413</v>
       </c>
       <c r="G73" s="3" t="s">
         <v>311</v>
@@ -4734,13 +4739,13 @@
         <v>227</v>
       </c>
       <c r="E74" s="3" t="s">
-        <v>412</v>
+        <v>410</v>
       </c>
       <c r="F74" s="3" t="s">
         <v>168</v>
       </c>
       <c r="G74" s="3" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="H74" s="3" t="s">
         <v>314</v>
@@ -4755,20 +4760,22 @@
         <v>14</v>
       </c>
     </row>
-    <row r="75" spans="1:21" ht="25.5" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A75" s="3" t="s">
+    <row r="75" spans="1:21" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="A75" s="16" t="s">
         <v>183</v>
       </c>
       <c r="B75" s="3" t="s">
+        <v>334</v>
+      </c>
+      <c r="C75" s="3" t="s">
         <v>335</v>
       </c>
-      <c r="C75" s="3" t="s">
-        <v>336</v>
-      </c>
       <c r="D75" s="3" t="s">
         <v>222</v>
       </c>
-      <c r="E75" s="3"/>
+      <c r="E75" s="3" t="s">
+        <v>420</v>
+      </c>
       <c r="F75" s="3" t="s">
         <v>10</v>
       </c>
@@ -4788,31 +4795,33 @@
         <v>26</v>
       </c>
     </row>
-    <row r="76" spans="1:21" ht="14.25" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A76" s="3" t="s">
+    <row r="76" spans="1:21" ht="14.25" x14ac:dyDescent="0.25">
+      <c r="A76" s="16" t="s">
         <v>186</v>
       </c>
       <c r="B76" s="3" t="s">
+        <v>334</v>
+      </c>
+      <c r="C76" s="3" t="s">
         <v>335</v>
       </c>
-      <c r="C76" s="3" t="s">
-        <v>336</v>
-      </c>
       <c r="D76" s="3" t="s">
         <v>222</v>
       </c>
-      <c r="E76" s="3"/>
+      <c r="E76" s="3" t="s">
+        <v>420</v>
+      </c>
       <c r="F76" s="3" t="s">
         <v>10</v>
       </c>
       <c r="G76" s="3" t="s">
+        <v>421</v>
+      </c>
+      <c r="H76" s="3" t="s">
         <v>329</v>
       </c>
-      <c r="H76" s="3" t="s">
+      <c r="I76" s="3" t="s">
         <v>330</v>
-      </c>
-      <c r="I76" s="3" t="s">
-        <v>331</v>
       </c>
       <c r="J76" s="3" t="s">
         <v>30</v>
@@ -4821,31 +4830,33 @@
         <v>14</v>
       </c>
     </row>
-    <row r="77" spans="1:21" ht="14.25" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A77" s="3" t="s">
+    <row r="77" spans="1:21" ht="14.25" x14ac:dyDescent="0.25">
+      <c r="A77" s="16" t="s">
         <v>324</v>
       </c>
       <c r="B77" s="3" t="s">
+        <v>334</v>
+      </c>
+      <c r="C77" s="3" t="s">
         <v>335</v>
       </c>
-      <c r="C77" s="3" t="s">
-        <v>336</v>
-      </c>
       <c r="D77" s="3" t="s">
         <v>222</v>
       </c>
-      <c r="E77" s="3"/>
+      <c r="E77" s="3" t="s">
+        <v>420</v>
+      </c>
       <c r="F77" s="3" t="s">
         <v>10</v>
       </c>
       <c r="G77" s="3" t="s">
+        <v>337</v>
+      </c>
+      <c r="H77" s="3" t="s">
         <v>338</v>
       </c>
-      <c r="H77" s="3" t="s">
+      <c r="I77" s="3" t="s">
         <v>339</v>
-      </c>
-      <c r="I77" s="3" t="s">
-        <v>340</v>
       </c>
       <c r="J77" s="3" t="s">
         <v>30</v>
@@ -4854,31 +4865,33 @@
         <v>14</v>
       </c>
     </row>
-    <row r="78" spans="1:21" ht="14.25" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A78" s="3" t="s">
+    <row r="78" spans="1:21" ht="14.25" x14ac:dyDescent="0.25">
+      <c r="A78" s="16" t="s">
         <v>328</v>
       </c>
       <c r="B78" s="3" t="s">
+        <v>334</v>
+      </c>
+      <c r="C78" s="3" t="s">
         <v>335</v>
       </c>
-      <c r="C78" s="3" t="s">
-        <v>336</v>
-      </c>
       <c r="D78" s="3" t="s">
         <v>222</v>
       </c>
-      <c r="E78" s="3"/>
+      <c r="E78" s="3" t="s">
+        <v>420</v>
+      </c>
       <c r="F78" s="3" t="s">
         <v>10</v>
       </c>
       <c r="G78" s="3" t="s">
+        <v>341</v>
+      </c>
+      <c r="H78" s="3" t="s">
         <v>342</v>
       </c>
-      <c r="H78" s="3" t="s">
-        <v>343</v>
-      </c>
       <c r="I78" s="3" t="s">
-        <v>344</v>
+        <v>422</v>
       </c>
       <c r="J78" s="3" t="s">
         <v>30</v>
@@ -4887,31 +4900,33 @@
         <v>26</v>
       </c>
     </row>
-    <row r="79" spans="1:21" ht="25.5" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A79" s="3" t="s">
-        <v>337</v>
+    <row r="79" spans="1:21" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="A79" s="16" t="s">
+        <v>336</v>
       </c>
       <c r="B79" s="3" t="s">
+        <v>334</v>
+      </c>
+      <c r="C79" s="3" t="s">
         <v>335</v>
       </c>
-      <c r="C79" s="3" t="s">
-        <v>336</v>
-      </c>
       <c r="D79" s="3" t="s">
         <v>222</v>
       </c>
-      <c r="E79" s="3"/>
+      <c r="E79" s="3" t="s">
+        <v>420</v>
+      </c>
       <c r="F79" s="3" t="s">
         <v>10</v>
       </c>
       <c r="G79" s="3" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="H79" s="3" t="s">
         <v>292</v>
       </c>
       <c r="I79" s="3" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
       <c r="J79" s="3" t="s">
         <v>30</v>
@@ -4920,9 +4935,9 @@
         <v>14</v>
       </c>
     </row>
-    <row r="80" spans="1:21" ht="14.25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:21" ht="14.25" x14ac:dyDescent="0.25">
       <c r="A80" s="3" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="B80" s="3" t="s">
         <v>319</v>
@@ -4953,9 +4968,9 @@
         <v>26</v>
       </c>
     </row>
-    <row r="81" spans="1:11" ht="25.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:11" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A81" s="3" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="B81" s="3" t="s">
         <v>319</v>
@@ -4986,9 +5001,9 @@
         <v>26</v>
       </c>
     </row>
-    <row r="82" spans="1:11" ht="14.25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:11" ht="14.25" x14ac:dyDescent="0.25">
       <c r="A82" s="3" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
       <c r="B82" s="3" t="s">
         <v>319</v>
@@ -5004,13 +5019,13 @@
         <v>10</v>
       </c>
       <c r="G82" s="3" t="s">
+        <v>347</v>
+      </c>
+      <c r="H82" s="3" t="s">
+        <v>348</v>
+      </c>
+      <c r="I82" s="3" t="s">
         <v>349</v>
-      </c>
-      <c r="H82" s="3" t="s">
-        <v>350</v>
-      </c>
-      <c r="I82" s="3" t="s">
-        <v>351</v>
       </c>
       <c r="J82" s="3" t="s">
         <v>30</v>
@@ -5021,7 +5036,7 @@
     </row>
     <row r="83" spans="1:11" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A83" s="16" t="s">
-        <v>354</v>
+        <v>352</v>
       </c>
       <c r="B83" s="3" t="s">
         <v>218</v>
@@ -5033,19 +5048,19 @@
         <v>227</v>
       </c>
       <c r="E83" s="3" t="s">
-        <v>412</v>
+        <v>410</v>
       </c>
       <c r="F83" s="3" t="s">
         <v>10</v>
       </c>
       <c r="G83" s="3" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="H83" s="3" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="I83" s="3" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
       <c r="J83" s="3" t="s">
         <v>30</v>
@@ -5056,7 +5071,7 @@
     </row>
     <row r="84" spans="1:11" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A84" s="16" t="s">
-        <v>355</v>
+        <v>353</v>
       </c>
       <c r="B84" s="3" t="s">
         <v>218</v>
@@ -5068,19 +5083,19 @@
         <v>227</v>
       </c>
       <c r="E84" s="3" t="s">
-        <v>412</v>
+        <v>410</v>
       </c>
       <c r="F84" s="3" t="s">
         <v>10</v>
       </c>
       <c r="G84" s="3" t="s">
-        <v>363</v>
+        <v>361</v>
       </c>
       <c r="H84" s="3" t="s">
-        <v>364</v>
+        <v>362</v>
       </c>
       <c r="I84" s="3" t="s">
-        <v>405</v>
+        <v>403</v>
       </c>
       <c r="J84" s="3" t="s">
         <v>30</v>
@@ -5091,7 +5106,7 @@
     </row>
     <row r="85" spans="1:11" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A85" s="16" t="s">
-        <v>356</v>
+        <v>354</v>
       </c>
       <c r="B85" s="3" t="s">
         <v>218</v>
@@ -5103,19 +5118,19 @@
         <v>222</v>
       </c>
       <c r="E85" s="3" t="s">
-        <v>416</v>
+        <v>414</v>
       </c>
       <c r="F85" s="3" t="s">
-        <v>403</v>
+        <v>401</v>
       </c>
       <c r="G85" s="3" t="s">
-        <v>408</v>
+        <v>406</v>
       </c>
       <c r="H85" s="3" t="s">
-        <v>406</v>
+        <v>404</v>
       </c>
       <c r="I85" s="3" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
       <c r="J85" s="3" t="s">
         <v>30</v>
@@ -5126,7 +5141,7 @@
     </row>
     <row r="86" spans="1:11" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A86" s="16" t="s">
-        <v>357</v>
+        <v>355</v>
       </c>
       <c r="B86" s="3" t="s">
         <v>218</v>
@@ -5138,19 +5153,19 @@
         <v>227</v>
       </c>
       <c r="E86" s="3" t="s">
-        <v>412</v>
+        <v>410</v>
       </c>
       <c r="F86" s="3" t="s">
         <v>168</v>
       </c>
       <c r="G86" s="3" t="s">
-        <v>374</v>
+        <v>372</v>
       </c>
       <c r="H86" s="3" t="s">
-        <v>365</v>
+        <v>363</v>
       </c>
       <c r="I86" s="3" t="s">
-        <v>366</v>
+        <v>364</v>
       </c>
       <c r="J86" s="3" t="s">
         <v>30</v>
@@ -5161,7 +5176,7 @@
     </row>
     <row r="87" spans="1:11" ht="14.25" x14ac:dyDescent="0.25">
       <c r="A87" s="16" t="s">
-        <v>358</v>
+        <v>356</v>
       </c>
       <c r="B87" s="3" t="s">
         <v>218</v>
@@ -5173,19 +5188,19 @@
         <v>222</v>
       </c>
       <c r="E87" s="3" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
       <c r="F87" s="3" t="s">
         <v>10</v>
       </c>
       <c r="G87" s="3" t="s">
+        <v>365</v>
+      </c>
+      <c r="H87" s="3" t="s">
+        <v>366</v>
+      </c>
+      <c r="I87" s="3" t="s">
         <v>367</v>
-      </c>
-      <c r="H87" s="3" t="s">
-        <v>368</v>
-      </c>
-      <c r="I87" s="3" t="s">
-        <v>369</v>
       </c>
       <c r="J87" s="3" t="s">
         <v>30</v>
@@ -5196,7 +5211,7 @@
     </row>
     <row r="88" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A88" s="16" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
       <c r="B88" s="3" t="s">
         <v>218</v>
@@ -5208,19 +5223,19 @@
         <v>222</v>
       </c>
       <c r="E88" s="3" t="s">
-        <v>418</v>
+        <v>416</v>
       </c>
       <c r="F88" s="3" t="s">
         <v>168</v>
       </c>
       <c r="G88" s="3" t="s">
-        <v>370</v>
+        <v>368</v>
       </c>
       <c r="H88" s="3" t="s">
-        <v>368</v>
+        <v>366</v>
       </c>
       <c r="I88" s="3" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="J88" s="3" t="s">
         <v>30</v>
@@ -5229,9 +5244,9 @@
         <v>14</v>
       </c>
     </row>
-    <row r="89" spans="1:11" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:11" ht="114.75" x14ac:dyDescent="0.25">
       <c r="A89" s="3" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="B89" s="3" t="s">
         <v>218</v>
@@ -5242,35 +5257,37 @@
       <c r="D89" s="3" t="s">
         <v>227</v>
       </c>
-      <c r="E89" s="3"/>
+      <c r="E89" s="3" t="s">
+        <v>419</v>
+      </c>
       <c r="F89" s="3" t="s">
         <v>168</v>
       </c>
       <c r="G89" s="3" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="H89" s="3" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="I89" s="3" t="s">
-        <v>372</v>
+        <v>370</v>
       </c>
       <c r="J89" s="3" t="s">
         <v>30</v>
       </c>
       <c r="K89" s="15" t="s">
-        <v>353</v>
-      </c>
-    </row>
-    <row r="90" spans="1:11" ht="25.5" hidden="1" x14ac:dyDescent="0.25">
+        <v>351</v>
+      </c>
+    </row>
+    <row r="90" spans="1:11" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A90" s="3" t="s">
-        <v>384</v>
+        <v>382</v>
       </c>
       <c r="B90" s="3" t="s">
-        <v>335</v>
+        <v>218</v>
       </c>
       <c r="C90" s="3" t="s">
-        <v>336</v>
+        <v>221</v>
       </c>
       <c r="D90" s="3" t="s">
         <v>222</v>
@@ -5280,13 +5297,13 @@
         <v>168</v>
       </c>
       <c r="G90" s="3" t="s">
-        <v>381</v>
+        <v>379</v>
       </c>
       <c r="H90" s="3" t="s">
-        <v>378</v>
+        <v>376</v>
       </c>
       <c r="I90" s="3" t="s">
-        <v>375</v>
+        <v>373</v>
       </c>
       <c r="J90" s="3" t="s">
         <v>30</v>
@@ -5295,15 +5312,15 @@
         <v>14</v>
       </c>
     </row>
-    <row r="91" spans="1:11" ht="25.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:11" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A91" s="3" t="s">
-        <v>385</v>
+        <v>383</v>
       </c>
       <c r="B91" s="3" t="s">
-        <v>335</v>
+        <v>218</v>
       </c>
       <c r="C91" s="3" t="s">
-        <v>336</v>
+        <v>221</v>
       </c>
       <c r="D91" s="3" t="s">
         <v>222</v>
@@ -5313,13 +5330,13 @@
         <v>168</v>
       </c>
       <c r="G91" s="3" t="s">
-        <v>382</v>
+        <v>380</v>
       </c>
       <c r="H91" s="3" t="s">
-        <v>379</v>
+        <v>377</v>
       </c>
       <c r="I91" s="3" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
       <c r="J91" s="3" t="s">
         <v>30</v>
@@ -5328,9 +5345,9 @@
         <v>26</v>
       </c>
     </row>
-    <row r="92" spans="1:11" ht="25.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:11" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A92" s="3" t="s">
-        <v>386</v>
+        <v>384</v>
       </c>
       <c r="B92" s="3" t="s">
         <v>319</v>
@@ -5346,13 +5363,13 @@
         <v>168</v>
       </c>
       <c r="G92" s="8" t="s">
-        <v>383</v>
+        <v>381</v>
       </c>
       <c r="H92" s="9" t="s">
-        <v>380</v>
+        <v>378</v>
       </c>
       <c r="I92" s="3" t="s">
-        <v>377</v>
+        <v>375</v>
       </c>
       <c r="J92" s="3" t="s">
         <v>30</v>
@@ -5506,11 +5523,6 @@
     </row>
   </sheetData>
   <autoFilter ref="A3:U92" xr:uid="{00000000-0001-0000-0000-000000000000}">
-    <filterColumn colId="1">
-      <filters>
-        <filter val="Intégration"/>
-      </filters>
-    </filterColumn>
     <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A4:U92">
       <sortCondition ref="A3:A92"/>
     </sortState>
@@ -5580,7 +5592,7 @@
         <v>220</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>396</v>
+        <v>394</v>
       </c>
       <c r="F3" s="1" t="s">
         <v>3</v>
@@ -5679,7 +5691,7 @@
         <v>220</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>396</v>
+        <v>394</v>
       </c>
       <c r="F3" s="1" t="s">
         <v>3</v>
@@ -5702,7 +5714,7 @@
     </row>
     <row r="4" spans="1:11" ht="53.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="16" t="s">
-        <v>387</v>
+        <v>385</v>
       </c>
       <c r="B4" s="3" t="s">
         <v>217</v>
@@ -5714,7 +5726,7 @@
         <v>222</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>400</v>
+        <v>398</v>
       </c>
       <c r="F4" s="3" t="s">
         <v>198</v>
@@ -5726,7 +5738,7 @@
         <v>259</v>
       </c>
       <c r="I4" s="3" t="s">
-        <v>420</v>
+        <v>418</v>
       </c>
       <c r="J4" s="3" t="s">
         <v>13</v>
@@ -5737,7 +5749,7 @@
     </row>
     <row r="5" spans="1:11" ht="53.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="16" t="s">
-        <v>388</v>
+        <v>386</v>
       </c>
       <c r="B5" s="3" t="s">
         <v>217</v>
@@ -5749,7 +5761,7 @@
         <v>222</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>400</v>
+        <v>398</v>
       </c>
       <c r="F5" s="3" t="s">
         <v>198</v>
@@ -5761,7 +5773,7 @@
         <v>260</v>
       </c>
       <c r="I5" s="3" t="s">
-        <v>420</v>
+        <v>418</v>
       </c>
       <c r="J5" s="3" t="s">
         <v>13</v>
@@ -5772,7 +5784,7 @@
     </row>
     <row r="6" spans="1:11" ht="53.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="16" t="s">
-        <v>389</v>
+        <v>387</v>
       </c>
       <c r="B6" s="3" t="s">
         <v>217</v>
@@ -5784,7 +5796,7 @@
         <v>222</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>400</v>
+        <v>398</v>
       </c>
       <c r="F6" s="3" t="s">
         <v>198</v>
@@ -5796,7 +5808,7 @@
         <v>261</v>
       </c>
       <c r="I6" s="3" t="s">
-        <v>420</v>
+        <v>418</v>
       </c>
       <c r="J6" s="3" t="s">
         <v>212</v>
@@ -5807,7 +5819,7 @@
     </row>
     <row r="7" spans="1:11" ht="51" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
-        <v>390</v>
+        <v>388</v>
       </c>
       <c r="B7" s="3" t="s">
         <v>218</v>
@@ -5829,7 +5841,7 @@
         <v>202</v>
       </c>
       <c r="I7" s="3" t="s">
-        <v>419</v>
+        <v>417</v>
       </c>
       <c r="J7" s="3" t="s">
         <v>13</v>
@@ -5840,7 +5852,7 @@
     </row>
     <row r="8" spans="1:11" ht="165.75" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
-        <v>391</v>
+        <v>389</v>
       </c>
       <c r="B8" s="3" t="s">
         <v>218</v>
@@ -5873,7 +5885,7 @@
     </row>
     <row r="9" spans="1:11" ht="127.5" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
-        <v>392</v>
+        <v>390</v>
       </c>
       <c r="B9" s="3" t="s">
         <v>218</v>
@@ -5906,7 +5918,7 @@
     </row>
     <row r="10" spans="1:11" ht="76.5" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
-        <v>393</v>
+        <v>391</v>
       </c>
       <c r="B10" s="3" t="s">
         <v>218</v>
@@ -5939,7 +5951,7 @@
     </row>
     <row r="11" spans="1:11" ht="165.75" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
       <c r="B11" s="3" t="s">
         <v>218</v>
@@ -5972,7 +5984,7 @@
     </row>
     <row r="12" spans="1:11" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
-        <v>395</v>
+        <v>393</v>
       </c>
       <c r="B12" s="3" t="s">
         <v>218</v>
@@ -6076,7 +6088,7 @@
         <v>220</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>396</v>
+        <v>394</v>
       </c>
       <c r="F3" s="1" t="s">
         <v>3</v>
@@ -6162,7 +6174,7 @@
         <v>220</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>396</v>
+        <v>394</v>
       </c>
       <c r="F3" s="1" t="s">
         <v>3</v>
@@ -6248,7 +6260,7 @@
         <v>220</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>396</v>
+        <v>394</v>
       </c>
       <c r="F3" s="1" t="s">
         <v>3</v>
@@ -6334,7 +6346,7 @@
         <v>220</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>396</v>
+        <v>394</v>
       </c>
       <c r="F3" s="1" t="s">
         <v>3</v>
@@ -6420,7 +6432,7 @@
         <v>220</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>396</v>
+        <v>394</v>
       </c>
       <c r="F3" s="1" t="s">
         <v>3</v>
@@ -6506,7 +6518,7 @@
         <v>220</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>396</v>
+        <v>394</v>
       </c>
       <c r="F3" s="1" t="s">
         <v>3</v>
@@ -6592,7 +6604,7 @@
         <v>220</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>396</v>
+        <v>394</v>
       </c>
       <c r="F3" s="1" t="s">
         <v>3</v>

</xml_diff>

<commit_message>
test: integration - TC 79, 80
</commit_message>
<xml_diff>
--- a/docs/tests/breco - cas de test.xlsx
+++ b/docs/tests/breco - cas de test.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\wamp\www\breco_v2_0_0\docs\tests\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8B4A3F02-CE33-4DAF-A5F3-F8F7C531FE42}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{01A33FA2-26C4-406A-824C-FF80DFE9CBC4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1196" uniqueCount="423">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1198" uniqueCount="424">
   <si>
     <t>Plan de test Breco, cas de test</t>
   </si>
@@ -1825,6 +1825,9 @@
   </si>
   <si>
     <t>Étape 2 affichée</t>
+  </si>
+  <si>
+    <t>routerGuard.spec.ts</t>
   </si>
 </sst>
 </file>
@@ -5280,7 +5283,7 @@
       </c>
     </row>
     <row r="90" spans="1:11" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="A90" s="3" t="s">
+      <c r="A90" s="16" t="s">
         <v>382</v>
       </c>
       <c r="B90" s="3" t="s">
@@ -5292,7 +5295,9 @@
       <c r="D90" s="3" t="s">
         <v>222</v>
       </c>
-      <c r="E90" s="3"/>
+      <c r="E90" s="3" t="s">
+        <v>423</v>
+      </c>
       <c r="F90" s="3" t="s">
         <v>168</v>
       </c>
@@ -5313,7 +5318,7 @@
       </c>
     </row>
     <row r="91" spans="1:11" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="A91" s="3" t="s">
+      <c r="A91" s="16" t="s">
         <v>383</v>
       </c>
       <c r="B91" s="3" t="s">
@@ -5325,7 +5330,9 @@
       <c r="D91" s="3" t="s">
         <v>222</v>
       </c>
-      <c r="E91" s="3"/>
+      <c r="E91" s="3" t="s">
+        <v>423</v>
+      </c>
       <c r="F91" s="3" t="s">
         <v>168</v>
       </c>

</xml_diff>

<commit_message>
test: integration Story 2 TC 85 > 90
</commit_message>
<xml_diff>
--- a/docs/tests/breco - cas de test.xlsx
+++ b/docs/tests/breco - cas de test.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\wamp\www\breco_v2_0_0\docs\tests\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{01A33FA2-26C4-406A-824C-FF80DFE9CBC4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{91953D17-0BFF-44F8-86BE-07E5E32555F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Story1 - Auth" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1198" uniqueCount="424">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1204" uniqueCount="426">
   <si>
     <t>Plan de test Breco, cas de test</t>
   </si>
@@ -1059,9 +1059,6 @@
   </si>
   <si>
     <t>entre une ville avec caractères spéciaux (@#&lt;&gt;?&amp;+!)</t>
-  </si>
-  <si>
-    <t>Erreur 422 : "Caractères non autorisés dans la recherche"</t>
   </si>
   <si>
     <t>Type</t>
@@ -1828,6 +1825,15 @@
   </si>
   <si>
     <t>routerGuard.spec.ts</t>
+  </si>
+  <si>
+    <t>townSearch.integration.spec.ts + TownSearchServiceTest</t>
+  </si>
+  <si>
+    <t>Erreur : "Caractères non autorisés dans la recherche"</t>
+  </si>
+  <si>
+    <t>TownSearchServiceTest</t>
   </si>
 </sst>
 </file>
@@ -2228,16 +2234,16 @@
         <v>2</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="C3" s="1" t="s">
+        <v>218</v>
+      </c>
+      <c r="D3" s="1" t="s">
         <v>219</v>
       </c>
-      <c r="D3" s="1" t="s">
-        <v>220</v>
-      </c>
       <c r="E3" s="1" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="F3" s="1" t="s">
         <v>3</v>
@@ -2263,16 +2269,16 @@
         <v>9</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="F4" s="3" t="s">
         <v>10</v>
@@ -2284,7 +2290,7 @@
         <v>12</v>
       </c>
       <c r="I4" s="3" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="J4" s="3" t="s">
         <v>13</v>
@@ -2298,16 +2304,16 @@
         <v>15</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="F5" s="3" t="s">
         <v>10</v>
@@ -2319,7 +2325,7 @@
         <v>17</v>
       </c>
       <c r="I5" s="3" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="J5" s="3" t="s">
         <v>30</v>
@@ -2333,16 +2339,16 @@
         <v>18</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="F6" s="3" t="s">
         <v>10</v>
@@ -2354,7 +2360,7 @@
         <v>20</v>
       </c>
       <c r="I6" s="3" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="J6" s="3" t="s">
         <v>13</v>
@@ -2368,16 +2374,16 @@
         <v>21</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="F7" s="3" t="s">
         <v>10</v>
@@ -2403,16 +2409,16 @@
         <v>27</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="F8" s="3" t="s">
         <v>10</v>
@@ -2424,7 +2430,7 @@
         <v>29</v>
       </c>
       <c r="I8" s="3" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="J8" s="3" t="s">
         <v>30</v>
@@ -2435,19 +2441,19 @@
     </row>
     <row r="9" spans="1:11" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A9" s="16" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="F9" s="3" t="s">
         <v>10</v>
@@ -2459,7 +2465,7 @@
         <v>32</v>
       </c>
       <c r="I9" s="3" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="J9" s="3" t="s">
         <v>30</v>
@@ -2470,31 +2476,31 @@
     </row>
     <row r="10" spans="1:11" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A10" s="16" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="E10" s="3" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
       <c r="F10" s="3" t="s">
         <v>10</v>
       </c>
       <c r="G10" s="3" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="H10" s="7" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="I10" s="3" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="J10" s="3" t="s">
         <v>30</v>
@@ -2505,31 +2511,31 @@
     </row>
     <row r="11" spans="1:11" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A11" s="16" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="E11" s="3" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
       <c r="F11" s="3" t="s">
         <v>10</v>
       </c>
       <c r="G11" s="3" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="H11" s="7" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="I11" s="3" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="J11" s="3" t="s">
         <v>30</v>
@@ -2543,16 +2549,16 @@
         <v>33</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="E12" s="3" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="F12" s="3" t="s">
         <v>10</v>
@@ -2564,7 +2570,7 @@
         <v>35</v>
       </c>
       <c r="I12" s="3" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="J12" s="3" t="s">
         <v>30</v>
@@ -2578,16 +2584,16 @@
         <v>36</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="E13" s="3" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="F13" s="3" t="s">
         <v>10</v>
@@ -2599,7 +2605,7 @@
         <v>38</v>
       </c>
       <c r="I13" s="3" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="J13" s="3" t="s">
         <v>30</v>
@@ -2613,16 +2619,16 @@
         <v>39</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="E14" s="3" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="F14" s="3" t="s">
         <v>10</v>
@@ -2648,16 +2654,16 @@
         <v>43</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="D15" s="3" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="E15" s="3" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="F15" s="3" t="s">
         <v>10</v>
@@ -2669,7 +2675,7 @@
         <v>45</v>
       </c>
       <c r="I15" s="3" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="J15" s="3" t="s">
         <v>30</v>
@@ -2683,16 +2689,16 @@
         <v>46</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="D16" s="3" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="E16" s="3" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="F16" s="3" t="s">
         <v>10</v>
@@ -2704,7 +2710,7 @@
         <v>48</v>
       </c>
       <c r="I16" s="3" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="J16" s="3" t="s">
         <v>13</v>
@@ -2718,16 +2724,16 @@
         <v>49</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="D17" s="3" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="E17" s="3" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="F17" s="3" t="s">
         <v>10</v>
@@ -2736,10 +2742,10 @@
         <v>50</v>
       </c>
       <c r="H17" s="9" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="I17" s="3" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="J17" s="3" t="s">
         <v>30</v>
@@ -2753,16 +2759,16 @@
         <v>51</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="D18" s="3" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="E18" s="3" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="F18" s="3" t="s">
         <v>10</v>
@@ -2788,16 +2794,16 @@
         <v>55</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="C19" s="3" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="D19" s="3" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="E19" s="3" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="F19" s="3" t="s">
         <v>10</v>
@@ -2809,7 +2815,7 @@
         <v>57</v>
       </c>
       <c r="I19" s="3" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="J19" s="3" t="s">
         <v>30</v>
@@ -2823,16 +2829,16 @@
         <v>58</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="C20" s="3" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="D20" s="3" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="E20" s="3" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="F20" s="3" t="s">
         <v>10</v>
@@ -2844,7 +2850,7 @@
         <v>60</v>
       </c>
       <c r="I20" s="3" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="J20" s="3" t="s">
         <v>13</v>
@@ -2858,16 +2864,16 @@
         <v>61</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="C21" s="3" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="D21" s="3" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="E21" s="3" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="F21" s="3" t="s">
         <v>10</v>
@@ -2893,16 +2899,16 @@
         <v>65</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="C22" s="3" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="D22" s="3" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="E22" s="3" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="F22" s="3" t="s">
         <v>10</v>
@@ -2914,7 +2920,7 @@
         <v>67</v>
       </c>
       <c r="I22" s="3" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="J22" s="3" t="s">
         <v>30</v>
@@ -2928,16 +2934,16 @@
         <v>68</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="C23" s="3" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="D23" s="3" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="E23" s="3" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="F23" s="3" t="s">
         <v>10</v>
@@ -2963,16 +2969,16 @@
         <v>71</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="C24" s="3" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="D24" s="3" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="E24" s="3" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="F24" s="3" t="s">
         <v>10</v>
@@ -2998,16 +3004,16 @@
         <v>74</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="C25" s="3" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="D25" s="3" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="E25" s="3" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="F25" s="3" t="s">
         <v>10</v>
@@ -3033,16 +3039,16 @@
         <v>77</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="C26" s="3" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="D26" s="3" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="E26" s="3" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="F26" s="3" t="s">
         <v>10</v>
@@ -3068,16 +3074,16 @@
         <v>80</v>
       </c>
       <c r="B27" s="3" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="C27" s="3" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="D27" s="3" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="E27" s="3" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="F27" s="3" t="s">
         <v>10</v>
@@ -3089,7 +3095,7 @@
         <v>82</v>
       </c>
       <c r="I27" s="3" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="J27" s="3" t="s">
         <v>30</v>
@@ -3103,16 +3109,16 @@
         <v>83</v>
       </c>
       <c r="B28" s="3" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="C28" s="3" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="D28" s="3" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="E28" s="3" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="F28" s="3" t="s">
         <v>10</v>
@@ -3124,7 +3130,7 @@
         <v>85</v>
       </c>
       <c r="I28" s="3" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="J28" s="3" t="s">
         <v>13</v>
@@ -3138,16 +3144,16 @@
         <v>86</v>
       </c>
       <c r="B29" s="3" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="C29" s="3" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="D29" s="3" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="E29" s="3" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="F29" s="3" t="s">
         <v>10</v>
@@ -3173,16 +3179,16 @@
         <v>90</v>
       </c>
       <c r="B30" s="3" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="C30" s="3" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="D30" s="3" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="E30" s="3" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="F30" s="3" t="s">
         <v>10</v>
@@ -3194,7 +3200,7 @@
         <v>92</v>
       </c>
       <c r="I30" s="3" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="J30" s="3" t="s">
         <v>30</v>
@@ -3208,16 +3214,16 @@
         <v>93</v>
       </c>
       <c r="B31" s="3" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="C31" s="3" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="D31" s="3" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="E31" s="3" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="F31" s="3" t="s">
         <v>10</v>
@@ -3243,16 +3249,16 @@
         <v>96</v>
       </c>
       <c r="B32" s="3" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="C32" s="3" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="D32" s="3" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="E32" s="3" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="F32" s="3" t="s">
         <v>10</v>
@@ -3261,7 +3267,7 @@
         <v>97</v>
       </c>
       <c r="H32" s="9" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="I32" s="10" t="s">
         <v>89</v>
@@ -3278,16 +3284,16 @@
         <v>98</v>
       </c>
       <c r="B33" s="3" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="C33" s="3" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="D33" s="3" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="E33" s="3" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="F33" s="3" t="s">
         <v>10</v>
@@ -3296,7 +3302,7 @@
         <v>99</v>
       </c>
       <c r="H33" s="9" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="I33" s="10" t="s">
         <v>89</v>
@@ -3313,16 +3319,16 @@
         <v>100</v>
       </c>
       <c r="B34" s="3" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="C34" s="3" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="D34" s="3" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="E34" s="3" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="F34" s="3" t="s">
         <v>10</v>
@@ -3331,7 +3337,7 @@
         <v>101</v>
       </c>
       <c r="H34" s="9" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="I34" s="10" t="s">
         <v>89</v>
@@ -3348,16 +3354,16 @@
         <v>102</v>
       </c>
       <c r="B35" s="3" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="C35" s="3" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="D35" s="3" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="E35" s="3" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
       <c r="F35" s="3" t="s">
         <v>10</v>
@@ -3369,7 +3375,7 @@
         <v>104</v>
       </c>
       <c r="I35" s="8" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="J35" s="3" t="s">
         <v>30</v>
@@ -3380,19 +3386,19 @@
     </row>
     <row r="36" spans="1:11" ht="14.25" x14ac:dyDescent="0.25">
       <c r="A36" s="16" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="B36" s="3" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="C36" s="3" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="D36" s="3" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="E36" s="3" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
       <c r="F36" s="3" t="s">
         <v>10</v>
@@ -3415,28 +3421,28 @@
     </row>
     <row r="37" spans="1:11" ht="14.25" x14ac:dyDescent="0.25">
       <c r="A37" s="16" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="B37" s="3" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="C37" s="3" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="D37" s="3" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="E37" s="3" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
       <c r="F37" s="3" t="s">
         <v>10</v>
       </c>
       <c r="G37" s="8" t="s">
+        <v>280</v>
+      </c>
+      <c r="H37" s="9" t="s">
         <v>281</v>
-      </c>
-      <c r="H37" s="9" t="s">
-        <v>282</v>
       </c>
       <c r="I37" s="10" t="s">
         <v>107</v>
@@ -3450,31 +3456,31 @@
     </row>
     <row r="38" spans="1:11" ht="14.25" x14ac:dyDescent="0.25">
       <c r="A38" s="16" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="B38" s="3" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="C38" s="3" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="D38" s="3" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="E38" s="3" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
       <c r="F38" s="3" t="s">
         <v>10</v>
       </c>
       <c r="G38" s="8" t="s">
+        <v>282</v>
+      </c>
+      <c r="H38" s="9" t="s">
         <v>283</v>
       </c>
-      <c r="H38" s="9" t="s">
-        <v>284</v>
-      </c>
       <c r="I38" s="10" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="J38" s="3" t="s">
         <v>30</v>
@@ -3488,22 +3494,22 @@
         <v>108</v>
       </c>
       <c r="B39" s="3" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="C39" s="3" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="D39" s="3" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="E39" s="3" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
       <c r="F39" s="3" t="s">
         <v>10</v>
       </c>
       <c r="G39" s="8" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="H39" s="9" t="s">
         <v>109</v>
@@ -3520,31 +3526,31 @@
     </row>
     <row r="40" spans="1:11" ht="15" x14ac:dyDescent="0.25">
       <c r="A40" s="16" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="B40" s="3" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="C40" s="3" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="D40" s="3" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="E40" s="3" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
       <c r="F40" s="3" t="s">
         <v>10</v>
       </c>
       <c r="G40" s="8" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="H40" s="12" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="I40" s="8" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="J40" s="3" t="s">
         <v>13</v>
@@ -3555,31 +3561,31 @@
     </row>
     <row r="41" spans="1:11" ht="15" x14ac:dyDescent="0.25">
       <c r="A41" s="16" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="B41" s="3" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="C41" s="3" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="D41" s="3" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="E41" s="3" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
       <c r="F41" s="3" t="s">
         <v>10</v>
       </c>
       <c r="G41" s="8" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="H41" s="12" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="I41" s="8" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="J41" s="3" t="s">
         <v>30</v>
@@ -3590,31 +3596,31 @@
     </row>
     <row r="42" spans="1:11" ht="15" x14ac:dyDescent="0.25">
       <c r="A42" s="16" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="B42" s="3" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="C42" s="3" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="D42" s="3" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="E42" s="3" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
       <c r="F42" s="3" t="s">
         <v>10</v>
       </c>
       <c r="G42" s="8" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="H42" s="12" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="I42" s="8" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="J42" s="3" t="s">
         <v>30</v>
@@ -3628,16 +3634,16 @@
         <v>110</v>
       </c>
       <c r="B43" s="3" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="C43" s="3" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="D43" s="3" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="E43" s="3" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
       <c r="F43" s="3" t="s">
         <v>10</v>
@@ -3663,16 +3669,16 @@
         <v>114</v>
       </c>
       <c r="B44" s="3" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="C44" s="3" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="D44" s="3" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="E44" s="3" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
       <c r="F44" s="3" t="s">
         <v>10</v>
@@ -3698,16 +3704,16 @@
         <v>117</v>
       </c>
       <c r="B45" s="3" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="C45" s="3" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="D45" s="3" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="E45" s="3" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
       <c r="F45" s="3" t="s">
         <v>10</v>
@@ -3733,25 +3739,25 @@
         <v>118</v>
       </c>
       <c r="B46" s="3" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="C46" s="3" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="D46" s="3" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="E46" s="3" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
       <c r="F46" s="3" t="s">
         <v>10</v>
       </c>
       <c r="G46" s="8" t="s">
+        <v>240</v>
+      </c>
+      <c r="H46" s="12" t="s">
         <v>241</v>
-      </c>
-      <c r="H46" s="12" t="s">
-        <v>242</v>
       </c>
       <c r="I46" s="8" t="s">
         <v>123</v>
@@ -3768,16 +3774,16 @@
         <v>122</v>
       </c>
       <c r="B47" s="3" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="C47" s="3" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="D47" s="3" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="E47" s="3" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
       <c r="F47" s="3" t="s">
         <v>10</v>
@@ -3789,7 +3795,7 @@
         <v>126</v>
       </c>
       <c r="I47" s="3" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="J47" s="3" t="s">
         <v>13</v>
@@ -3803,16 +3809,16 @@
         <v>124</v>
       </c>
       <c r="B48" s="3" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="C48" s="3" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="D48" s="3" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="E48" s="3" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
       <c r="F48" s="3" t="s">
         <v>10</v>
@@ -3821,10 +3827,10 @@
         <v>128</v>
       </c>
       <c r="H48" s="12" t="s">
+        <v>243</v>
+      </c>
+      <c r="I48" s="3" t="s">
         <v>244</v>
-      </c>
-      <c r="I48" s="3" t="s">
-        <v>245</v>
       </c>
       <c r="J48" s="3" t="s">
         <v>13</v>
@@ -3838,16 +3844,16 @@
         <v>127</v>
       </c>
       <c r="B49" s="3" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="C49" s="3" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="D49" s="3" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="E49" s="3" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
       <c r="F49" s="3" t="s">
         <v>10</v>
@@ -3873,22 +3879,22 @@
         <v>129</v>
       </c>
       <c r="B50" s="3" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="C50" s="3" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="D50" s="3" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="E50" s="3" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
       <c r="F50" s="3" t="s">
         <v>10</v>
       </c>
       <c r="G50" s="8" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="H50" s="12" t="s">
         <v>134</v>
@@ -3908,16 +3914,16 @@
         <v>133</v>
       </c>
       <c r="B51" s="3" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="C51" s="3" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="D51" s="3" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="E51" s="3" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
       <c r="F51" s="3" t="s">
         <v>10</v>
@@ -3943,16 +3949,16 @@
         <v>135</v>
       </c>
       <c r="B52" s="3" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="C52" s="3" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="D52" s="3" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="E52" s="3" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
       <c r="F52" s="3" t="s">
         <v>10</v>
@@ -3961,10 +3967,10 @@
         <v>140</v>
       </c>
       <c r="H52" s="12" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="I52" s="3" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="J52" s="3" t="s">
         <v>13</v>
@@ -3978,16 +3984,16 @@
         <v>139</v>
       </c>
       <c r="B53" s="3" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="C53" s="3" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="D53" s="3" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="E53" s="3" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
       <c r="F53" s="3" t="s">
         <v>10</v>
@@ -3996,7 +4002,7 @@
         <v>142</v>
       </c>
       <c r="H53" s="12" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="I53" s="10" t="s">
         <v>143</v>
@@ -4013,25 +4019,25 @@
         <v>141</v>
       </c>
       <c r="B54" s="3" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="C54" s="3" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="D54" s="3" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="E54" s="3" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
       <c r="F54" s="3" t="s">
         <v>10</v>
       </c>
       <c r="G54" s="8" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="H54" s="12" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="I54" s="8" t="s">
         <v>123</v>
@@ -4048,16 +4054,16 @@
         <v>144</v>
       </c>
       <c r="B55" s="3" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="C55" s="3" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="D55" s="3" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="E55" s="3" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
       <c r="F55" s="3" t="s">
         <v>10</v>
@@ -4083,16 +4089,16 @@
         <v>145</v>
       </c>
       <c r="B56" s="3" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="C56" s="3" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="D56" s="3" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="E56" s="3" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
       <c r="F56" s="3" t="s">
         <v>10</v>
@@ -4101,10 +4107,10 @@
         <v>150</v>
       </c>
       <c r="H56" s="12" t="s">
+        <v>252</v>
+      </c>
+      <c r="I56" s="3" t="s">
         <v>253</v>
-      </c>
-      <c r="I56" s="3" t="s">
-        <v>254</v>
       </c>
       <c r="J56" s="3" t="s">
         <v>13</v>
@@ -4118,16 +4124,16 @@
         <v>149</v>
       </c>
       <c r="B57" s="3" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="C57" s="3" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="D57" s="3" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="E57" s="3" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
       <c r="F57" s="3" t="s">
         <v>10</v>
@@ -4153,16 +4159,16 @@
         <v>151</v>
       </c>
       <c r="B58" s="3" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="C58" s="3" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="D58" s="3" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="E58" s="3" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
       <c r="F58" s="3" t="s">
         <v>10</v>
@@ -4171,7 +4177,7 @@
         <v>156</v>
       </c>
       <c r="H58" s="12" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="I58" s="8" t="s">
         <v>123</v>
@@ -4188,16 +4194,16 @@
         <v>155</v>
       </c>
       <c r="B59" s="3" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="C59" s="3" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="D59" s="3" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="E59" s="3" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
       <c r="F59" s="3" t="s">
         <v>10</v>
@@ -4209,7 +4215,7 @@
         <v>159</v>
       </c>
       <c r="I59" s="3" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="J59" s="3" t="s">
         <v>13</v>
@@ -4223,16 +4229,16 @@
         <v>157</v>
       </c>
       <c r="B60" s="3" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="C60" s="3" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="D60" s="3" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="E60" s="3" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
       <c r="F60" s="3" t="s">
         <v>10</v>
@@ -4244,7 +4250,7 @@
         <v>162</v>
       </c>
       <c r="I60" s="3" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="J60" s="3" t="s">
         <v>13</v>
@@ -4258,16 +4264,16 @@
         <v>160</v>
       </c>
       <c r="B61" s="3" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="C61" s="3" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="D61" s="3" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="E61" s="3" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
       <c r="F61" s="3" t="s">
         <v>10</v>
@@ -4290,34 +4296,34 @@
     </row>
     <row r="62" spans="1:21" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A62" s="16" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="B62" s="3" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="C62" s="3" t="s">
+        <v>222</v>
+      </c>
+      <c r="D62" s="3" t="s">
         <v>223</v>
       </c>
-      <c r="D62" s="3" t="s">
-        <v>224</v>
-      </c>
       <c r="E62" s="3" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="F62" s="3" t="s">
         <v>10</v>
       </c>
       <c r="G62" s="3" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="H62" s="3" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
       <c r="I62" s="3" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="J62" s="3" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="K62" s="5" t="s">
         <v>26</v>
@@ -4325,34 +4331,34 @@
     </row>
     <row r="63" spans="1:21" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A63" s="16" t="s">
+        <v>266</v>
+      </c>
+      <c r="B63" s="3" t="s">
+        <v>217</v>
+      </c>
+      <c r="C63" s="3" t="s">
+        <v>222</v>
+      </c>
+      <c r="D63" s="3" t="s">
+        <v>223</v>
+      </c>
+      <c r="E63" s="3" t="s">
+        <v>398</v>
+      </c>
+      <c r="F63" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="G63" s="3" t="s">
         <v>267</v>
       </c>
-      <c r="B63" s="3" t="s">
-        <v>218</v>
-      </c>
-      <c r="C63" s="3" t="s">
-        <v>223</v>
-      </c>
-      <c r="D63" s="3" t="s">
-        <v>224</v>
-      </c>
-      <c r="E63" s="3" t="s">
-        <v>399</v>
-      </c>
-      <c r="F63" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="G63" s="3" t="s">
-        <v>268</v>
-      </c>
       <c r="H63" s="3" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="I63" s="3" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="J63" s="3" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="K63" s="4" t="s">
         <v>14</v>
@@ -4363,16 +4369,16 @@
         <v>163</v>
       </c>
       <c r="B64" s="3" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="C64" s="3" t="s">
+        <v>222</v>
+      </c>
+      <c r="D64" s="3" t="s">
         <v>223</v>
       </c>
-      <c r="D64" s="3" t="s">
-        <v>224</v>
-      </c>
       <c r="E64" s="3" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
       <c r="F64" s="3" t="s">
         <v>168</v>
@@ -4408,16 +4414,16 @@
         <v>167</v>
       </c>
       <c r="B65" s="3" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="C65" s="3" t="s">
+        <v>222</v>
+      </c>
+      <c r="D65" s="3" t="s">
         <v>223</v>
       </c>
-      <c r="D65" s="3" t="s">
-        <v>224</v>
-      </c>
       <c r="E65" s="3" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
       <c r="F65" s="3" t="s">
         <v>168</v>
@@ -4432,7 +4438,7 @@
         <v>42</v>
       </c>
       <c r="J65" s="3" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="K65" s="5" t="s">
         <v>26</v>
@@ -4453,16 +4459,16 @@
         <v>169</v>
       </c>
       <c r="B66" s="3" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="C66" s="3" t="s">
+        <v>222</v>
+      </c>
+      <c r="D66" s="3" t="s">
         <v>223</v>
       </c>
-      <c r="D66" s="3" t="s">
-        <v>224</v>
-      </c>
       <c r="E66" s="3" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
       <c r="F66" s="3" t="s">
         <v>168</v>
@@ -4474,7 +4480,7 @@
         <v>185</v>
       </c>
       <c r="I66" s="3" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="J66" s="3" t="s">
         <v>174</v>
@@ -4488,16 +4494,16 @@
         <v>170</v>
       </c>
       <c r="B67" s="3" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="C67" s="3" t="s">
+        <v>222</v>
+      </c>
+      <c r="D67" s="3" t="s">
         <v>223</v>
       </c>
-      <c r="D67" s="3" t="s">
-        <v>224</v>
-      </c>
       <c r="E67" s="3" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="F67" s="3" t="s">
         <v>168</v>
@@ -4512,7 +4518,7 @@
         <v>189</v>
       </c>
       <c r="J67" s="3" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="K67" s="5" t="s">
         <v>26</v>
@@ -4523,28 +4529,28 @@
         <v>175</v>
       </c>
       <c r="B68" s="3" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="C68" s="3" t="s">
+        <v>225</v>
+      </c>
+      <c r="D68" s="3" t="s">
         <v>226</v>
       </c>
-      <c r="D68" s="3" t="s">
-        <v>227</v>
-      </c>
       <c r="E68" s="3" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="F68" s="3" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
       <c r="G68" s="3" t="s">
+        <v>295</v>
+      </c>
+      <c r="H68" s="3" t="s">
         <v>296</v>
       </c>
-      <c r="H68" s="3" t="s">
+      <c r="I68" s="3" t="s">
         <v>297</v>
-      </c>
-      <c r="I68" s="3" t="s">
-        <v>298</v>
       </c>
       <c r="J68" s="3" t="s">
         <v>174</v>
@@ -4558,28 +4564,28 @@
         <v>177</v>
       </c>
       <c r="B69" s="3" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="C69" s="3" t="s">
+        <v>225</v>
+      </c>
+      <c r="D69" s="3" t="s">
         <v>226</v>
       </c>
-      <c r="D69" s="3" t="s">
-        <v>227</v>
-      </c>
       <c r="E69" s="3" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="F69" s="3" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
       <c r="G69" s="3" t="s">
+        <v>298</v>
+      </c>
+      <c r="H69" s="3" t="s">
         <v>299</v>
       </c>
-      <c r="H69" s="3" t="s">
+      <c r="I69" s="3" t="s">
         <v>300</v>
-      </c>
-      <c r="I69" s="3" t="s">
-        <v>301</v>
       </c>
       <c r="J69" s="3" t="s">
         <v>174</v>
@@ -4593,28 +4599,28 @@
         <v>178</v>
       </c>
       <c r="B70" s="3" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="C70" s="3" t="s">
+        <v>225</v>
+      </c>
+      <c r="D70" s="3" t="s">
         <v>226</v>
       </c>
-      <c r="D70" s="3" t="s">
-        <v>227</v>
-      </c>
       <c r="E70" s="3" t="s">
+        <v>410</v>
+      </c>
+      <c r="F70" s="3" t="s">
         <v>411</v>
       </c>
-      <c r="F70" s="3" t="s">
-        <v>412</v>
-      </c>
       <c r="G70" s="3" t="s">
+        <v>301</v>
+      </c>
+      <c r="H70" s="3" t="s">
         <v>302</v>
       </c>
-      <c r="H70" s="3" t="s">
+      <c r="I70" s="3" t="s">
         <v>303</v>
-      </c>
-      <c r="I70" s="3" t="s">
-        <v>304</v>
       </c>
       <c r="J70" s="3" t="s">
         <v>174</v>
@@ -4628,28 +4634,28 @@
         <v>179</v>
       </c>
       <c r="B71" s="3" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="C71" s="3" t="s">
+        <v>222</v>
+      </c>
+      <c r="D71" s="3" t="s">
         <v>223</v>
       </c>
-      <c r="D71" s="3" t="s">
-        <v>224</v>
-      </c>
       <c r="E71" s="3" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
       <c r="F71" s="3" t="s">
         <v>168</v>
       </c>
       <c r="G71" s="3" t="s">
+        <v>304</v>
+      </c>
+      <c r="H71" s="3" t="s">
         <v>305</v>
       </c>
-      <c r="H71" s="3" t="s">
+      <c r="I71" s="3" t="s">
         <v>306</v>
-      </c>
-      <c r="I71" s="3" t="s">
-        <v>307</v>
       </c>
       <c r="J71" s="3" t="s">
         <v>174</v>
@@ -4663,28 +4669,28 @@
         <v>180</v>
       </c>
       <c r="B72" s="3" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="C72" s="3" t="s">
+        <v>225</v>
+      </c>
+      <c r="D72" s="3" t="s">
         <v>226</v>
       </c>
-      <c r="D72" s="3" t="s">
-        <v>227</v>
-      </c>
       <c r="E72" s="3" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="F72" s="3" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
       <c r="G72" s="3" t="s">
+        <v>307</v>
+      </c>
+      <c r="H72" s="3" t="s">
         <v>308</v>
       </c>
-      <c r="H72" s="3" t="s">
+      <c r="I72" s="3" t="s">
         <v>309</v>
-      </c>
-      <c r="I72" s="3" t="s">
-        <v>310</v>
       </c>
       <c r="J72" s="3" t="s">
         <v>30</v>
@@ -4698,28 +4704,28 @@
         <v>181</v>
       </c>
       <c r="B73" s="3" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="C73" s="3" t="s">
+        <v>225</v>
+      </c>
+      <c r="D73" s="3" t="s">
         <v>226</v>
       </c>
-      <c r="D73" s="3" t="s">
-        <v>227</v>
-      </c>
       <c r="E73" s="3" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="F73" s="3" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
       <c r="G73" s="3" t="s">
+        <v>310</v>
+      </c>
+      <c r="H73" s="3" t="s">
         <v>311</v>
       </c>
-      <c r="H73" s="3" t="s">
+      <c r="I73" s="3" t="s">
         <v>312</v>
-      </c>
-      <c r="I73" s="3" t="s">
-        <v>313</v>
       </c>
       <c r="J73" s="3" t="s">
         <v>30</v>
@@ -4733,28 +4739,28 @@
         <v>182</v>
       </c>
       <c r="B74" s="3" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="C74" s="3" t="s">
+        <v>225</v>
+      </c>
+      <c r="D74" s="3" t="s">
         <v>226</v>
       </c>
-      <c r="D74" s="3" t="s">
-        <v>227</v>
-      </c>
       <c r="E74" s="3" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="F74" s="3" t="s">
         <v>168</v>
       </c>
       <c r="G74" s="3" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="H74" s="3" t="s">
+        <v>313</v>
+      </c>
+      <c r="I74" s="3" t="s">
         <v>314</v>
-      </c>
-      <c r="I74" s="3" t="s">
-        <v>315</v>
       </c>
       <c r="J74" s="3" t="s">
         <v>30</v>
@@ -4768,28 +4774,28 @@
         <v>183</v>
       </c>
       <c r="B75" s="3" t="s">
+        <v>333</v>
+      </c>
+      <c r="C75" s="3" t="s">
         <v>334</v>
       </c>
-      <c r="C75" s="3" t="s">
-        <v>335</v>
-      </c>
       <c r="D75" s="3" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="E75" s="3" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="F75" s="3" t="s">
         <v>10</v>
       </c>
       <c r="G75" s="3" t="s">
+        <v>315</v>
+      </c>
+      <c r="H75" s="3" t="s">
         <v>316</v>
       </c>
-      <c r="H75" s="3" t="s">
+      <c r="I75" s="3" t="s">
         <v>317</v>
-      </c>
-      <c r="I75" s="3" t="s">
-        <v>318</v>
       </c>
       <c r="J75" s="3" t="s">
         <v>174</v>
@@ -4803,28 +4809,28 @@
         <v>186</v>
       </c>
       <c r="B76" s="3" t="s">
+        <v>333</v>
+      </c>
+      <c r="C76" s="3" t="s">
         <v>334</v>
       </c>
-      <c r="C76" s="3" t="s">
-        <v>335</v>
-      </c>
       <c r="D76" s="3" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="E76" s="3" t="s">
+        <v>419</v>
+      </c>
+      <c r="F76" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="G76" s="3" t="s">
         <v>420</v>
       </c>
-      <c r="F76" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="G76" s="3" t="s">
-        <v>421</v>
-      </c>
       <c r="H76" s="3" t="s">
+        <v>328</v>
+      </c>
+      <c r="I76" s="3" t="s">
         <v>329</v>
-      </c>
-      <c r="I76" s="3" t="s">
-        <v>330</v>
       </c>
       <c r="J76" s="3" t="s">
         <v>30</v>
@@ -4835,31 +4841,31 @@
     </row>
     <row r="77" spans="1:21" ht="14.25" x14ac:dyDescent="0.25">
       <c r="A77" s="16" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="B77" s="3" t="s">
+        <v>333</v>
+      </c>
+      <c r="C77" s="3" t="s">
         <v>334</v>
       </c>
-      <c r="C77" s="3" t="s">
-        <v>335</v>
-      </c>
       <c r="D77" s="3" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="E77" s="3" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="F77" s="3" t="s">
         <v>10</v>
       </c>
       <c r="G77" s="3" t="s">
+        <v>336</v>
+      </c>
+      <c r="H77" s="3" t="s">
         <v>337</v>
       </c>
-      <c r="H77" s="3" t="s">
+      <c r="I77" s="3" t="s">
         <v>338</v>
-      </c>
-      <c r="I77" s="3" t="s">
-        <v>339</v>
       </c>
       <c r="J77" s="3" t="s">
         <v>30</v>
@@ -4870,31 +4876,31 @@
     </row>
     <row r="78" spans="1:21" ht="14.25" x14ac:dyDescent="0.25">
       <c r="A78" s="16" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="B78" s="3" t="s">
+        <v>333</v>
+      </c>
+      <c r="C78" s="3" t="s">
         <v>334</v>
       </c>
-      <c r="C78" s="3" t="s">
-        <v>335</v>
-      </c>
       <c r="D78" s="3" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="E78" s="3" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="F78" s="3" t="s">
         <v>10</v>
       </c>
       <c r="G78" s="3" t="s">
+        <v>340</v>
+      </c>
+      <c r="H78" s="3" t="s">
         <v>341</v>
       </c>
-      <c r="H78" s="3" t="s">
-        <v>342</v>
-      </c>
       <c r="I78" s="3" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
       <c r="J78" s="3" t="s">
         <v>30</v>
@@ -4905,31 +4911,31 @@
     </row>
     <row r="79" spans="1:21" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A79" s="16" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="B79" s="3" t="s">
+        <v>333</v>
+      </c>
+      <c r="C79" s="3" t="s">
         <v>334</v>
       </c>
-      <c r="C79" s="3" t="s">
-        <v>335</v>
-      </c>
       <c r="D79" s="3" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="E79" s="3" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="F79" s="3" t="s">
         <v>10</v>
       </c>
       <c r="G79" s="3" t="s">
+        <v>343</v>
+      </c>
+      <c r="H79" s="3" t="s">
+        <v>291</v>
+      </c>
+      <c r="I79" s="3" t="s">
         <v>344</v>
-      </c>
-      <c r="H79" s="3" t="s">
-        <v>292</v>
-      </c>
-      <c r="I79" s="3" t="s">
-        <v>345</v>
       </c>
       <c r="J79" s="3" t="s">
         <v>30</v>
@@ -4940,29 +4946,29 @@
     </row>
     <row r="80" spans="1:21" ht="14.25" x14ac:dyDescent="0.25">
       <c r="A80" s="3" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="B80" s="3" t="s">
+        <v>318</v>
+      </c>
+      <c r="C80" s="3" t="s">
         <v>319</v>
       </c>
-      <c r="C80" s="3" t="s">
-        <v>320</v>
-      </c>
       <c r="D80" s="3" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="E80" s="3"/>
       <c r="F80" s="3" t="s">
         <v>10</v>
       </c>
       <c r="G80" s="3" t="s">
+        <v>320</v>
+      </c>
+      <c r="H80" s="3" t="s">
         <v>321</v>
       </c>
-      <c r="H80" s="3" t="s">
+      <c r="I80" s="3" t="s">
         <v>322</v>
-      </c>
-      <c r="I80" s="3" t="s">
-        <v>323</v>
       </c>
       <c r="J80" s="3" t="s">
         <v>30</v>
@@ -4973,29 +4979,29 @@
     </row>
     <row r="81" spans="1:11" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A81" s="3" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="B81" s="3" t="s">
+        <v>318</v>
+      </c>
+      <c r="C81" s="3" t="s">
         <v>319</v>
       </c>
-      <c r="C81" s="3" t="s">
-        <v>320</v>
-      </c>
       <c r="D81" s="3" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="E81" s="3"/>
       <c r="F81" s="3" t="s">
         <v>168</v>
       </c>
       <c r="G81" s="3" t="s">
+        <v>324</v>
+      </c>
+      <c r="H81" s="3" t="s">
         <v>325</v>
       </c>
-      <c r="H81" s="3" t="s">
+      <c r="I81" s="3" t="s">
         <v>326</v>
-      </c>
-      <c r="I81" s="3" t="s">
-        <v>327</v>
       </c>
       <c r="J81" s="3" t="s">
         <v>30</v>
@@ -5006,29 +5012,29 @@
     </row>
     <row r="82" spans="1:11" ht="14.25" x14ac:dyDescent="0.25">
       <c r="A82" s="3" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="B82" s="3" t="s">
+        <v>318</v>
+      </c>
+      <c r="C82" s="3" t="s">
         <v>319</v>
       </c>
-      <c r="C82" s="3" t="s">
-        <v>320</v>
-      </c>
       <c r="D82" s="3" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="E82" s="3"/>
       <c r="F82" s="3" t="s">
         <v>10</v>
       </c>
       <c r="G82" s="3" t="s">
+        <v>346</v>
+      </c>
+      <c r="H82" s="3" t="s">
         <v>347</v>
       </c>
-      <c r="H82" s="3" t="s">
+      <c r="I82" s="3" t="s">
         <v>348</v>
-      </c>
-      <c r="I82" s="3" t="s">
-        <v>349</v>
       </c>
       <c r="J82" s="3" t="s">
         <v>30</v>
@@ -5039,31 +5045,31 @@
     </row>
     <row r="83" spans="1:11" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A83" s="16" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="B83" s="3" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="C83" s="3" t="s">
+        <v>225</v>
+      </c>
+      <c r="D83" s="3" t="s">
         <v>226</v>
       </c>
-      <c r="D83" s="3" t="s">
-        <v>227</v>
-      </c>
       <c r="E83" s="3" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="F83" s="3" t="s">
         <v>10</v>
       </c>
       <c r="G83" s="3" t="s">
+        <v>358</v>
+      </c>
+      <c r="H83" s="3" t="s">
         <v>359</v>
       </c>
-      <c r="H83" s="3" t="s">
-        <v>360</v>
-      </c>
       <c r="I83" s="3" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="J83" s="3" t="s">
         <v>30</v>
@@ -5074,31 +5080,31 @@
     </row>
     <row r="84" spans="1:11" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A84" s="16" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="B84" s="3" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="C84" s="3" t="s">
+        <v>225</v>
+      </c>
+      <c r="D84" s="3" t="s">
         <v>226</v>
       </c>
-      <c r="D84" s="3" t="s">
-        <v>227</v>
-      </c>
       <c r="E84" s="3" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="F84" s="3" t="s">
         <v>10</v>
       </c>
       <c r="G84" s="3" t="s">
+        <v>360</v>
+      </c>
+      <c r="H84" s="3" t="s">
         <v>361</v>
       </c>
-      <c r="H84" s="3" t="s">
-        <v>362</v>
-      </c>
       <c r="I84" s="3" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="J84" s="3" t="s">
         <v>30</v>
@@ -5109,31 +5115,31 @@
     </row>
     <row r="85" spans="1:11" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A85" s="16" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="B85" s="3" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="C85" s="3" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="D85" s="3" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="E85" s="3" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="F85" s="3" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="G85" s="3" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="H85" s="3" t="s">
+        <v>403</v>
+      </c>
+      <c r="I85" s="3" t="s">
         <v>404</v>
-      </c>
-      <c r="I85" s="3" t="s">
-        <v>405</v>
       </c>
       <c r="J85" s="3" t="s">
         <v>30</v>
@@ -5144,31 +5150,31 @@
     </row>
     <row r="86" spans="1:11" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A86" s="16" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="B86" s="3" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="C86" s="3" t="s">
+        <v>225</v>
+      </c>
+      <c r="D86" s="3" t="s">
         <v>226</v>
       </c>
-      <c r="D86" s="3" t="s">
-        <v>227</v>
-      </c>
       <c r="E86" s="3" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="F86" s="3" t="s">
         <v>168</v>
       </c>
       <c r="G86" s="3" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="H86" s="3" t="s">
+        <v>362</v>
+      </c>
+      <c r="I86" s="3" t="s">
         <v>363</v>
-      </c>
-      <c r="I86" s="3" t="s">
-        <v>364</v>
       </c>
       <c r="J86" s="3" t="s">
         <v>30</v>
@@ -5179,31 +5185,31 @@
     </row>
     <row r="87" spans="1:11" ht="14.25" x14ac:dyDescent="0.25">
       <c r="A87" s="16" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="B87" s="3" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="C87" s="3" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="D87" s="3" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="E87" s="3" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="F87" s="3" t="s">
         <v>10</v>
       </c>
       <c r="G87" s="3" t="s">
+        <v>364</v>
+      </c>
+      <c r="H87" s="3" t="s">
         <v>365</v>
       </c>
-      <c r="H87" s="3" t="s">
+      <c r="I87" s="3" t="s">
         <v>366</v>
-      </c>
-      <c r="I87" s="3" t="s">
-        <v>367</v>
       </c>
       <c r="J87" s="3" t="s">
         <v>30</v>
@@ -5214,31 +5220,31 @@
     </row>
     <row r="88" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A88" s="16" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="B88" s="3" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="C88" s="3" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="D88" s="3" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="E88" s="3" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="F88" s="3" t="s">
         <v>168</v>
       </c>
       <c r="G88" s="3" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="H88" s="3" t="s">
+        <v>365</v>
+      </c>
+      <c r="I88" s="3" t="s">
         <v>366</v>
-      </c>
-      <c r="I88" s="3" t="s">
-        <v>367</v>
       </c>
       <c r="J88" s="3" t="s">
         <v>30</v>
@@ -5249,66 +5255,66 @@
     </row>
     <row r="89" spans="1:11" ht="114.75" x14ac:dyDescent="0.25">
       <c r="A89" s="3" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="B89" s="3" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="C89" s="3" t="s">
+        <v>225</v>
+      </c>
+      <c r="D89" s="3" t="s">
         <v>226</v>
       </c>
-      <c r="D89" s="3" t="s">
-        <v>227</v>
-      </c>
       <c r="E89" s="3" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
       <c r="F89" s="3" t="s">
         <v>168</v>
       </c>
       <c r="G89" s="3" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="H89" s="3" t="s">
+        <v>368</v>
+      </c>
+      <c r="I89" s="3" t="s">
         <v>369</v>
-      </c>
-      <c r="I89" s="3" t="s">
-        <v>370</v>
       </c>
       <c r="J89" s="3" t="s">
         <v>30</v>
       </c>
       <c r="K89" s="15" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
     </row>
     <row r="90" spans="1:11" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A90" s="16" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="B90" s="3" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="C90" s="3" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="D90" s="3" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="E90" s="3" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="F90" s="3" t="s">
         <v>168</v>
       </c>
       <c r="G90" s="3" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="H90" s="3" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="I90" s="3" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="J90" s="3" t="s">
         <v>30</v>
@@ -5319,31 +5325,31 @@
     </row>
     <row r="91" spans="1:11" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A91" s="16" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
       <c r="B91" s="3" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="C91" s="3" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="D91" s="3" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="E91" s="3" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="F91" s="3" t="s">
         <v>168</v>
       </c>
       <c r="G91" s="3" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="H91" s="3" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="I91" s="3" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="J91" s="3" t="s">
         <v>30</v>
@@ -5354,29 +5360,29 @@
     </row>
     <row r="92" spans="1:11" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A92" s="3" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="B92" s="3" t="s">
+        <v>318</v>
+      </c>
+      <c r="C92" s="3" t="s">
         <v>319</v>
       </c>
-      <c r="C92" s="3" t="s">
-        <v>320</v>
-      </c>
       <c r="D92" s="3" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="E92" s="3"/>
       <c r="F92" s="3" t="s">
         <v>168</v>
       </c>
       <c r="G92" s="8" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="H92" s="9" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="I92" s="3" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="J92" s="3" t="s">
         <v>30</v>
@@ -5590,16 +5596,16 @@
         <v>2</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="C3" s="1" t="s">
+        <v>218</v>
+      </c>
+      <c r="D3" s="1" t="s">
         <v>219</v>
       </c>
-      <c r="D3" s="1" t="s">
-        <v>220</v>
-      </c>
       <c r="E3" s="1" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="F3" s="1" t="s">
         <v>3</v>
@@ -5645,7 +5651,8 @@
   <dimension ref="A1:K12"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.5703125" defaultRowHeight="53.25" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="5" width="11.5703125" style="6"/>
+    <col min="1" max="4" width="11.5703125" style="6"/>
+    <col min="5" max="5" width="25" style="6" customWidth="1"/>
     <col min="6" max="6" width="21.7109375" style="6" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="44" style="6" customWidth="1"/>
     <col min="8" max="8" width="48.28515625" style="6" bestFit="1" customWidth="1"/>
@@ -5689,16 +5696,16 @@
         <v>2</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="C3" s="1" t="s">
+        <v>218</v>
+      </c>
+      <c r="D3" s="1" t="s">
         <v>219</v>
       </c>
-      <c r="D3" s="1" t="s">
-        <v>220</v>
-      </c>
       <c r="E3" s="1" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="F3" s="1" t="s">
         <v>3</v>
@@ -5721,31 +5728,31 @@
     </row>
     <row r="4" spans="1:11" ht="53.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="16" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="F4" s="3" t="s">
         <v>198</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="I4" s="3" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="J4" s="3" t="s">
         <v>13</v>
@@ -5756,31 +5763,31 @@
     </row>
     <row r="5" spans="1:11" ht="53.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="16" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="F5" s="3" t="s">
         <v>198</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="H5" s="3" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="I5" s="3" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="J5" s="3" t="s">
         <v>13</v>
@@ -5791,19 +5798,19 @@
     </row>
     <row r="6" spans="1:11" ht="53.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="16" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="F6" s="3" t="s">
         <v>198</v>
@@ -5812,10 +5819,10 @@
         <v>214</v>
       </c>
       <c r="H6" s="3" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="I6" s="3" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="J6" s="3" t="s">
         <v>212</v>
@@ -5825,30 +5832,32 @@
       </c>
     </row>
     <row r="7" spans="1:11" ht="51" x14ac:dyDescent="0.25">
-      <c r="A7" s="3" t="s">
-        <v>388</v>
+      <c r="A7" s="16" t="s">
+        <v>387</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="C7" s="3" t="s">
+        <v>222</v>
+      </c>
+      <c r="D7" s="3" t="s">
         <v>223</v>
       </c>
-      <c r="D7" s="3" t="s">
-        <v>224</v>
-      </c>
-      <c r="E7" s="3"/>
+      <c r="E7" s="3" t="s">
+        <v>423</v>
+      </c>
       <c r="F7" s="3" t="s">
         <v>198</v>
       </c>
       <c r="G7" s="3" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="H7" s="3" t="s">
         <v>202</v>
       </c>
       <c r="I7" s="3" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
       <c r="J7" s="3" t="s">
         <v>13</v>
@@ -5858,19 +5867,21 @@
       </c>
     </row>
     <row r="8" spans="1:11" ht="165.75" x14ac:dyDescent="0.25">
-      <c r="A8" s="3" t="s">
-        <v>389</v>
+      <c r="A8" s="16" t="s">
+        <v>388</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="C8" s="3" t="s">
+        <v>222</v>
+      </c>
+      <c r="D8" s="3" t="s">
         <v>223</v>
       </c>
-      <c r="D8" s="3" t="s">
-        <v>224</v>
-      </c>
-      <c r="E8" s="3"/>
+      <c r="E8" s="3" t="s">
+        <v>423</v>
+      </c>
       <c r="F8" s="3" t="s">
         <v>198</v>
       </c>
@@ -5891,19 +5902,21 @@
       </c>
     </row>
     <row r="9" spans="1:11" ht="127.5" x14ac:dyDescent="0.25">
-      <c r="A9" s="3" t="s">
-        <v>390</v>
+      <c r="A9" s="16" t="s">
+        <v>389</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="C9" s="3" t="s">
+        <v>222</v>
+      </c>
+      <c r="D9" s="3" t="s">
         <v>223</v>
       </c>
-      <c r="D9" s="3" t="s">
-        <v>224</v>
-      </c>
-      <c r="E9" s="3"/>
+      <c r="E9" s="3" t="s">
+        <v>423</v>
+      </c>
       <c r="F9" s="3" t="s">
         <v>198</v>
       </c>
@@ -5924,19 +5937,21 @@
       </c>
     </row>
     <row r="10" spans="1:11" ht="76.5" x14ac:dyDescent="0.25">
-      <c r="A10" s="3" t="s">
-        <v>391</v>
+      <c r="A10" s="16" t="s">
+        <v>390</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="C10" s="3" t="s">
+        <v>222</v>
+      </c>
+      <c r="D10" s="3" t="s">
         <v>223</v>
       </c>
-      <c r="D10" s="3" t="s">
-        <v>224</v>
-      </c>
-      <c r="E10" s="3"/>
+      <c r="E10" s="3" t="s">
+        <v>423</v>
+      </c>
       <c r="F10" s="3" t="s">
         <v>198</v>
       </c>
@@ -5957,19 +5972,21 @@
       </c>
     </row>
     <row r="11" spans="1:11" ht="165.75" x14ac:dyDescent="0.25">
-      <c r="A11" s="3" t="s">
-        <v>392</v>
+      <c r="A11" s="16" t="s">
+        <v>391</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="C11" s="3" t="s">
+        <v>222</v>
+      </c>
+      <c r="D11" s="3" t="s">
         <v>223</v>
       </c>
-      <c r="D11" s="3" t="s">
-        <v>224</v>
-      </c>
-      <c r="E11" s="3"/>
+      <c r="E11" s="3" t="s">
+        <v>423</v>
+      </c>
       <c r="F11" s="3" t="s">
         <v>198</v>
       </c>
@@ -5990,19 +6007,21 @@
       </c>
     </row>
     <row r="12" spans="1:11" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="A12" s="3" t="s">
-        <v>393</v>
+      <c r="A12" s="16" t="s">
+        <v>392</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="C12" s="3" t="s">
+        <v>225</v>
+      </c>
+      <c r="D12" s="3" t="s">
         <v>226</v>
       </c>
-      <c r="D12" s="3" t="s">
-        <v>227</v>
-      </c>
-      <c r="E12" s="3"/>
+      <c r="E12" s="3" t="s">
+        <v>425</v>
+      </c>
       <c r="F12" s="3" t="s">
         <v>198</v>
       </c>
@@ -6013,7 +6032,7 @@
         <v>213</v>
       </c>
       <c r="I12" s="3" t="s">
-        <v>215</v>
+        <v>424</v>
       </c>
       <c r="J12" s="3" t="s">
         <v>212</v>
@@ -6086,16 +6105,16 @@
         <v>2</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="C3" s="1" t="s">
+        <v>218</v>
+      </c>
+      <c r="D3" s="1" t="s">
         <v>219</v>
       </c>
-      <c r="D3" s="1" t="s">
-        <v>220</v>
-      </c>
       <c r="E3" s="1" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="F3" s="1" t="s">
         <v>3</v>
@@ -6158,7 +6177,7 @@
     </row>
     <row r="2" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="19" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="B2" s="19"/>
       <c r="C2" s="19"/>
@@ -6172,16 +6191,16 @@
         <v>2</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="C3" s="1" t="s">
+        <v>218</v>
+      </c>
+      <c r="D3" s="1" t="s">
         <v>219</v>
       </c>
-      <c r="D3" s="1" t="s">
-        <v>220</v>
-      </c>
       <c r="E3" s="1" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="F3" s="1" t="s">
         <v>3</v>
@@ -6258,16 +6277,16 @@
         <v>2</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="C3" s="1" t="s">
+        <v>218</v>
+      </c>
+      <c r="D3" s="1" t="s">
         <v>219</v>
       </c>
-      <c r="D3" s="1" t="s">
-        <v>220</v>
-      </c>
       <c r="E3" s="1" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="F3" s="1" t="s">
         <v>3</v>
@@ -6344,16 +6363,16 @@
         <v>2</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="C3" s="1" t="s">
+        <v>218</v>
+      </c>
+      <c r="D3" s="1" t="s">
         <v>219</v>
       </c>
-      <c r="D3" s="1" t="s">
-        <v>220</v>
-      </c>
       <c r="E3" s="1" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="F3" s="1" t="s">
         <v>3</v>
@@ -6430,16 +6449,16 @@
         <v>2</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="C3" s="1" t="s">
+        <v>218</v>
+      </c>
+      <c r="D3" s="1" t="s">
         <v>219</v>
       </c>
-      <c r="D3" s="1" t="s">
-        <v>220</v>
-      </c>
       <c r="E3" s="1" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="F3" s="1" t="s">
         <v>3</v>
@@ -6516,16 +6535,16 @@
         <v>2</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="C3" s="1" t="s">
+        <v>218</v>
+      </c>
+      <c r="D3" s="1" t="s">
         <v>219</v>
       </c>
-      <c r="D3" s="1" t="s">
-        <v>220</v>
-      </c>
       <c r="E3" s="1" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="F3" s="1" t="s">
         <v>3</v>
@@ -6602,16 +6621,16 @@
         <v>2</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="C3" s="1" t="s">
+        <v>218</v>
+      </c>
+      <c r="D3" s="1" t="s">
         <v>219</v>
       </c>
-      <c r="D3" s="1" t="s">
-        <v>220</v>
-      </c>
       <c r="E3" s="1" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="F3" s="1" t="s">
         <v>3</v>

</xml_diff>